<commit_message>
Built json->excel raw data processing pipeline and tested link filtering+extraction for 24
</commit_message>
<xml_diff>
--- a/research_data.xlsx
+++ b/research_data.xlsx
@@ -1,77 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amd9m\Downloads\HQSS 495\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A35A54-FC59-4672-BB47-546C32402430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" xr2:uid="{CC503BD6-7AF3-445D-A6BB-7C3FDB04D7CD}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
+    <sheet name="raw_data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>Sender</t>
-  </si>
-  <si>
-    <t>Subject</t>
-  </si>
-  <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Processed</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -90,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -424,31 +439,617 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AF4EFE1-3DFD-4C3A-A1C0-13D0CD8F4D2E}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="38.21875" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="61.88671875" customWidth="1"/>
+    <col width="13.77734375" customWidth="1" min="1" max="1"/>
+    <col width="38.21875" customWidth="1" min="2" max="2"/>
+    <col width="15.5546875" customWidth="1" min="3" max="3"/>
+    <col width="61.88671875" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Sender</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Links</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pillanatok alatt hullott darabokra az Orbán által felépített világ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>23 April 2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F23%2Forban-rendszere-vilag-felborult-szemelyi-diplomacia-elemzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260423";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Ftorok-gabor-ruff-balint-reakcio-ironia-propaganda-index%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fruff-balint-miniszter-lesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fszijjarto-peter-interju-telex%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fkozteve-helyreigazitas-tota-w-arpad-szado-mazo-szex%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fruff-balint-miniszterelnokseget-vezeto-miniszter-tisza-kormany-magyar-peter-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Forban-gaspar-magyar-honvedseg-tavozas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F22%2Fmagyar-drogbaro-mexiko-elfogas-fbi%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fmnb-jegybank-matolcsy-gyorgy-nyomozas-vagyonvesztes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fmagyar-peter-orban-viktor-videk-kovach-imre%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fmedian-valasztas-utani-kutatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fszabo-bence-nyomozas-ugyeszseg-hivatali-visszaeles-gundalf%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F22%2Fnagy-adam-valyi-istvan-rainer-micsinyei-nora-interju-orban-rendszer%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fmiklosi-zoltan-autokracia-orban-bukas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftudomany%2F2026%2F04%2F22%2Fzaptojasszag-adand-illegalis-hulladekkezeles%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F23%2Forban-rendszere-vilag-felborult-szemelyi-diplomacia-elemzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fmenczer-tamas-valasztas-megszolalt%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F22%2Fgaspar-evelin-kulugy-tavozas-szijjarto-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fgimnazium-igazgatok-magyar-peter-rubovszky-rita-talalkozo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F22%2Fkviz-magyar-hiressegek-mosoly%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F22%2Fpuzser-robert-wolf-kati-poszt-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F22%2Flilu-ruff-balint-kinevezes-tisza-kormany-miniszter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F22%2Fkapitany-istvan-szja-csokkentes%2F";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fszijjarto-peter-interju-telex%2F";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Ftorok-gabor-median-kutatas%2F";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Fparlament-felszolalok-orszaggyules-2022-2026%2F";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Fsimor-andras-mnb-erste-matolcsy-gyorgy%2F";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fgyor-per-levetkoztette-poloska%2F";"https://ad.admail.hu/tl.php?p=2lah/m1v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F23%2Fcsezy-politika-tisza-mezokovesd-fellepesek-csalad%2F"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>„Akik eddig a propaganda működtetését végezték, eltűnnek a háttérből” – mi vár a közmédiára, és mit várhatunk tőle?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>22 April 2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fkozmedia-propaganda-tisza-magyar%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260422";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fmatolcsy-adam-visszavagott-magyar-peternek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F21%2Farany-aranytartalek-devizatartalek-mnb%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Flegfobb-ugyeszseg-matolcsy-ugy-mnb%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fbbc-pendriveokkal-kerestek-meg-hivatalnokok-a-tiszat-hogy-megtarthassak-az-allasukat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fmagyar-legfobb-ugyeszseg-megkesett%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fzarug-peter-farkas-orban-viktor-fidesz-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F21%2Fdemeter-szilard-orban-viktor-valasztas-2026-mandiner%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fmnb-botrany-legfobb-ugyeszseg-alapitvany%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fsulyok-tamas-peticio-fidesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fpodcast-haromharmad-napirend-utan-52%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fparlament-alakulo-ules-idopont-mikor-lesz-magyar-peter-esku%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F21%2Fakkumulatortesztelo-budapest-erd-logisztikai-park-veszelyes-uzem%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fgyermekvedelmi-torveny-europai-unio-birosag-itelet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Femberoles-csaladon-beluli-eroszak%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F21%2Fpodcast-della-kokarda-valasztas-jelasity-radovan-erste%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F21%2Fbaratsag-koolajvezetek-ukrajna-energia-eu%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F21%2Fzelenszkij-ukrajna-megjavitotta-a-baratsag-vezeteket%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F22%2Fkozmedia-propaganda-tisza-magyar%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F21%2Ferzsebet100-ii-erzsebet-kiralyno-gyerekkora%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F21%2Frtl-hirado-eros-antonia-szello-istvan-gonczi-gabor-marsi-aniko%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Ftakacs-peter-egeszsegugyi-allamtitkar-anyazas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F21%2Ftiborcz-istvan-scheer-sandor-bn-referencia-zrt-ner%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F21%2Fanne-hathaway-az-ordog-pradat-visel-2-legszebb-sztar-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fgulyas-mandatum-fidesz-parlament%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9v/m1t/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F21%2Fbaratsag-koolajvezetes-ukran-tamadas-orosz-ukran-haboru%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>„Két jó vezetője volt Magyarországnak: Kádár János és Orbán Viktor” – választási sokkból éledő kelet-nógrádiakkal beszéltünk</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>21 April 2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fvalasztas-2026-nograd-riport-salgotarjan-matraverebely%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260421";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fruszin-szendi-romulusz-honvedelmi-miniszter-uzenet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fbaranyi-krisztina-bayer-construct-horvath-csaba%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fmagyar-peter-het-miniszter-frakcioules-sajtotajekoztato%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fmagyar-peter-gimnaziumok-oktatasi-miniszter-kivalasztasa%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fbicske-gyermekotthon-szabadlab-v-janos%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fkozep-europara-fokuszal-tisza-rmdsz-elemzok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F20%2Fkende-annak-szocalpszichologus-valasztas-2026-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2Ffoci%2F2026%2F04%2F20%2Fnb1-bajnoki-hajra-eto-ferencvaros-elemzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fminden-mozdithatot-ertekesitenek-es-elutalnak-meszaros-lorinc-kornyezetgazdalkodasi-cegebol%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Frogan-antal-parancs-miniszteriumok-fideszes-uzenetek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fkdnp-frakcio-bepanikoltak-orban-terv%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fmi-hazank-3-joszabaly-modositas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F20%2Ftimothy-garton-ash-interju-orban-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F20%2Fgeszti-peter-tisza-kormany-petofi-tv-olah-gergo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F21%2Fszolidaritasi-ado-fovaros-karacsony%2F";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F21%2Frtl-hirado-eros-antonia-szello-istvan-gonczi-gabor-marsi-aniko%2F";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F20%2Froman-miniszterelnok-psd-tamogatas-lemondas%2F";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F20%2Ffluor-rendszerbonto-nagykoncert%2F";"https://ad.admail.hu/tl.php?p=2l9c/m1s/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fsalgotarjtan-auto-lopasok%2F"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A Fidesz bukása előtt egy kiváltságos üzletbe szállt be Nagy Márton köre Tiborcz Istvánék mellé</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F20%2Fszeleromu-nagy-marton-magantokealap-tiborcz-orban%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260420";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Fszabo-tunde-ugyved-parlament-kiesett-fidesz-kepviselo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Fkocsis-mate-arulo-borbas-marcsi%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Fbalogh-levente-reakcio-kocsis-mate-orban-viktor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Flotto-fonyeremeny-szerencsejatek-zrt-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F19%2Flengyel-tamas-ledaralt-iratok-mti%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Feuropion-orban-kormany-kozjogi-meltosagok-lemondasa-magyar-peter-kozmedia-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Fjeszenszky-zsolt-india-orban-viktor-balvanyimadas-vereseg-lehetsges-ok-hajdu-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l92/m1q/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F19%2Fmajka-kocsis-mate-rakai-philip%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hatalmas vagyont halmoztak fel az Orbán-érában a Fidesz-közeli alapítványok: 617 milliárdnál állt meg a számlálónk</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>17 April 2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F17%2Ffidesz-alapitvany-vagyon-mcc-schmidt-maria-kesma%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260417";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Forban-viktor-interju-vereseg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fvalasztas-2026-ferencz-orsolya-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F17%2Fkutyapart-kampanytamogatas-visszafizetes-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fivanyi-gabor-interju-koztarsasagi-elnok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F17%2Fhann-endre-kozteve%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Flevelszavazatok-eredmeny-fidesz-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fszalai-vivien-tv2-tavozas-hirigazgato%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fszijjarto-peter-valasztas-2026-kulugyminiszter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Ffelcsut-valasztas-2026-orban-viktor-vereseg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F16%2Fnadasdy-adam-temetes-grecso-krisztian%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F16%2Fmajka-papai-joci-fidesz-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Frubovszky-rita-habony-arpad-tanacsado-ceg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F17%2Fsilhavy-mate-kuratoriumi-tag-lemondas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F17%2Fsulyok-tamas-bodo-bernadett-felmentes-pinter-sandor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fmagyar-peter-vedett-benzinar-mol%2F";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Forban-viktor-interju-vereseg%2F%23ha-kell-szertaros-lesz-orban-de-ha-ugy-dontenek-szivesen-ujra-a-palyara-vezeti-a-csapatot";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F16%2Fkarman-andras-arresstopok%2F";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fruszin-szendi-romulusz-iratmegsemmisites-honvedelmi-miniszterium%2F";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Flevelszavazatok-eredmeny-fidesz-tisza%2F";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fdj-seggszaggato-nagy-istvan-agrarminiszter%2F";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F17%2Fhann-endre-kozteve%2F";"https://ad.admail.hu/tl.php?p=2l7k/m1m/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F04%2F16%2Fmilak-kristof-aranyerem-uszo-ob-100-gyors%2F"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pócs János: A Fideszben nincs más, aki főnixmadárként a semmiből képes felemelkedni, csak Orbán Viktor</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>16 April 2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F16%2Fpocs-janos-interju-jaszbereny-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260416";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fmagyar-peter-miniszterelnok-tisza-kozmedia-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fmagyar-peter-miniszterelnok-tisza-kozmedia-interju%2F%23a-musorvezeto-elnezest-kert-az-interjut-hangnemeert%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fgyorfi-mihaly-ultimatum-szita-karoly-mjvsz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fkaracsony-gergely-bizonyos-szentkiralyi-alexandra-eva-maganszemely-feljelentett%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fgulyas-gergely-kampany-tevedtunk%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Forban-magyar-karmelita-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F15%2Fordog-nora-valasztas-utani-poszt-kajdi-csaba-torolt-komment%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fkozmedia-lazadas-korleves-koveteles-fuggetken-hirszolgaltatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F15%2Fpasztor-anna-toth-gabi-fidesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l70/m1k/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Fwaberer-mav-lazar-fidesz-befolyas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A Tisza a narancsvidékre is kiöntött – így vette be az országot Magyar Péter, körzetről körzetre</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F15%2Ftisza-egyeni-valasztokerulet-csataterkorzet-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260415";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fpinter-fekete-pufajkasok-kitiltas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260415";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Ftolgyessy-peter-orban-viktor-visszavonulas-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Forban-anita-iratmegsemmisites%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F14%2Fmeszaros-csoport-meszaros-lorinc-opus-global-valasztas2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Fvalasztas-2026-piliscsaba-jegyzo-buzizas-felmentes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F14%2Fgalvolgyi-janos-orban-viktor-uzenet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F14%2Feu-penz-europai-bizottsag-unios-forras-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Fdeak-daniel-bocsanatkeres-hann-endre%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Fkovacs-gergely-felszamolas-mkkp-tartozas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Ftovabb-erosodik-a-forint-2%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l6o/m1i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F14%2Firatmegsemmisito-belugyminiszterium-pinter-sandor-beszerzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hadházy Ákos: Azt gondolom, volt szerepem abban, hogy Magyar Péternek kinyílt a szeme</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>14 April 2026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F14%2Fhadhazy-akos-lekoszon-interju-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260414";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Forban-viktor-eletut-kepgaleria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fafrikai-ut-honvedseg-gepei-falcon%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fmagyar-peter-ket-ev-kepgaleria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F04%2F13%2Felon-musk-magyar-peter-alex-soros-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fvalasztas-masnap-hetfo-galeria-tisza-magyar-peter-budapest%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F13%2Ftoth-gabi-tisza-part-gyozelem-gratulacio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fmagyar-peter-nemzetkozi-sajtotajekoztato-elo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fvalasztas-2026-masnap-elo-hirfolyam%2F%23lazar-janos-megtorte-a-csendet%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Ftisza-ketharmad-magyar-peter-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l60/m1h/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fbuzi-magyar-peter-piliscsabai-jegyzo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1990 óta nem látott elitcsere, ledönthetetlennek hitt Fidesz-bástyák estek el</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>13 April 2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F13%2Fvalasztas-2026-eredmenyek-fidesz-rendszervaltas-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260413";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F04%2F11%2Fvalasztokeruleti-kisokos-indikator-korzetek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F04%2F11%2Fmagyar-peter-debrecen-szombat-beszed-kampanyzaro%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Fxiii-kerulet-baleset-versenyzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Fpodcast-torokules-orban-viktor-magyar-peter-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Frendszerbonto-nagykoncert-puzser-robert-saiid-dzsudlo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftudomany%2F2026%2F04%2F11%2Ftrianon-kisantant-fenyegetes-tortenelem%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Ffidesz-valasztasi-csalas-elelmiszercsomag%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Fnadudvar-tisza-auto-ruszin-szendi-romulusz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F04%2F11%2Fkapufa-peto-peter-valasztas-2026-barkoczi-balazs%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Fkampanyhajra-onmerenylet-hackertamadas-titkosszolgalat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Fmagyar-peter-kampanyzaro-debrecen-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F12%2Fvalasztas-2026-elo-hirfolyam%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F04%2F11%2Frobert-fico-orban-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F11%2Frendszerbonto-nagykoncert-hosok-tere-ember-mark%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F11%2Fhernadi-judit-hetven-szuletesnap-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F11%2Ftoth-gabi-rendszerbonto-nagykoncert-drogos-kutyak%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F11%2Fvarga-judit-valasztas-szavazas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F11%2Fontario-felgyujtott-raktar-fizetes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F04%2F11%2Fhann-endre-median-valasztas-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l5e/m1f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F11%2Fhajdu-peter-orban-viktor-interju-kikotes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>„Ha valaki meg akar élni, kénytelen másodállást vállalni” – interjú a rendőrszakszervezet vezetőivel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>09 April 2026</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F09%2Frendorseg-rendorszakszervezet-rendorhiany-krsz-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260409";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fnni-rendorseg-interju-politika-virag-norman-viktor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fcseuscsak-renata-birosag-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fmedian-tisza-ketharmad-mandatumbecsles%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F08%2Fpodcast-della-csaba-laszlo-utolso-tanacs-orban-viktornak%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F08%2Fdemjen-ferenc-mi-vagyunk-a-ner%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Forban-valasztas-2026-edeleny-kazincbarcika%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2Ffoci%2F2026%2F04%2F08%2Fbajnokok-ligaja-negyeddonto-psg-liverpool-barcelona-atletico-madrid%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2F21-kutatokozpont-kozvelemeny-kutatas-felmeres-progressziv-ado-tobbkulcsos-ado%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fnagy-david-interju-mkkp-listavezeto-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F08%2Firan-usa-izrael-tuzszunet-elemzes-sarkozy-miklos%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F08%2Fszatmari-peter-buntenyek-podcast-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F09%2Frendorseg-rendorszakszervezet-rendorhiany-krsz-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fracz-andras-orban-putyin-telefonbeszelgetes-leirat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fpecs-gyermekorvos-nagymama-tamadas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Forban-viktor-valasztas-csad%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fszijjarto-valasztas-jd-vance-lavrov-putyin%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fmagyar-peter-nagykanizsan%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Forban-vance-oroszok-orszagjaras-sopron%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Foscsadbank-nav-meghamisitotta-videot%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fvegrehajtok-ah-sebok-krisztian-titkosszolgalat-interju%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F09%2Funios-tagsag-euro-magyarorszag-kutatas-21-kutatokozpont%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2F27-milliard-forint-csadi-missziot%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Ffidesz-eredmenyvaro-balna-2026%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F09%2Firan-kozel-kelet-haboru-usa-trump-izrael%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F08%2Firan-kozel-kelet-haboru-usa-izrael-trump-elo%2F%23jd-vance-alelnok-vezeti-az-irannal-targyalo-amerikai-delegaciot-szombaton";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F08%2Firan-usa-izrael-tuzszunet-elemzes-sarkozy-miklos%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F08%2Fpuzser-robert-rendszerbonto-nagykoncert-majka%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fgyor-per-rejtozkodo-fideszesek%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F09%2Ft-danny-drogfuggoseg-dokumentumfilm%2F";"https://ad.admail.hu/tl.php?p=2l3e/m19/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fuj-utemmel-folytatodik-deli-korvasut-fejlesztese-ezert-aprilis-7-tol-ujabb-valtozasok"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>150 milliós Rolls-Royce-t azonosítottunk Matolcsy Ádám barátjánál, ám azt állítja, tévedésből jegyezték be a luxusautó adatait</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>08 April 2026</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fmnb-matolcsy-somlai-balint-rolls-royce%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260408";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F08%2Fcseuscsak-renata-birosag-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260408";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fjd-vance-magyarorszag-orban-viktor-elo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F07%2Fjd-vance-magyarorszagon-orban-miniszterelnok-megmentesi-kiserlete%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F07%2Fjd-vance-budapest-orban-elemzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Ftorok-gabor-jd-vance-segitokesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fjd-vance-orban-talalkozo-elemzes-mikecz-daniel%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fvance-amerika-alelnok-kepek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Forban-putyin-teljes-beszelgetes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Forban-putyin-telefonbeszelgetes-leirat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fmagyar-peter-interju-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Forosz-ukran-haboru-tisza-part-21-kutatokozpont-kozvelemeny-kutatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fwaberer-gyorgy-coming-out-facebook-europa-vagy-oroszok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fdirekt36-4ig-jaszai-gellert-hadiipari-cegek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Ftoroczkai-laszlo-mi-hazank-interju-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fomsz-tisza-budaors-magan-mentok-egeszsegugyi-biztositas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F04%2F07%2Fartemis-2-kuldetes-fotok-hold%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fvalasztasi-csalas-tisza-fidesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Frogan-antal-nemzetbiztonsagi-szolgalatok-50-millios-lakaskolcson%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F07%2Fheti-hetes-utolso-szereplo-linczenyi-marko%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fsenki-nem-volt-munkaidoben-rogan-szendrei-cecilia-es-sarka-kata-osztalekhanyo-lapjanal%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F07%2Flilu-miert-nem-szavaz-orban-viktorra%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2x/m18/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fdelegacio-budapesten-forgalmi-valtozasok-kedden-es-szerdan"</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>A magyarok többsége nem gondolja, hogy a Tisza háborúba sodorná az országot</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>07 April 2026</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Forosz-ukran-haboru-tisza-part-21-kutatokozpont-kozvelemeny-kutatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260407";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fmagyar-peter-interju-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260407";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F07%2Fjd-vance-magyarorszagon-orban-miniszterelnok-megmentesi-kiserlete%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fjaszapati-pocs-janos-farady-zoltan%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Frobbanoszerkezet-szerbia-gazvezetek-orban%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fvalasztas-2026-milyen-okmannyal-szavazhatok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fgereb-agnes-baba-gondozas-nyugdij-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Forban-gazvezetek-szabotazs-muvelet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F06%2Fpolitikai-nyomas-gvh-vezeto-kozgazdasz-berezvai-zombor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F04%2F06%2Fartemis-2-hold-elerese%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fjasdi-juli-tintalo-alkoholizmus-konyv%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fdebreceni-lakhatasi-valsag-iparositas-akkugyar%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftudomany%2F2026%2F04%2F06%2Fartemis-2-orion-hold-orientale-medence%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fvalasztas-szavazas-budapest-atjelentkezes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F06%2Fzelenszkij-energetikai-letesitmenyek-tuzszunet-javaslat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fmozgourrna-igenyles-szavazas-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F06%2Fmagyar-sztarok-gyerekei-kepes-kviz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F06%2Flovas-annabella-nagy-o-meghalt%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F04%2F06%2Fpapp-dia-serules-felso-fogsor-sopon-mk-donto%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftudomany%2F2026%2F04%2F06%2Fmatyas-kiraly-halal-stoke-fuge%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F07%2Fjd-vance-magyarorszagon-orban-miniszterelnok-megmentesi-kiserlete%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F07%2Fvalasztasi-csalas-tisza-fidesz%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F06%2Fpolitikai-nyomas-gvh-vezeto-kozgazdasz-berezvai-zombor%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Fdebreceni-lakhatasi-valsag-iparositas-akkugyar%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F06%2Fzelenszkij-energetikai-letesitmenyek-tuzszunet-javaslat%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F07%2Ftoth-vera-szavazas-politikai-kiallas%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F04%2F06%2Fartemis-2-kuldetes-rekord-apollo-13%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F04%2F06%2Fvizilabda-vilagkupa-magyarorszag-gorogorszag%2F";"https://ad.admail.hu/tl.php?p=2l2k/m17/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fuj-utemmel-folytatodik-deli-korvasut-fejlesztese-ezert-aprilis-7-tol-ujabb-valtozasok"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Orbán Viktor a szabotázsakció miatt személyesen ellenőrzi a Török Áramlat magyar szakaszát</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>06 April 2026</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F06%2Forban-fidesz-szabotazs-vezetek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260406";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F05%2Fmagyar-szerb-hatar-gazvezetek-racz-andras-orban-viktor-vucic%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F04%2F05%2Fracz-andras-szerbia-gazvezetek-vajdasag-robbanoanyag-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Forban-viktor-hotel-lentulai-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F05%2Foromhegyes-lezaras-hadsereg-magyar-szerb-hatar%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F05%2Fmagyar-szerb-hatar-robbanoszer-orban-vedelmi-tanacs-vucic%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Frobbanoanyag-hadhazy-vucic-orban-vicces-merenyletkiserlet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Fujhelyi-istvan-tisza-orban-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Fvalasztas-husvet-publicisztika%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Fsarvari-furdo-fantomallas-nyomozas-kondora-polgarmester%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Filyen-lett-az-uj-citadella%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F05%2Fcitadella-foto-kiallitas-szabadsag-szobor-gellerthegy-gellert-hegy%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F05%2Fhusvet-katalin-hercegne-rak-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Fvalasztas-2026-riport-bbc-magyar-peter-orban-viktor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F05%2Ftrump-hormuzi-szoros-irani-haboru%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F05%2Frubint-reka-betegsege-schobert-norbi%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l21/m16/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F05%2Forban-viktor-citadella-atadas-beszed%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Brutális Európába lép be a Tisza-kormány</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>25 April 2026</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F25%2Feu-tisza-feladatok-europa-penzek-vedelem%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260425";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Ftisza-oktatasi-miniszter-lannert-judit%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fvitezy-david-kozlekedesi-miniszter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fsemjen-kdnp-lemondas-elutasitas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fpodcast-haromharmad-tisza-kormany-miniszterek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F24%2Fpodcast-bazishatas-magyar-peter-eu-moro-tamas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F24%2Fromania-kormanyvalsag-kreml-rmdsz-bolojan%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fjambor-andras-lendvai-ildiko-interju-baloldal-jovoje%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Foktatas-miniszter-lannert-pdsz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F24%2Fmagyar-filmszakma-nemzeti-filmintezet-muhi-andras-deak-daniel%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Forban-viktor-helyettes-allamtitkar-lemondas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fradi-feriz-elfogatoparancs%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F24%2Fsajtofoto-palyazat-szajki-balint-mohos-marton-kepei%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fvitezy-david-kozlekedesi-miniszter-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Ftakacs-peter-anyazas-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fgulyas-gergely-valasztas-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fotthontamogatas-orban-viktor-rendelet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lbk/m21/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Ftorok-gabor-tisza-kormany-fidesz-light%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Karácsony Gergely: Fideszes politikusok négyszemközt elmondták, csodálják, hogy még nem döglöttünk meg</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>24 April 2026</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fkaracsony-gergely-interju-valasztas-2026-tisza-part%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260424";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Forban-viktor-helyettes-allamtitkar-lemondas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Ftisza-kampanyfonok-toth-peter-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Fportre-rubovszky-rita%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Fpodcast-torokules-torok-gabor-tisza-ruff-balint%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Ftv2-tenyek-index-belharc%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F23%2Fallamadossag-koltsegvetes-ngm-hiany%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Fmagyar-peter-ugynokaktak-feher-haz-bejelentes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F23%2Fszerencsejatek-gyanus-lottonyeremeny-interju-sorsolas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F24%2Fzsarolas-erste-bank-simor-andras-mnb%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F23%2Fszijjarto-peter-milliard-profit-feleseg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F24%2Fjambor-andras-lendvai-ildiko-interju-baloldal-jovoje%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F24%2Fmagyar-peter-csaladja-foto%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F23%2Fbaratsag-koolaj-unios-hitel-elindul%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2lay/m1y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F24%2Fszlovenia-kormanyalakitas-janez-jansa-2%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kapitány István Magyar Péternél is jobb értékelést kapott a választóktól, Lázár Jánost sokkal kevésbé szeretik a fideszesek, mint Orbán Viktort</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>02 April 2026</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F02%2Fpolitikusok-nepszerusege-orban-magyar-kapitany-lazar-szijjarto%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260402";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fmagyar-peter-andi-tomeg-bekescsaba-szabo-bence%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Ftorok-gabor-21-kutatokozpont-felmeres-tisza-fidesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F01%2Ftrump-nepszerutlenseg-elemzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Forban-viktor-tisza-part-munka-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F01%2Foroszorszag-lavrov-szijjarto-lehallgatas-telefon%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F01%2Ftiborcz-istvan-andezit-magantokealap%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F01%2Ffreddie-kozteve-vitalyos-eszter-komment%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fkosa-lajos-fidesz-ferrari-baszna-gabona-sikkasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fnagy-ervin-visszalepes-dunaujvaros-dk%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F01%2Fner-es-tozsdecegek-tundoklese-es-bukasa-jaszai-gellert-meszaros-lorinc-mbh-bank%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2Ffoci%2F2026%2F04%2F01%2Folasz-focivalogatott-elbukott-vb-potselejtezo-elemzes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F04%2F01%2Fa-kreml-magusa-kritika-putyin-film%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fvalasztas-2026-ruszin-szendi-romulusz-kaba%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F02%2Fpolitikusok-nepszerusege-orban-magyar-kapitany-lazar-szijjarto%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fr-benedek-duna-eltunt-megtalaltak%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fszijjarto-peter-tanar-megtagadta-bekesi-laszlo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fgyor-csaladi-tragedia-emberoles%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Frepublikon-haboru-kutatas-fidesz-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fszabo-bence-titkosszolgalat-tisza-part-orban-viktor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F01%2Fnyugdij-valorizacios-szorzo-ujraszamitas-nyugdijeloleg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F01%2Fkiara-lord-hirnev-szereples%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Forban-viktor-tisza-part-munka-magyar-peter%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fmagyar-peter-andi-tomeg-bekescsaba-szabo-bence%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fvalasztas-2026-ruszin-szendi-romulusz-kaba%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Fmagyar-peter-tatarszentgyorgy-gyerek-polgarmester-valasztas-2026%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2Ftoroczkai-laszlo-mi-hazank-visszalepes-magyar-peter%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F01%2Fszlovakia-szijjarto-lavrov%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F02%2Forban-viktor-hajdu-peter-interju-hazassag%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F04%2F02%2Ftrump-iran-kokorszak%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F04%2F01%2Ftrump-noem-ferj-noi-ruha-botrany%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F04%2F02%2Fartemis-2-felbocsatas-nasa-holdmisszio%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F04%2F01%2Ffreddie-kozteve-vitalyos-eszter-komment%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F04%2F01%2Fchelsea-rekordveszteseg-262-millio-font%2F";"https://ad.admail.hu/tl.php?p=2l06/m11/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fbefejezodott-del-balatoni-vonal-szezonra-torteno-felkeszitese-hetfotol-eszaki-parton"</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>21 Kutatóközpont: Tovább nőtt a Tisza előnye, 900 ezerrel több belföldi szavazója van Magyar Péteréknek, mint a Fidesznek</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>01 April 2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F04%2F01%2F21-kutatokozpont-2026-marcius-partpreferencia%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260401";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F04%2F01%2Ftiborcz-istvan-andezit-magantokealap%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F31%2Fszijjarto-peter-szergej-lavrov-felvetelek-orosz-erdek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F31%2Fszijjarto-peter-reakcio-lehallgatas-2%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Felemzok-kampany-kemugy-titkosszolgalat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fgundalf-interju-kemugy-ertelmezes-buda-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fmagyar-peter-gundalf-telefon%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fradnai-mark-fidesz-kitiltas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Ftordai-bence-visszalepes-ultimatum%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fzavecz-kutatas-2026-marcius-vege-fidesz-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fhann-endre-deak-daniel-nem-letezo-kutatasok-nem-letezo-szamaival-hozakodott-elo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fmszp-vagyon-parlament-alapitvany-ingatlan%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fmagyar-peter-sulyok-tamas-uzenet-titkosszolgalat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F31%2Fhaboru-odessza-aram-energetikai-terror%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F31%2Fpodcast-della-beregszaszi-hegyi-zsolt-mav%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F31%2Frakosrendezo-tervpalyazat-gyoztes-karacsony-gergely-epiteszet-mini-dubaj%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fvalasztas-elemzok-atombomba-matolcsyek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F31%2Fhajdu-peter-orban-viktor-interju-elozetes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Ftelkes-andras-allambiztonsag-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fkosa-lajos-ferrari-baszna-gabona%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F31%2Flegszomj-covid-film-filmintezet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F03%2F31%2Ffacebook-messenger-com-meta-megszunik%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kzg/m0y/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fbudapest-cegled-szolnok-jelentos-fennakadas-hosszabb-eljutasi-ido-terelt-vonatok-potlobusz"</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>„Csak azért nem tartóztatták le Szabó Bencét, mert nem akartak mártírt faragni belőle” – Bartha Károly százados a rendőrség politikai befolyásolásáról</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>31.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Frendorseg-bartha-karoly-politika-befolyas-szabo-bence%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260331";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Forban-viktor-gyor-ronin-security%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F30%2Fheti-hetes-rtl-uj-szereplo-hever-gabor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fgundalf-informatikus-video-tisza-hraboczki-daniel%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fmagyar-peter-drogteszt-eredmeny%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2F21-kutatokozpont-tisza-vezetes-fideszes-korzetben%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fnato-kibervedelem-gundalf-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F30%2Fmeghalt-nadasdy-adam-kolto-mufordito%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fmkkp-kutyapart-szekhely-torvenyszeki-eljaras%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F30%2Fpolitico-orban-gyozelem-eu-veszforgatokonyvvek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fmagyar-peter-gundalf-alkotmanyvedelmi-hivatal-titkosszolgalat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F30%2Fszijjarto-peter-allami-tamogatas-bayer%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fmagyar-peter-miniszterelnok-retteg-vecses%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F30%2Firani-haboru-usa-trump-forgatokonyvek-szalai%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fkormany-tisza-informatikus-titkosszolgalat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Frendorseg-bartha-karoly-politika-befolyas-szabo-bence%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F03%2F30%2Flabdarugo-vilagbajnoksagok-legkisebb-csapatai%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F31%2Fmszp-vagyon-parlament-alapitvany-ingatlan%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F30%2Fcurtis-a-nagy-duett-aprilis-gyozelem%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F30%2Flutri-lotto-szerencsejatek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Ftorok-gabor-valasztas-fidesz-tisza%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F30%2Fazsia-expressz-uj-szereplok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Fpek-szabolcs-valasztas-2026-fekete-sereg-orban-fidesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F30%2Fember-mark-szavazas-aprilis-12%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kz2/m0x/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fsiohid_0330_0402"</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Meghalt Nádasdy Ádám</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>30.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F30%2Fmeghalt-nadasdy-adam-kolto-mufordito%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260330";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F30%2Forban-viktor-magyar-peter-tulajdonsagok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Fvalasztas-2026-orban-viktor-bekescsaba%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Ftelkes-andras-alkotmanyvedelmi-hivatal-gundalf-kihallgatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Fkihallgatas-video-elemzes-buda-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Fmagyar-peter-keszthely%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Fivancsa-csatater-valasztas-2026-akkugyar%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftudomany%2F2026%2F03%2F29%2Ferdo-tuzifa-eromu-fatuzeles%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Ffreddie-szerencseszombat-komment-vitalyos-eszter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Fnyirbogat-mok-rizsak-ildiko-szavazatvasarlas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F29%2Fmagyar-peter-gyozelmet-bearaztak-a-piacok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F29%2Fbartha-karoly-pinter-sandor-szabo-bence-rendorseg-hamisitas-orban%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F29%2Firigyek-pusztuljanak-toth-gabi-papp-mate-bence%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kyh/m0v/rs/pj0/63u/rs//https%3A%2F%2Fwww.utinform.hu%2Fhu%2Fnews%2Fbalesetek-torlodasok-rendkivuli-kozlekedesi-esemenyek%3Fd%3D0"</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Nemcsak lelkesebbek, de elkötelezettebbek is a tiszások</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>25.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F25%2F21-kutatokozpont-tisza-part-fidesz-valasztas-2026-kozvelemeny-kutatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260325";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F24%2Fheti-hetes-rtl-szereplok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F25%2Fkampanykorut-magyar-tisza-hodmezovasarhely-riport%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Ftisza-hazkutatas-informatikai-rendszer-bedontes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fforsthoffer-agnes-fidesz-barba-trukkok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Flevelszavazas-halottak-hataron-tuli-magyarok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Flazar-janos-mi-hazank-lazarinfo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Forban-viktor-nagykanizsa-orszagjaras-beszed%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fpusztai-emese-nadja-ongyilkossag-nyiro-pszichiatria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F24%2Forban-jansa-black-cube-szloveniai-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fterrorizmus-elleni-nemzeti-lista-magyar-kozlony-vulkan-csoport-vulkangrup%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Forban-viktor-orszagjaras-kecskemet-mnb%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F24%2Fpodcast-della-jaksity-gyorgy-uj-gazdasagi-valsag%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F03%2F24%2Fszijjarto-peter-panyi-szabolcs-fresz-ferenc%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fmagyar-peter-orban-drontilalom%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fvalasztas-jelolt-tisza-fidesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F25%2F21-kutatokozpont-tisza-part-fidesz-valasztas-2026-kozvelemeny-kutatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftech%2F2026%2F03%2F24%2Fbudapest-comic-con-2026-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F03%2F24%2Fernyey-bela-balaton-dora-nevvaltoztatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F24%2Fkoncz-zsuzsa-politika-aprilis-valasztasok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F24%2Fszlovakia-szijjarto-lavrov-pellegrini%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F24%2Fukran-penzszallito-ekb-tek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fmiskolcs-szexualis-visszaeles-13-eves-lany%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fherczeg-zoltan-besugas-kabitoszer%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Forban-viktor-nagykanizsa-orszagjaras-beszed%2F";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Flazar-janos-mi-hazank-lazarinfo%2F";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F25%2F21-kutatokozpont-tisza-part-fidesz-valasztas-2026-kozvelemeny-kutatas%2F";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F25%2Fkampanykorut-magyar-tisza-hodmezovasarhely-riport%2F";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fkocsis-tisza-informatikus-titkosszolgalat%2F";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F24%2Firan-izrael-haboru-elo-hirfolyam%2F%23trump-megnyertuk-ezt-a-haborut";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F24%2Firan-izrael-haboru-elo-hirfolyam%2F%23trump-szerint-iran-beleegyezett-abba-hogy-sosem-lehet-atomfegyveruk";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F24%2Firan-izrael-haboru-elo-hirfolyam%2F%23ujabb-katonakat-vezenyel-a-kozel-keletre-az-egyesult-allamok";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F25%2Fsztrajk-noks-beremeles-maruzsa-zoltan%2F";"https://ad.admail.hu/tl.php?p=2kvy/m0o/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fmarcius-16-tol-27-ig-atmenetileg-modosul-menetrend-szekesfehervar-szabadbattyan-es-lepseny"</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Megkérdeztük a magyarokat, kire szavaznak az ismerőseik, a Tisza örülhet a válaszoknak</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>24.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fvalasztas-2026-ki-fog-nyerni-varakozasok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260324";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Flattmann-szijjarto-lavrov-lehallgatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fpanyi-szabolcs-lavrov-szijjarto-lehallgatas-orosz-szivarogtatas-orban-anita-tisza-part%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fpellegrini-szijjarto-lavrov%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Forban-utasitottam-az-igazsagugyi-minisztert-hogy-a-szijjarto-peter-lehallgatasaval-kapcsolatos-informaciokat-haladektalanul-vizsgalja-ki%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fpanyi-szabolcs-orban-anita-reakcio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F23%2Ftisztazast-szivarogtatas-europai-bizottsag%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Forban-anita-panyi-szabolcs%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fmagyar-peter-nyiregyhaza-beszed%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fszijjarto-peter-reakcio-lehallgatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Forban-viktor-hirdetes-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F24%2Fmagyar-peter-orban-drontilalom%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Ftisza-magyar-peter-nagykanizsa-tamadas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F23%2Feuropoli-eu-targyalas-kizaras-orban-viktor-orosz-szivarogtatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fracz-andras-szijjarto%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F23%2Fnetflix-dragulas-streaming-film%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fkinai-plakatok-debrecen%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Forban-viktor-brusszel-patriota-beszed%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kve/m0n/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fmarcius-16-tol-27-ig-atmenetileg-modosul-menetrend-szekesfehervar-szabadbattyan-es-lepseny"</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mégsem tartja hitelesnek Magyar Pétert a fideszes kivagyiságot kritizáló kormánypárti polgármester</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>23.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F23%2Fvalasztas-2026-szegi-emma-interju-lazar-orban%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260323";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F22%2Forban-viktor-hodmezovasarhely-kifutyultek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F22%2Fmagyar-peter-szentgotthard-keses-tamgadas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F22%2Fpanyi-az-orosz-titkos-halozat-orban-elleni-merenylet-kamuvideojat-kezdte-terjeszteni%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F22%2Forban-fidesz-valasztas-nagy-siker-lesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F22%2Fnagy-fero-dpk-masfelmillios-gazsi%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fszorakozas%2F2026%2F03%2F23%2Fnagy-adri-dpk-egymillios-fizetes-cafolat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F22%2Fszloven-exit-poll-nem-orban-szovetsegesenek-all-a-zaszlo%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F22%2Fdonald-tusk-orban-emberei-tajekoztatjak-moszkvat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F23%2Firan-haboru-kozel-kelet-energiavalsag-olajblokad-trump%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F23%2Futkozott-kifutopalyan-repulogep%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F22%2Ftotkomlos-bolcsode-bugyi-rendorseg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F03%2F22%2Fszoboszlai-dominik-margitsziget-vivicitta%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2kuy/m0l/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fmarcius-16-tol-27-ig-atmenetileg-modosul-menetrend-szekesfehervar-szabadbattyan-es-lepseny"</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Csatatér lett a NER szívcsakrájából, ahol a kegyelmi ügy és Hatvanpuszta árnyéka is rávetül a választásra</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>20.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F20%2Fbicske-tessely-kegyelmi-ugy-riport-csatater%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260320";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Ftatabanya-zsambok-tancosok-harman-haltak-meg%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F03%2F19%2Fukran-penzszallitok-provokacio-titkosszolgalat-kampany-ertesules%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Fukrajna-fidesz-orban-valasztas-2026-kijev%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Flaponyi-zsolt-rendorseg-arca-felmondas-interju%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F19%2Fforint-forintarfolyam-euro-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fvalasztas-putyin-tolmacsa-bojarszkaja-megfigyelo-ebesz%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fkocsis-mate-matolcsy-adam-mnb-botrany%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fgulyas-kormanyinfo-fidesz-orban-2%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F19%2Fmbh-egyenlegproblemak-babavaro-torleszto%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fervenytelen-ajanlas-sermer-adam-dk-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fnadudvar-metoallomas-csatater-bodo-sandor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Forban-viktor-ukran-zaszlo-fidelitas-nemzet-menete%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Fpodcast-foldosztas-macron-franciaorszag-kerner-pal-paumero%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F20%2Fbicske-tessely-kegyelmi-ugy-riport-csatater%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F19%2Fnemzetkozi-macska-es-kutyakiallitas-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fket-rendort-utottek-el%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Feurologus-husz-orszag-vezetoje-szolalt-fel-es-itelte-el-orban-viktort-az-eu-csucson%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fbencsik-andras-pofan-verne-magyar-petert%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Famikor-videon-bekapcsolodott-zelenszkij-az-eu-csucs-ulesere-orban-otthagyta-a-targyaloasztalt%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F19%2Fnmhh-mediatanacs-balazsek-birsag%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ffn%2Fgazdasag%2F2026%2F03%2F19%2Fnyugdij-utalas-magyar-allamkincstar-magyar-posta-2%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Ftorokules-elo-akvarium-galeria-fotok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F03%2F19%2Fukran-penzszallitok-provokacio-titkosszolgalat-kampany-ertesules%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Forban-viktor-ukran-zaszlo-fidelitas-nemzet-menete%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fkocsis-mate-matolcsy-adam-mnb-botrany%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Famikor-videon-bekapcsolodott-zelenszkij-az-eu-csucs-ulesere-orban-otthagyta-a-targyaloasztalt%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fvalasztas-putyin-tolmacsa-bojarszkaja-megfigyelo-ebesz%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fjuhasz-peter-par-orban-viktor-irasbeli-kerdes-valasz-legfobb-ugyesz%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Firan-haboru-marcius-19-percrol-percre%2F%23hazatertek-a-magyar-katonak-bagdadbol";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F20%2Fbicske-tessely-kegyelmi-ugy-riport-csatater%2F";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F19%2Firan-haboru-marcius-19-percrol-percre%2F%23ot-nyugat-europai-orszag-es-japan-kesz-hozzajarulni-a-biztonsagos-hajozas-helyreallitasahoz-a-hormuzi-szorosban";"https://ad.admail.hu/tl.php?p=2ktf/m0i/rs/pj0/63u/rs//https%3A%2F%2Fwww.mavcsoport.hu%2Fmavinform%2Fvgz_120a_0320_0322"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>A nyugdíjasoknál simán vezet a Fidesz, a 30 alattiak között majdnem ötször annyian támogatják a Tiszát</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>19.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Ffidesz-tisza-felmeres-demografia-21-kutatokozpont%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260319";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Fbekemenet-orban-magyar-tomegbecsles%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Ftragedia-honvedtisztjelolt-lezuhant%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Forban-viktor-dunaujvaros-orszagjaras%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Fvalasztas-2026-mandatumkalkulator%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Fnagy-ervin-dunaujvaros-kampany%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F18%2Fmagyarorszag-jd-vance-latogatas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F18%2Fwang-mester-interju-kinai-konyha%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F19%2Fnadudvar-metoallomas-csatater-bodo-sandor%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Fhegedus-zsolt-valasztas-2026-egeszsegugy-takacs-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F18%2Fvarga-csaba-betalalta-nagy-ferot%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F18%2Fschilling-arpad-kossuth-dijasok%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F18%2Ftisza-judak-zsolt-harta-magyar-peter-kalocsa%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ksx/m0f/rs/pj0/63u/rs//https%3A%2F%2Fwww.utinform.hu%2Fhu%2Fnews%2Fbalesetek-torlodasok-rendkivuli-kozlekedesi-esemenyek%3Fd%3D0"</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>A legjobban kereső miniszterek fizetését is lekörözik az álláshalmozó államtitkárok, amihez egy széles joghézagot kell átugraniuk</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>17.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F17%2Fallamtitkar-allashalmozas-allami-cegek%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260317";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fpodcast-haromharmad-marcius-15-bekemenet-nemzeti-menet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fnavracsics-tibor-bekemenet-kulonutas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fmagyar-peter-kamera-felvetel-nemzeti-menet%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fmi-hazank-marcius-15-toroczkai-laszlo-video%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fmagyar-peter-tisza-nemzeti-menet-rendszervalto-hangulat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fszafko-zoltan-peter-interju-tisza-salgotarjan%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Forban-viktor-menekulttabor-ukrajna-kaposvar%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F16%2Flengyelorszag-donald-tusk-orban-viktor-europai-unio%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fpeto-peter-leborotvalt-orszag-konyvbemutato-beszelgetes%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2ks1/m0d/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Felet-stilus%2F2026%2F03%2F16%2Foscar-dijatado-gala-2026-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>24.hu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>„Minden lélegzetvételben érezni a rendszerváltó hangulatot”</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>16.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F16%2Fmagyar-peter-tisza-nemzeti-menet-rendszervalto-hangulat%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_20260316";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fzarug-orban-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fmarcius-15-2026-tisza-part-orban-viktor-fidesz-magyar-peter%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Forban-viktor-marcius-15-beszed%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fzarug-peter-farkas-orban-oriasi-kockazatot-vallalt-a-beszedeben%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fmarcius15-bekemenet-fidesz-tisza-valasztas%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fmagyar-peter-marcius-15-beszed%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fbekemenet-marcius-15-fotok-kepgaleria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fkijev-tajekoztato-baratseg-koolajvezetek-druzsba-czepek-gabor-orban%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fmarcius-15-nemzeti-menet-tisza-galeria%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fmarcius-15-2026-tisza-part-orban-viktor-fidesz-magyar-peter%2F%23toroczkai-laszlo-holnap-elmegyek-magyar-peter-hazahoz-uzenem-neki-hogy-legyen-otthon%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkulfold%2F2026%2F03%2F15%2Fzelenszkij-putyin-magyarorszag%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fbelfold%2F2026%2F03%2F15%2Fkaracsony-gergely-marcius-15-beszed-valasztas-2026%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkultura%2F2026%2F03%2F16%2Foscar-2026-sean-penn%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fsport%2F2026%2F03%2F15%2Ftottenham-hotspur-szenvedes-bajnokok-ligaja-premier-league%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Ftudomany%2F2026%2F03%2F15%2Fmohacsi-csata-ulaszlo-honvedelem%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_";"https://ad.admail.hu/tl.php?p=2krf/m0b/rs/pj0/63u/rs//https%3A%2F%2F24.hu%2Fkozelet%2F2026%2F03%2F15%2Fmegosztottsag-erkolcs-ipsos-magyarorszag-felmeres%2F%3Ftsrc%3Dhirlevel%26utm_source%3Dnewsletter%26utm_medium%3Demail%26utm_campaign%3Dnapi_"</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Developed and tested link filtering+extraction origo
</commit_message>
<xml_diff>
--- a/research_data.xlsx
+++ b/research_data.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.77734375" customWidth="1" min="1" max="1"/>
@@ -1052,6 +1052,908 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>25 April 2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/CBQN2XIM43EON4E3V3WHVKA5Y7S2YSK6YPDFD7OPKXJT2CCKTLSKQ6UNEMHBEA6EW4IUXXGWB2YYVXRM6IEGCEAMEGKLENVW";"https://ct.automizy.com/8/B7RDFE4YJLFKKNQK2FXEW6MREVFURP7VLTTYZYLOGC3GCLUN3RHD5OOBXY6XMGU7M727GRUGDV7KEHSZAHBLEQKL3S2FMZEU";"https://ct.automizy.com/8/BEKKOGEOWF3HHU3AHETL7NTMMJ4GNUHR4CAOS6INHVPG7UNIKGEDF2PDYGCKMXFNZMTRWA2ICE3NCRC327KYVSUD3ENEHNYB";"https://ct.automizy.com/8/SN56T3EVUZJSBJV72THB6ZUSVHAHFATRW4KYPORCPF6G3M6FEKHH4TOVKNCP4EIMQDEKJBG6OKLTZDQP6UTJV67ILGXMPRDY";"https://ct.automizy.com/8/BRATTYO4TGO7FVL36W3YPPS3FU5BTOEY24TBJXNKIZEXLUVMDSHFBY5ZC4DFKC7OZZCYETXEMPDMHDCGJEHQSRLIG7HCNNIW";"https://ct.automizy.com/8/D5P5G53EWL5I5FO7H6QLZ6HNEFY4DMEDIFEWDFCCKA7WUJNRMV5AAIUFMP4VBFL26Q6HX5OQORZ32M54U62PV4POOI66O4MH";"https://ct.automizy.com/8/Q5ATLOUI32SF5YECIEFNZFRAQPEEBJ2APD5KSMI5TACIRX6ZRBWIHPKDACTSX6CLEAUL6TBBFEMTYDEBW7VFU7VQA67FTJQQ";"https://ct.automizy.com/8/JLH45HDMF7EHMYWXU5GCLVTUILXUYDMQAHESP54X5QIMG7LHAYRH5UK5XQKE4QKWR3VJGBMW6S4KVLFYVZJU6LKZ3QQY4GKZ";"https://ct.automizy.com/8/5DEBV5YBT3XJOVCP3CUGRS5AZOJMQ3YYEEJZEYY2TNMEPJEJY7ETTQ5JHYRA4NE7ORE5HZQGGCU2S7XLU5GDI4MTFPUFBQNL";"https://ct.automizy.com/8/T3426SNQ3MFZV5U6WHE2SU3U7MY7MIA2VF6ZALQ3ORU6GKPPV2A5ZZA3IM2DET72DNDJA52L46IHV4OJZJLDKYQTFUXKCRXH"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>24 April 2026</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/E6DD7ZYYKJKU5EQUPCZKNS5W5LXEI67WO4SM536FE6EKJDPKCX4FTLPHNQRIQPIIOD3MDDCO4UUD4R277DOGU2ZWDXZQKHWH";"https://ct.automizy.com/8/TIPBDEOMXJEPHPMIPSKD22HHDSPDCG2IN6I26AO5MDNXZFD6ALE3WRWVHJPOUESPKXPC4SNZPOEQQBBCFXUKOC7SNUNCXOMD";"https://ct.automizy.com/8/U4ABE5RBCIIKGY3HTJL3BK6SFFBYDINAXAML7ZGRCNVYI3TFAOGGOEQQJ4J6ITZIGEOUJVB3UPHZFH2LS44D5PJNIHDHW2LE";"https://ct.automizy.com/8/MDANCFOV7QIOHD25YELJJDL6FPE3F4YFW4RPGF7LLP4U5VHU3LUGD2MUXURN5K2E2QLZ5FORD3SX4TLLYOAGSLOWKYMRIVAQ";"https://ct.automizy.com/8/A62GWIII2Z4FXUOY75DOVDPNCSLQ2FGLARPQ666P7LWCJCLS2EXPTBVAUIEWO5KP3T2V4PIGP55RDBJ5AIXIYBNQBSA2J3SO";"https://ct.automizy.com/8/EMTL6WE4VMSBJZT4AGECLPYBUBQLD3G23E76NJBZTKZIVUHZMHQ5O7BW6UQWCXHST3AJVYC45FQNEIWEEHNUBC3VPUCW6IMV";"https://ct.automizy.com/8/HFPUESIB6BI3M2JBGAUI5OZHPR5D4DGEJN4SHBJJJPDQRTXEU5ZPBLU7P5ENHVFEXVUL5APQP62N2MTHTYGXQSC6K3IYMKTQ";"https://ct.automizy.com/8/7NNVXNKMU6A333NJH7FLYGTKXYGYQ4W6VLHXJIIB5SAERQ46RKXDDGIZ2TG6BVBZRMSYR5WLB4SA6NPLJR3J5MQEYHYQ7EZ2";"https://ct.automizy.com/8/F6CYNAXHPIMNBOLBEI5VNPGB7U76HHSPADLPR3SGLKQPXDH4DBOEZL3QMCYX2E2P7R3NHZBVDKUKEQBP7R2WX4FKAJRM6IV3";"https://ct.automizy.com/8/QPOJP6OGBFPVJIQU344QX4BNQAINJLBG7P4GV6GBX6OFOPE3CX5RYG5CIYUNFVTHZTPAVNVIARERIIO5QEEG3MSHZHDRMHLT"</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23 April 2026</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/ZKAYC3U6TEF6IVX3DRXEJJEFQTTQTH5I6B3CKLYUCVFJJSB6DROJOQLP7BRLJWWUYDIN4XXOLBWIMJQCXI7GHSFCDKZMOILL";"https://ct.automizy.com/8/XNXGMEEDX2UUSIYD7ZNOBKWX3YUNZC4ZL2NWFB542DKSBN6L473MJZE35I52RIMW3YHQ2IPFTW3N3Z25GJM32CWJ727VSOYE";"https://ct.automizy.com/8/YE6G6KD2JB6XY4BQCJKCL3UOIZ6WB72J6347VJZ5B646OZXS3EP5CR5ZSYZFQKHBH2NLZXV2TL2A5HSKVKV4IMYATORBQDYV";"https://ct.automizy.com/8/O32C6RYLRFBKW3Y4XK3MCMHRVF5MHQONTLBREJLM4MDMOQY5ERCMDNREP44QN5BPZQV4PF3FQDQKT2LZBGPPV43VE57MU7RS";"https://ct.automizy.com/8/HQJTGJHY2EKDDK4FZOWKXZGESO56QPAYTVINTFJZC64AXIURKP7WUUDIX55NVN3XMKEFUULFQWGTCQ4HYTQQ52DQ5BY2S75E";"https://ct.automizy.com/8/DLLTYDTTRNXROAARDNYSQPMFADHBPCQLL5RFIMXWIDEOE2R72H3MCUSMXCSALKTEYJGCBQMD3F3BZDV7U22TRDZRWRHVPLPD";"https://ct.automizy.com/8/5Z7SGCBEXF722FX5ACAHVAM7CJAQH7ZLEWQEUGULWWGGY7HHGBJECEUYXUO4ZE76EDXZ7EIE2N47ODQQ7PBXLHLF3AITBWES";"https://ct.automizy.com/8/KH4BQMKJX3CEYYHYWLJZUSD4ERRQ5OSIU2URKTYLQ454DEOQDM4GRGD6BEOIJQGY2EPKJSBZBBJGATB2MJTZQUGYPFO6RVAU";"https://ct.automizy.com/8/6USDETFEMV645L5TJCLRENPQGTSZE46EX7WXJQZDHKGKAOCDWHPVNC6C7WEFURDVN74HRHLDYJCGBAXAGKDK2Q4BNFZILNNI";"https://ct.automizy.com/8/YRZJ75GHPWEHPDWFF62AO3MUOEORGE4KTN5WIYT6MJGRAQ3FDJZVWOJBCZKGQ23JF5IDY6WFXOXUHMVT5KL7SKZTB3OP2NLE"</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>22 April 2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/VVL7G5FIDKND3FZ3LZ65RXIZV3DAZX62XEDE6NVG2P2FNA3Z7FOLE642D7P2WFMREGUWVK32ROFHNLFBYTYOJ5LOKRYQETSI";"https://ct.automizy.com/8/ZAWE6MS4V5KGRASLRRVC3A6UT6PY64S5GRDTUTHUVD2L4NCTJZ5QVSPFTN5UFLYQ7K7VWYDE4KU2HIRUH5IWB5DO2ZWRZ6L4";"https://ct.automizy.com/8/D3SPLQX7VLYWFGAYIYKJ7KK2DE2IQRMTL3FUGIUUUBCXPLKV3OBVFSY2JMRLCIFSPYDAQ75UUHFGGKE3O6B7XNDPMNZKDKQO";"https://ct.automizy.com/8/4UR23XD3ZHP5NY3F2W4XZJUX2EUHNPSH5TPAD3KWTSJVAXFOSTZ2OH4UO4KCGN3GD6KQI6S343WUSYUBWDYXYDV7A5UBXLYK";"https://ct.automizy.com/8/IYGRUILQIIW2KXWK4S3OM3RJTI2GPHCFZIGYA26I3JSMM5WNOBWKEUKGTBL3KSRWPNI7UBFKDPLKTOPUJWB4LH3R7VGST63T";"https://ct.automizy.com/8/PI4B6D7OPH4ENBXQFBS2TOT7MOVEUNAMSG5CTE57GDBPJLHAL43OBQQKTFFO4LQK7LTHA5UPNXWDBLU57ODGRWNRICM6Z2G5";"https://ct.automizy.com/8/P6AGP2HGFWSIR7TLQQUUGB7KT3GGKGOGKCRA6TT5WAD62JJIPQX5SGQWFNJITKOG2RWHOUQ6VF2FB45TXPEGBSLMFVS4BHCT";"https://ct.automizy.com/8/MFQP2FHHNSRPCC5JOKUMQLEZQAZE6LFJKPNUQDENFQGZD7SS23UIH76FQELEKG2EQLKF33KFUMKZ4F6G7CUJRH5QVSOQCVPY";"https://ct.automizy.com/8/SW4KFZAGWSNFU5H7WTYQXUMQ3NZH2K7XNTXFMTHSRTJIXHYF55UO6YXJYLD4IKG7IO6FRYDWQSUHVSRXDMAX3CA3SCWX4PJP";"https://ct.automizy.com/8/7E2P5HUPPF6TSL5H2XL3IUROY322RN46WQVHD37J3KQIN5YWXLUZQ7OIBZKZHNSDP3Y54JAZUM6NGNTH5EM4JAKJAPYV53RO"</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>21 April 2026</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/IGAERI5WV64BPJGULBYZAUR7Y7ZKSFCIQOVWGWQNTY5OCQD4LM344NJ7QG2SCV5X2YXSWLREUN3XZKPUC6YEIN5GENNPGREB";"https://ct.automizy.com/8/6EC25CJYARGU2HK3SCZQNNXBIUCYMVOBD6OH3CXEUKVVKHYR4GX2YOS4TZC5Y2Q5KAI26F6FDBHQUOMLURK2DHFFJ2N3TTSU";"https://ct.automizy.com/8/GIFKUWHNEUCCL6MHCLOZU5RWHATZQIGF5SIOJ3NAS3NB5NIQWEYAVCM27GJHDIWYBMTMR72HZU54S7XTTUNW53INXCOT5ANS";"https://ct.automizy.com/8/XLTMB3MSS7J75RNR2SIA3C7RXK55MWRMKERLF76VAMBGEUFFGQWHPZKDLYCB76HRPXO4F75VGXKESNHAI5XLX6TH6TFR6ZME";"https://ct.automizy.com/8/73POXQ3VLBOLUV44YK2JDBZ4CZLEJWNSBJE4VLEOSB7OXNSCX23U7KGRCW2RPEENGOZ6P5CYXU6FPOLR5QNMPBNUNNOMHOYT";"https://ct.automizy.com/8/N7U3IJSVVB2FIAVRXSVDUMXBQNO4WSN4KSX5JWGBLOULJ4KCV55FWPORUS67C3TSAQOJVABM6HVZ4RHQQUHXWHBCYKVBEKZ6";"https://ct.automizy.com/8/44DOTD67RSQASJIXZTS3CLZDBJGNYAXTWMFIM3AVG4NFDIU7QUG2JC3FHDT2KTNOAAITGF3UU6XOOLX5M32D2IL4GKCQNDBQ";"https://ct.automizy.com/8/AZCIAWEWYUZ2R7MZSG6VY6AAJI64RUJ6LBD3WM3LVZLE26TJ23WKAB5RW5XYLOLO6H5FCDYEZ5KSOKISZ4HVFFQS2KVISE6K";"https://ct.automizy.com/8/DWIFEP3BXWXCM7QTBTM7FNNILGG2L2VWATF5QSIWRCXV25PEKE6X53OKQ2HL4EUOJ2ZQIH5H3NQMLUZGMNDQHJIQSUMTGJ42";"https://ct.automizy.com/8/URK6KWVIY3RZDCNJTC6RKKNQVWCZ3Q5TKHJDS3I5OKTXBSOY25754URPVPYYZQXSSLBRVFAAZBY5UPEZKCSK3TPLL6OTMH57"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/4CX4FSD4BQK5CVWZRGOPABG7UQ6XYX6OWUZOE6ACSR23LW4MFSLFNH3NKQ4WI7KN626EHPUAEQE4QNFTSRV4POH4ELLNOKO4";"https://ct.automizy.com/8/K4T2JEHWX437OB4TAUEMTYAOPHOOOKF3F7AZASFNYHDFDOPA3YQPIPG5RWR4UM3455F3U5TYNILT6RACXVCZKOCJ4BQCAB3Z";"https://ct.automizy.com/8/IJACZKZWBGASDBJYCW4HVMJ26J6TQTYU3EFR2TK7DMP4UMOI6QAP4YWBACQM5BIWBC2CRBA3Z76JSGSAUPDMBUYQ5ZXIP2PW";"https://ct.automizy.com/8/JO7R6SMPNIQFL24KWPRZEH4J3KAZC5J3QWMIKIUJHLG4UDUBIX5KER7KO6M4JZKPAIWO53RLHPQHJYUO4C4COH6LBDXKJLBD";"https://ct.automizy.com/8/SAF7GUAX7H6JTN7EIMKTCA6R5T5POT2HF6G6LKGEIXFCKEAUEYGYHX4PQN3BOJP5ISCMBK4PXS4YBH2SGNFPJPQ7IXQ7KM7N";"https://ct.automizy.com/8/WOS7RGTUFNZ6RMXURTVWEDDXIGAAG4LC6LZR77SUTAMBXPQUTI7ADPB7NLJAZCZ6AEMNETKZKQOMMWJSS5PWO5GPE3HOEQIO";"https://ct.automizy.com/8/ZX7NZP7NIJHZFOJ4AXYMDL3ZEA4VPQCKTIWB2ACGGDOGALXQSN7LNJYAIUEY3I7KF5EZO4QTMBBMNBY5XZCQSIANDCCOJ3IP";"https://ct.automizy.com/8/SZFW23ZPLY5U6LORBBZXZ7UGE2GGONQELVJZ2F6ZQPRF265OPLCL2G5FBPNIWT44FJ3BFNS6NSFOAQ6VNOR5ZMUKPB7LLMRJ";"https://ct.automizy.com/8/4ODGKFXGOWKGCQFBVPAVCPICYG3JFSET7QWNVSIVEEWWMEQT7GWIOPVTY2M2GP6MEIGQTWAV2AO3OMOIHQ36HY6YGEHNVGIQ";"https://ct.automizy.com/8/EZZTVXYOHOO7VPGEQAK47VM5Q5AHYQVFIJQE3WHCBCVW7FXPKHAFCSWB7AWSNSKAG5ZHUDGG3JH74XQPG62XVM4Z25YJF5WO"</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>19 April 2026</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/U33JL22IAZS2T7AXPMBYRWLHV2A7P6VN6KOKBRTXYSUMGCPTA4DPGU7PQF6HQKYY3R6MWAQRACKL6VF7PI7RILUWENFSKYD3";"https://ct.automizy.com/8/5OWXDCVCO2XFXEV7VIUSCGACMJHT245TBRKLIXSPAYS7MA5WPK6RGC2L2KP37DLS4BS2ATX32MS4IQSLPUT2MPX24MUKH4D4";"https://ct.automizy.com/8/OGKDGA6LWP7CRDMRJWB57IVT2GUI2Y63RSRCHR56WNTXC6QUMWDGO3FDOUEZQE6TA5K4JBHJGFVFKT2W2GPF3AX4GOOWZPPG";"https://ct.automizy.com/8/R6MTH3AUK4DNJRL422T77DU4ZQLFTD7STDDYXIYKZXKJU42NT6RHDSBN4TYOULINU5DP5YMOIDIRPMMDBZJG6MJSPAAXA3AA";"https://ct.automizy.com/8/DXGJU7WV6SYOUJOTDNU2EH6CXWBKHRB6DLO6URS54FBC7PLL4SUADYABFDSPRRHBPSKMLH6RZKCD5EV35I6H6AGIVHKN7RPN";"https://ct.automizy.com/8/M3A3XKE5OCWNOBKPTTS56RSV3MQG5HGTAP4DVO3IPLARXCWXS2KQWS4EBMX6THB2LHO3MI63MGTPUV7J2BGIPTSSWQV4QWYQ";"https://ct.automizy.com/8/MIFRCTMQWNIVD2O25LH57XD75WSA6A7UUS6AUJUSQ53C35ZQKZCTQ65WLHR5YVTYBXHJBAHHXCYLDCBE6G4ESE7ENGQOWBAG";"https://ct.automizy.com/8/HV32TMVXOII525W672W7R6TLS5MYUK6EQBVCAHORGSTXWHZPKMWU2M7HIXMCAYSNSN3OOXLP3RACTM2PP24TAWDNJ4JEFVUE";"https://ct.automizy.com/8/7JVB5JCYRNQUNNOIZOACXMOJHIEMTEQQTBKNTUPAEZZWQ6SLG2AR6GV4R7WPETDRPBG3AHWCEBYKYJLN3JFRCZJ7ERJDUAD6";"https://ct.automizy.com/8/DC3ADO4A4VHP2IIAHWO2X2PKCSCUH2YU45QTZ435S4BH7RVLHYF4EKYPL75E27OJMVLHHWPYTW7EXQQUJN3ZHZEZSDLX73D7"</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>18 April 2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/BLJLPTSQAFWEOXPJXMJ6CIHZAE2SLTD3YDKJ5E5RHTBN77Z73WLOFZIQSBMGYLOAGSLA2ZCOOAW2CKTV4VFCUE5INOR2YJGC";"https://ct.automizy.com/8/6YZ5Z4W2K76IPBAT3QKMWXQITVGQGNEVWZTQQVQBKIKXNYWFUNT4Z5ZKMPZFGMX7KXVGYN7OVWNS23OUQKAJJFGYCH6LIUZR";"https://ct.automizy.com/8/SC46KIFANQF2SPGBUWBN3ZHX4XIZACY6XSOZ2JQJ43IOSY7M3TIXZT4BAL73C6HGEWJJUCG5UMCREABZAHV4HDMGWVO7CDLM";"https://ct.automizy.com/8/NDHSJMHIX6C3NVJGZ5SNETJMAGDX5RXWAAVEVG33F2F5CDYS7YE5WBQM6ADG3QHSVVXA6XHOE2NIPTGWNESKXUZFORPPOBI6";"https://ct.automizy.com/8/X2YWROWNMABF7XADB6RX6CSUNEPPIBEQUS436XQDXR4HNPE27K7PJUENPNJAJINWCDYNRVSMLWG3JQGOSERK6NQS5RD4TE3I";"https://ct.automizy.com/8/JGM54MFX3MXX5LOPTE2J4KRZUEKPNAX2AMXZQZ75HSDFNP6RD2FTU3L4AR6SKVSBEXAEKWLVM3GSSMJ72KXK4A4HBDI4CEBV";"https://ct.automizy.com/8/WTWTQDBUBRYMZKNV6OGLPW3XCZASBLQARCJIUIQLBFV2YDRLOAGOPBN4KYCJS6TZRWOEQK3LLF64IYXNIBH3J6F5CYZBSEWE";"https://ct.automizy.com/8/XWFQTC2C2SB7AFTXJM6PD5WEUVDIMBF7DN55KT47Z2NUORJWP3EOZJTSMYJGOVV6UK5NOVIH3UKKFAD7PUNWHKJF5Y5KZFHR";"https://ct.automizy.com/8/SLMPQA4CRWIPUUQ2CZJ2VTLONOVRHCBP7FZ3ZVMXMGBFWAURVYWKOEBKPVC6IAO7UTYFVF5DXGUEWQLQDPU25ERKC4TV7RQQ";"https://ct.automizy.com/8/RMSYXUUSIYDXFJJPHGWF7N5IUPW6MHC3ZLTU7KLYZMO3VLTUB7BHBT7B42EK624AGPX4EHKCVU5UM7FSO2Z53DVPRBYOWWM6"</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>17 April 2026</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/Q52IVQNBEJC3SZCUK5ODCB2DYSTW4CZERWKGXGQTKJMRXTIQSJYL5LMKBMRM6TXUILYXGZGGHMQOA3QV4XNNCMCHYCURYAV7";"https://ct.automizy.com/8/BJHLXIMDINPKPY2UA3ASOMPRXO3CXVMOTSV3FF662AQ5JQKUGBRFFDMOVDPGAAI55RCOXD5KXDTDBUTCF4NPHDCFQFXC657M";"https://ct.automizy.com/8/GY3O7DARAOM27EKUJC3ONE6M3B4ZZSJVR6LZ64BOR2Z3Q2RR6H4R3HAEVBHZY7RJKHR3FXN776EKWBPQYOUY2SWKGCEECTUS";"https://ct.automizy.com/8/A44UPDNK64AHVK6XKTOMBDLA2CLTDH7D3YOSZI7TQDART4XIMSWTG34KBTEWQGLBDKO2ROYKMZLLHAWR2J4IPCYSN4JZWFEV";"https://ct.automizy.com/8/4A33KXTQ7VHZKDRD5HRUJFLN3QA3SKYSQANOXNB55BFIT7GR3INBCGPIUREN4OLVOPME4WODUPTJS2DINE2MHUOTNCNVJVTS";"https://ct.automizy.com/8/GOWMB6UXPBN73MRLAD4X4QKZJFA2STGAMAYQEK6WHTKTWQWBQY2VAWU4HBGYSA6FPCRNATFD7Z4VCLGFNSN2PNIOB3VB3MFY";"https://ct.automizy.com/8/OLM5CPMQ3NHRHAW47Y4UCHU3FBMS3VBY6WOP3EMMNN4DLQKEUQ6WVJ36OU7T3NMAQE462XG6DO5MM3HQ4CDU33SM6OG7SRSF";"https://ct.automizy.com/8/GOOGOFHZH5ZYVLX4ESLWMHF5CRLOQKZJXX5IQ52AMDDBRLECPLTL2E44WAJCA5M7PGI7LWZQJHDAHC43EF3VYRHY4WSAERMU";"https://ct.automizy.com/8/UCFQ4FYVN2INWRNANY5KNQYZA2PDDOXLZD4HFPBSSGGIJRDFV4ZUOSQBRHBEGMJZZORFXVY3PEVECG6Q5TU64COR6PX33LXQ";"https://ct.automizy.com/8/PMPWTAFLJLR2QIWZ7NUDGEGUI2RFH5ZVC5CCRZRCDPDKKWOTDLHMWUKBUQLAWS5VZWTUUUFMQSYO6I2U3PVCUOJJZPEYLC3P"</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>16 April 2026</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/ANFHRK7Z23TSASPYAARHQC644DJYB45PDGII3UBGZXHSY7OSVHXTQPGYP5BXAGI4U7ZURQGAEPVBD275UBFOQDMBIBWVSZYL";"https://ct.automizy.com/8/4BCIF6LTO325YUMD6HGZQXY3FR2RIU4UBKRCV5MKDP2DRLQSBRSETDNW2DKOPF5L5UMCCPKL2H5LYN3LVUCNQ3L2UKPHXBMR";"https://ct.automizy.com/8/JWM76H42Y36JER7QSOUJOFGZAJ2SOYWMPNFTEPYHWXM5Q5ITZAGDJ4FU273ZNBIGBWXBS3MC732WRQ7SUPWZ34Q7OKKFPZSC";"https://ct.automizy.com/8/57SY5ANLZKLHBKLZHVGMDF4EEX2USIHMKQMYMTNDRX46ABXCDICAEIB3HPHYD2VVUEBFSNLZWANOMSLDOP2E54GVUUQE6AEM";"https://ct.automizy.com/8/VU6RABOGCFBHXMMAIZ67RB55QHTW6JKYDM7ZI5S5LTDTIHSLLBV2FKRIPISBPZ3RWNTQXO5GVOZ2BP7CAINB2EYPRJZS6HFU";"https://ct.automizy.com/8/GGUJOFZLTZNHAHYC2UHMJAGZDQLI5KNAFSRG57O2GV2L7P2BDKCQKV2BIDRAHH7JFMN6CWV6X5PX7LDIJMTZKQ3QOUT2FXB7";"https://ct.automizy.com/8/HVFTTGWCIVIUDEZH25D7KKX3F42VOT56U2V7QGH5RIXQLY6DP52S4NRRG4BVZCJNUM22IZ2RW7UNUECLUT542YJG3CUOBJ6S";"https://ct.automizy.com/8/XPWVVSPRFGCENJ4UET4LUSK6VCJG72K7OOLIGQ7HSMXVSRRBQL25HCT5UEBRVKMBVQHMYUZVCZRRSDMKPOTXCRZY7XSZLQVI";"https://ct.automizy.com/8/S7MCDFSDJKX4NHNNSSZG5F47QYE4I2LTK4B5Z3ELNXBB5HLJ6RYSA7M55ZKQLVJCIP6B7Q2IQDQGYVMPFSHB6JPFQ5JNXITZ";"https://ct.automizy.com/8/62TQEXY4CM2BYHBXB3TAE4IK7FWLM353TS32HSRUR2FV47CF3BJVCFGFIMBVLM5NU5DHFE7FBYDIV77HFKL7W2UUD6V5D7V2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/4QXPPWLZXOG4OABOYLUQE5R5GW47F6WTMFU4CNW2IQPIJYY3Y3DZ5OVOL27QPQLIHRC2DU7R727R2EVRFSMZC6UNUV76U3VM";"https://ct.automizy.com/8/BOQACJTR6777NE6DUAKU37BIOZACR3SD2O3443THLGKBLK34GCBWXT7KNTNMWSGMMPEC62OETWFRSXVFHNNQ2TP3S55L5F2Z";"https://ct.automizy.com/8/LXHAOLQQM7GNRDEWRH3RPEAVQHWWCQ3HN2WDONRL6HROY74DXOLAVRW4NHMC4FTFTGDI7YZM57DKK4ADHHLY7W3JZO5446M3";"https://ct.automizy.com/8/YLB2Z27GX5OTTMHK4W3WXVC3RWTMGLP55IM545QSJA42TE227OF4LKBMKJQRXUHJ37ETHJA5WAZ6P6VBPM7NTJHIJGPRNPSK";"https://ct.automizy.com/8/6GJLTSARNNRQPECPC5VRY3CQX7UL3CENUGC5MSFE2JQZPH5CPBM56SABLILUI623KYYJTQQV6IY3UGP33OBOZSLJI26ZOC4I";"https://ct.automizy.com/8/BB6ZED7FEMPVLMPWK7IUVFXWCLUUN3JALKY4M2NCCJWHQ2D6DROCINTYWI5WMWX4REHATKTV42GCTXZLLYUWMO2WLN7E4ZOZ";"https://ct.automizy.com/8/3INB2KXF6WPVOQNFKWT7KGUIO6OV7UO4KVGUT3EGYHN7BO7RJYCTTBFOOMO6PNIRLIVRL2UA7KRLZHF67MUPR23672WMEFOR";"https://ct.automizy.com/8/FRC5RZCQ7KCMY6RSPAJXDLOUPIUBFUPNBIVXTI5GIZZOUTA7LVD6ACF6GTJ2X6NEDZZWV43GZMQ3E3IXAQAWTXURCTK2IBKC";"https://ct.automizy.com/8/WCBTRHVWVFZERL2PCCFZFOZJDX3L6JPDB6IAWQCXJ3RBCXO25NMNXDFGI2MZYH5YWTPW2NYU5ZOIISQHSCZZBYFAVLCB425B";"https://ct.automizy.com/8/ALERFO5EK4OCWRMP6OXKGMI4QFK5Z7YB4ETR7N3XQKWXXIYKGSZ6RCGTYB5DGNPCPMAM7UV43PRNLITQ5JE3UW4VTLSNFTAQ"</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>14 April 2026</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/GJQBMF2JFO3G2RWAWUPEACAR2AFPWBK2VCFX57PQ5RV6L23OMRAOCN4BX2P47FQT2G4BE5JYIQ5PIYR7EA6Y5XKJQDN6NPL4";"https://ct.automizy.com/8/ZAUMMJWIO5L6HPI6HNZUNOSFGSPCE6EHW2R322ZDUSTBUMTCQWKLWDMG7FE7W2GCYVU6IWS6UHGAPT7PS4PN3PEAHGFEBZNU";"https://ct.automizy.com/8/NV3HVFUORJGAHF4GIWGMOES5BUOUD4FRT6JEJHY47F4V4DJTNE4XOGZXXNJIS4CS3IOVQI77CTFNQJTDDFBFFQTTHCWXQDZC";"https://ct.automizy.com/8/PLRD2GF2SIOGOM6MSSRQYY5STITANJCKO73HOVMHRXPHP7RJVP5DUCWVMLT4EQ6YFVCAPL76MU67R73YPMECAPVKYZXMUNOJ";"https://ct.automizy.com/8/UWYPEDLHXIQNILJJ4N4VIAY4JKINS6NRO4AXFT6NWEZRB5FR6LZ4TI622RZJNRFXWYMDY7ZODVTZUA4CQCCKT3M6OAKZ5QLR";"https://ct.automizy.com/8/365V2XXT7PAXLLP2GR2YSFVOMAT6QAYLZK3TMVX6WZAVR5HB5ATRTISHAUYOEJQLIZZE4QO7OPJHPH22YO7M3QQYZPO3GYME";"https://ct.automizy.com/8/3BAERRSXI35DJBP65IFAQACIDUL5WRH5ZS4EIABRFAC6IFJ74R7CLBA2P6NLWQG7NYTD774T57JS35256P3CBVUBNWDIYPTO";"https://ct.automizy.com/8/HX2I7EYZ6KFIWVMPADN7KSPBWC4TFVBQZEWGHBKEU2WHFB6DR3QB5BOC55QJLZ23VPLCPDHWROTHKQZRAL7SD6KIO4VZTLVP";"https://ct.automizy.com/8/2MXDQYUJ6K3NODFRNSRUW25KDBUZRI6CZL5UKZ7FUIQBDBCL5KKOX3ADT2SVQH7ZRQ5QMMCK7YEQYAR3JVG7ENKYWYHI5BDZ";"https://ct.automizy.com/8/4FTLLE7PFFKXBY6K6WNP6RF7ZVSSEDYB3DEFTOFW35FLUPTJ6QQBGTXY5LKODBCTNKFMRQJCWYSO35AWM64QA6S3DH5UD3LE"</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>13 April 2026</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/IWUCM3X2E66MKVPK7DLH3IJIRYNS5OH75N5WE7P32BRAY2MNVL67EHDAF3OXA34QJIFKE3E6MADZZG32AJNDUAJMNUD4X3YI";"https://ct.automizy.com/8/EBJAEJLPRDRI6C7XHK2ZNRWYLCKYDGBTL5WHROWYI7FXOUUOX42EKL52WSTVP2KA46JB6S7IEVQROOO2PIZFI35YQFRV5U6D";"https://ct.automizy.com/8/7Z3ET63GXY5E362U56PPYRKIXBMTKPWGUDZ74XZHIAMO5BOBFRJ2654ZTLMWVYZHTF4HDQPCTPTWKAJDMZFLVTOIGJBH7ELJ";"https://ct.automizy.com/8/PL4I7UIG4YA4PWAVGYKD5LZ63ING7ECH6N55HF5AWTFKZVM3PQUEBDRM2MABZOL5FJNQU6CL6BYOHVYTN2FQJ7WJ2LLRYWJA";"https://ct.automizy.com/8/6P6WQPBR4DCUILYE7GPOYMXY5JMHUOUWSNRLA5U3QDOXYTZPUE6ANVKM37BL37UVEYDZHPFJSBYOFNBKY2Z7UKAMHPSDZSRV";"https://ct.automizy.com/8/KDFBVPEODN5U4WIFN7K543AT4Z3KNMGYFWLEV7ULT56BO7DPIX633IMMW6EWCARFWMHMEVL7APPTFWVUELZDPNC3IAZQ3XFE";"https://ct.automizy.com/8/6HX74IGP2GDJEJ7MMAQ4XNBPZQOOIDZMQX4IHVWI55C7F25NDDEUBW3L2V775BR2GDAADEBRGG654DJ6M2DYJEWE3WWR3ZPE";"https://ct.automizy.com/8/GZ5JJSR6I577RDCC7VZBEV726FCGDBUFFGFL2XVYCXS6LBWJCJTSM3NYMLBH4AHXE7NSWAIDMBOR2I2DA6YKNSQLQUVDIQML";"https://ct.automizy.com/8/JINE2Z7VVITPFKWTKIWNF5A6ONCAENYJBC7OK5MX4WSJ3SOPSQJOVSCSNQG4ZIMPBEDGEDSWZX5H6ZIGDXQ4EQRTVXY5S5SG";"https://ct.automizy.com/8/GHWGE27PNFK5M7M45JB3VFZQSCPRSQIAOOYG5V3UZ7LP34XEY3JQUGCHTX7NHBZAPUEEAHJSL3M36M4IEFMBQFSB7H2MLL5F"</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>25 April 2026</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/B7RDFE4YJLFKKNQK2FXEW6MREVFURP7VLTTYZYLOGC3GCLUN3RHD5OOBXY6XMGU7M727GRUGDV7KEHSZAHBLEQKL3S2FMZEU";"https://ct.automizy.com/8/Q5ATLOUI32SF5YECIEFNZFRAQPEEBJ2APD5KSMI5TACIRX6ZRBWIHPKDACTSX6CLEAUL6TBBFEMTYDEBW7VFU7VQA67FTJQQ";"https://ct.automizy.com/8/D5P5G53EWL5I5FO7H6QLZ6HNEFY4DMEDIFEWDFCCKA7WUJNRMV5AAIUFMP4VBFL26Q6HX5OQORZ32M54U62PV4POOI66O4MH";"https://ct.automizy.com/8/BRATTYO4TGO7FVL36W3YPPS3FU5BTOEY24TBJXNKIZEXLUVMDSHFBY5ZC4DFKC7OZZCYETXEMPDMHDCGJEHQSRLIG7HCNNIW";"https://ct.automizy.com/8/CBQN2XIM43EON4E3V3WHVKA5Y7S2YSK6YPDFD7OPKXJT2CCKTLSKQ6UNEMHBEA6EW4IUXXGWB2YYVXRM6IEGCEAMEGKLENVW";"https://ct.automizy.com/8/BEKKOGEOWF3HHU3AHETL7NTMMJ4GNUHR4CAOS6INHVPG7UNIKGEDF2PDYGCKMXFNZMTRWA2ICE3NCRC327KYVSUD3ENEHNYB";"https://ct.automizy.com/8/5DEBV5YBT3XJOVCP3CUGRS5AZOJMQ3YYEEJZEYY2TNMEPJEJY7ETTQ5JHYRA4NE7ORE5HZQGGCU2S7XLU5GDI4MTFPUFBQNL";"https://ct.automizy.com/8/JLH45HDMF7EHMYWXU5GCLVTUILXUYDMQAHESP54X5QIMG7LHAYRH5UK5XQKE4QKWR3VJGBMW6S4KVLFYVZJU6LKZ3QQY4GKZ";"https://ct.automizy.com/8/T3426SNQ3MFZV5U6WHE2SU3U7MY7MIA2VF6ZALQ3ORU6GKPPV2A5ZZA3IM2DET72DNDJA52L46IHV4OJZJLDKYQTFUXKCRXH";"https://ct.automizy.com/8/SN56T3EVUZJSBJV72THB6ZUSVHAHFATRW4KYPORCPF6G3M6FEKHH4TOVKNCP4EIMQDEKJBG6OKLTZDQP6UTJV67ILGXMPRDY"</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>24 April 2026</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/A62GWIII2Z4FXUOY75DOVDPNCSLQ2FGLARPQ666P7LWCJCLS2EXPTBVAUIEWO5KP3T2V4PIGP55RDBJ5AIXIYBNQBSA2J3SO";"https://ct.automizy.com/8/7NNVXNKMU6A333NJH7FLYGTKXYGYQ4W6VLHXJIIB5SAERQ46RKXDDGIZ2TG6BVBZRMSYR5WLB4SA6NPLJR3J5MQEYHYQ7EZ2";"https://ct.automizy.com/8/E6DD7ZYYKJKU5EQUPCZKNS5W5LXEI67WO4SM536FE6EKJDPKCX4FTLPHNQRIQPIIOD3MDDCO4UUD4R277DOGU2ZWDXZQKHWH";"https://ct.automizy.com/8/HFPUESIB6BI3M2JBGAUI5OZHPR5D4DGEJN4SHBJJJPDQRTXEU5ZPBLU7P5ENHVFEXVUL5APQP62N2MTHTYGXQSC6K3IYMKTQ";"https://ct.automizy.com/8/MDANCFOV7QIOHD25YELJJDL6FPE3F4YFW4RPGF7LLP4U5VHU3LUGD2MUXURN5K2E2QLZ5FORD3SX4TLLYOAGSLOWKYMRIVAQ";"https://ct.automizy.com/8/F6CYNAXHPIMNBOLBEI5VNPGB7U76HHSPADLPR3SGLKQPXDH4DBOEZL3QMCYX2E2P7R3NHZBVDKUKEQBP7R2WX4FKAJRM6IV3";"https://ct.automizy.com/8/EMTL6WE4VMSBJZT4AGECLPYBUBQLD3G23E76NJBZTKZIVUHZMHQ5O7BW6UQWCXHST3AJVYC45FQNEIWEEHNUBC3VPUCW6IMV";"https://ct.automizy.com/8/U4ABE5RBCIIKGY3HTJL3BK6SFFBYDINAXAML7ZGRCNVYI3TFAOGGOEQQJ4J6ITZIGEOUJVB3UPHZFH2LS44D5PJNIHDHW2LE";"https://ct.automizy.com/8/QPOJP6OGBFPVJIQU344QX4BNQAINJLBG7P4GV6GBX6OFOPE3CX5RYG5CIYUNFVTHZTPAVNVIARERIIO5QEEG3MSHZHDRMHLT";"https://ct.automizy.com/8/TIPBDEOMXJEPHPMIPSKD22HHDSPDCG2IN6I26AO5MDNXZFD6ALE3WRWVHJPOUESPKXPC4SNZPOEQQBBCFXUKOC7SNUNCXOMD"</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>23 April 2026</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/DLLTYDTTRNXROAARDNYSQPMFADHBPCQLL5RFIMXWIDEOE2R72H3MCUSMXCSALKTEYJGCBQMD3F3BZDV7U22TRDZRWRHVPLPD";"https://ct.automizy.com/8/6USDETFEMV645L5TJCLRENPQGTSZE46EX7WXJQZDHKGKAOCDWHPVNC6C7WEFURDVN74HRHLDYJCGBAXAGKDK2Q4BNFZILNNI";"https://ct.automizy.com/8/5Z7SGCBEXF722FX5ACAHVAM7CJAQH7ZLEWQEUGULWWGGY7HHGBJECEUYXUO4ZE76EDXZ7EIE2N47ODQQ7PBXLHLF3AITBWES";"https://ct.automizy.com/8/YRZJ75GHPWEHPDWFF62AO3MUOEORGE4KTN5WIYT6MJGRAQ3FDJZVWOJBCZKGQ23JF5IDY6WFXOXUHMVT5KL7SKZTB3OP2NLE";"https://ct.automizy.com/8/XNXGMEEDX2UUSIYD7ZNOBKWX3YUNZC4ZL2NWFB542DKSBN6L473MJZE35I52RIMW3YHQ2IPFTW3N3Z25GJM32CWJ727VSOYE";"https://ct.automizy.com/8/KH4BQMKJX3CEYYHYWLJZUSD4ERRQ5OSIU2URKTYLQ454DEOQDM4GRGD6BEOIJQGY2EPKJSBZBBJGATB2MJTZQUGYPFO6RVAU";"https://ct.automizy.com/8/HQJTGJHY2EKDDK4FZOWKXZGESO56QPAYTVINTFJZC64AXIURKP7WUUDIX55NVN3XMKEFUULFQWGTCQ4HYTQQ52DQ5BY2S75E";"https://ct.automizy.com/8/ZKAYC3U6TEF6IVX3DRXEJJEFQTTQTH5I6B3CKLYUCVFJJSB6DROJOQLP7BRLJWWUYDIN4XXOLBWIMJQCXI7GHSFCDKZMOILL";"https://ct.automizy.com/8/YE6G6KD2JB6XY4BQCJKCL3UOIZ6WB72J6347VJZ5B646OZXS3EP5CR5ZSYZFQKHBH2NLZXV2TL2A5HSKVKV4IMYATORBQDYV";"https://ct.automizy.com/8/O32C6RYLRFBKW3Y4XK3MCMHRVF5MHQONTLBREJLM4MDMOQY5ERCMDNREP44QN5BPZQV4PF3FQDQKT2LZBGPPV43VE57MU7RS"</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>22 April 2026</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/ZAWE6MS4V5KGRASLRRVC3A6UT6PY64S5GRDTUTHUVD2L4NCTJZ5QVSPFTN5UFLYQ7K7VWYDE4KU2HIRUH5IWB5DO2ZWRZ6L4";"https://ct.automizy.com/8/P6AGP2HGFWSIR7TLQQUUGB7KT3GGKGOGKCRA6TT5WAD62JJIPQX5SGQWFNJITKOG2RWHOUQ6VF2FB45TXPEGBSLMFVS4BHCT";"https://ct.automizy.com/8/4UR23XD3ZHP5NY3F2W4XZJUX2EUHNPSH5TPAD3KWTSJVAXFOSTZ2OH4UO4KCGN3GD6KQI6S343WUSYUBWDYXYDV7A5UBXLYK";"https://ct.automizy.com/8/PI4B6D7OPH4ENBXQFBS2TOT7MOVEUNAMSG5CTE57GDBPJLHAL43OBQQKTFFO4LQK7LTHA5UPNXWDBLU57ODGRWNRICM6Z2G5";"https://ct.automizy.com/8/VVL7G5FIDKND3FZ3LZ65RXIZV3DAZX62XEDE6NVG2P2FNA3Z7FOLE642D7P2WFMREGUWVK32ROFHNLFBYTYOJ5LOKRYQETSI";"https://ct.automizy.com/8/7E2P5HUPPF6TSL5H2XL3IUROY322RN46WQVHD37J3KQIN5YWXLUZQ7OIBZKZHNSDP3Y54JAZUM6NGNTH5EM4JAKJAPYV53RO";"https://ct.automizy.com/8/MFQP2FHHNSRPCC5JOKUMQLEZQAZE6LFJKPNUQDENFQGZD7SS23UIH76FQELEKG2EQLKF33KFUMKZ4F6G7CUJRH5QVSOQCVPY";"https://ct.automizy.com/8/IYGRUILQIIW2KXWK4S3OM3RJTI2GPHCFZIGYA26I3JSMM5WNOBWKEUKGTBL3KSRWPNI7UBFKDPLKTOPUJWB4LH3R7VGST63T";"https://ct.automizy.com/8/SW4KFZAGWSNFU5H7WTYQXUMQ3NZH2K7XNTXFMTHSRTJIXHYF55UO6YXJYLD4IKG7IO6FRYDWQSUHVSRXDMAX3CA3SCWX4PJP";"https://ct.automizy.com/8/D3SPLQX7VLYWFGAYIYKJ7KK2DE2IQRMTL3FUGIUUUBCXPLKV3OBVFSY2JMRLCIFSPYDAQ75UUHFGGKE3O6B7XNDPMNZKDKQO"</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>21 April 2026</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/GIFKUWHNEUCCL6MHCLOZU5RWHATZQIGF5SIOJ3NAS3NB5NIQWEYAVCM27GJHDIWYBMTMR72HZU54S7XTTUNW53INXCOT5ANS";"https://ct.automizy.com/8/IGAERI5WV64BPJGULBYZAUR7Y7ZKSFCIQOVWGWQNTY5OCQD4LM344NJ7QG2SCV5X2YXSWLREUN3XZKPUC6YEIN5GENNPGREB";"https://ct.automizy.com/8/XLTMB3MSS7J75RNR2SIA3C7RXK55MWRMKERLF76VAMBGEUFFGQWHPZKDLYCB76HRPXO4F75VGXKESNHAI5XLX6TH6TFR6ZME";"https://ct.automizy.com/8/DWIFEP3BXWXCM7QTBTM7FNNILGG2L2VWATF5QSIWRCXV25PEKE6X53OKQ2HL4EUOJ2ZQIH5H3NQMLUZGMNDQHJIQSUMTGJ42";"https://ct.automizy.com/8/44DOTD67RSQASJIXZTS3CLZDBJGNYAXTWMFIM3AVG4NFDIU7QUG2JC3FHDT2KTNOAAITGF3UU6XOOLX5M32D2IL4GKCQNDBQ";"https://ct.automizy.com/8/6EC25CJYARGU2HK3SCZQNNXBIUCYMVOBD6OH3CXEUKVVKHYR4GX2YOS4TZC5Y2Q5KAI26F6FDBHQUOMLURK2DHFFJ2N3TTSU";"https://ct.automizy.com/8/N7U3IJSVVB2FIAVRXSVDUMXBQNO4WSN4KSX5JWGBLOULJ4KCV55FWPORUS67C3TSAQOJVABM6HVZ4RHQQUHXWHBCYKVBEKZ6";"https://ct.automizy.com/8/AZCIAWEWYUZ2R7MZSG6VY6AAJI64RUJ6LBD3WM3LVZLE26TJ23WKAB5RW5XYLOLO6H5FCDYEZ5KSOKISZ4HVFFQS2KVISE6K";"https://ct.automizy.com/8/73POXQ3VLBOLUV44YK2JDBZ4CZLEJWNSBJE4VLEOSB7OXNSCX23U7KGRCW2RPEENGOZ6P5CYXU6FPOLR5QNMPBNUNNOMHOYT";"https://ct.automizy.com/8/URK6KWVIY3RZDCNJTC6RKKNQVWCZ3Q5TKHJDS3I5OKTXBSOY25754URPVPYYZQXSSLBRVFAAZBY5UPEZKCSK3TPLL6OTMH57"</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/SAF7GUAX7H6JTN7EIMKTCA6R5T5POT2HF6G6LKGEIXFCKEAUEYGYHX4PQN3BOJP5ISCMBK4PXS4YBH2SGNFPJPQ7IXQ7KM7N";"https://ct.automizy.com/8/EZZTVXYOHOO7VPGEQAK47VM5Q5AHYQVFIJQE3WHCBCVW7FXPKHAFCSWB7AWSNSKAG5ZHUDGG3JH74XQPG62XVM4Z25YJF5WO";"https://ct.automizy.com/8/SZFW23ZPLY5U6LORBBZXZ7UGE2GGONQELVJZ2F6ZQPRF265OPLCL2G5FBPNIWT44FJ3BFNS6NSFOAQ6VNOR5ZMUKPB7LLMRJ";"https://ct.automizy.com/8/WOS7RGTUFNZ6RMXURTVWEDDXIGAAG4LC6LZR77SUTAMBXPQUTI7ADPB7NLJAZCZ6AEMNETKZKQOMMWJSS5PWO5GPE3HOEQIO";"https://ct.automizy.com/8/IJACZKZWBGASDBJYCW4HVMJ26J6TQTYU3EFR2TK7DMP4UMOI6QAP4YWBACQM5BIWBC2CRBA3Z76JSGSAUPDMBUYQ5ZXIP2PW";"https://ct.automizy.com/8/K4T2JEHWX437OB4TAUEMTYAOPHOOOKF3F7AZASFNYHDFDOPA3YQPIPG5RWR4UM3455F3U5TYNILT6RACXVCZKOCJ4BQCAB3Z";"https://ct.automizy.com/8/ZX7NZP7NIJHZFOJ4AXYMDL3ZEA4VPQCKTIWB2ACGGDOGALXQSN7LNJYAIUEY3I7KF5EZO4QTMBBMNBY5XZCQSIANDCCOJ3IP";"https://ct.automizy.com/8/4ODGKFXGOWKGCQFBVPAVCPICYG3JFSET7QWNVSIVEEWWMEQT7GWIOPVTY2M2GP6MEIGQTWAV2AO3OMOIHQ36HY6YGEHNVGIQ";"https://ct.automizy.com/8/4CX4FSD4BQK5CVWZRGOPABG7UQ6XYX6OWUZOE6ACSR23LW4MFSLFNH3NKQ4WI7KN626EHPUAEQE4QNFTSRV4POH4ELLNOKO4";"https://ct.automizy.com/8/JO7R6SMPNIQFL24KWPRZEH4J3KAZC5J3QWMIKIUJHLG4UDUBIX5KER7KO6M4JZKPAIWO53RLHPQHJYUO4C4COH6LBDXKJLBD"</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>19 April 2026</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/5OWXDCVCO2XFXEV7VIUSCGACMJHT245TBRKLIXSPAYS7MA5WPK6RGC2L2KP37DLS4BS2ATX32MS4IQSLPUT2MPX24MUKH4D4";"https://ct.automizy.com/8/R6MTH3AUK4DNJRL422T77DU4ZQLFTD7STDDYXIYKZXKJU42NT6RHDSBN4TYOULINU5DP5YMOIDIRPMMDBZJG6MJSPAAXA3AA";"https://ct.automizy.com/8/OGKDGA6LWP7CRDMRJWB57IVT2GUI2Y63RSRCHR56WNTXC6QUMWDGO3FDOUEZQE6TA5K4JBHJGFVFKT2W2GPF3AX4GOOWZPPG";"https://ct.automizy.com/8/MIFRCTMQWNIVD2O25LH57XD75WSA6A7UUS6AUJUSQ53C35ZQKZCTQ65WLHR5YVTYBXHJBAHHXCYLDCBE6G4ESE7ENGQOWBAG";"https://ct.automizy.com/8/7JVB5JCYRNQUNNOIZOACXMOJHIEMTEQQTBKNTUPAEZZWQ6SLG2AR6GV4R7WPETDRPBG3AHWCEBYKYJLN3JFRCZJ7ERJDUAD6";"https://ct.automizy.com/8/M3A3XKE5OCWNOBKPTTS56RSV3MQG5HGTAP4DVO3IPLARXCWXS2KQWS4EBMX6THB2LHO3MI63MGTPUV7J2BGIPTSSWQV4QWYQ";"https://ct.automizy.com/8/DXGJU7WV6SYOUJOTDNU2EH6CXWBKHRB6DLO6URS54FBC7PLL4SUADYABFDSPRRHBPSKMLH6RZKCD5EV35I6H6AGIVHKN7RPN";"https://ct.automizy.com/8/HV32TMVXOII525W672W7R6TLS5MYUK6EQBVCAHORGSTXWHZPKMWU2M7HIXMCAYSNSN3OOXLP3RACTM2PP24TAWDNJ4JEFVUE";"https://ct.automizy.com/8/U33JL22IAZS2T7AXPMBYRWLHV2A7P6VN6KOKBRTXYSUMGCPTA4DPGU7PQF6HQKYY3R6MWAQRACKL6VF7PI7RILUWENFSKYD3";"https://ct.automizy.com/8/DC3ADO4A4VHP2IIAHWO2X2PKCSCUH2YU45QTZ435S4BH7RVLHYF4EKYPL75E27OJMVLHHWPYTW7EXQQUJN3ZHZEZSDLX73D7"</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>18 April 2026</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/X2YWROWNMABF7XADB6RX6CSUNEPPIBEQUS436XQDXR4HNPE27K7PJUENPNJAJINWCDYNRVSMLWG3JQGOSERK6NQS5RD4TE3I";"https://ct.automizy.com/8/NDHSJMHIX6C3NVJGZ5SNETJMAGDX5RXWAAVEVG33F2F5CDYS7YE5WBQM6ADG3QHSVVXA6XHOE2NIPTGWNESKXUZFORPPOBI6";"https://ct.automizy.com/8/RMSYXUUSIYDXFJJPHGWF7N5IUPW6MHC3ZLTU7KLYZMO3VLTUB7BHBT7B42EK624AGPX4EHKCVU5UM7FSO2Z53DVPRBYOWWM6";"https://ct.automizy.com/8/WTWTQDBUBRYMZKNV6OGLPW3XCZASBLQARCJIUIQLBFV2YDRLOAGOPBN4KYCJS6TZRWOEQK3LLF64IYXNIBH3J6F5CYZBSEWE";"https://ct.automizy.com/8/XWFQTC2C2SB7AFTXJM6PD5WEUVDIMBF7DN55KT47Z2NUORJWP3EOZJTSMYJGOVV6UK5NOVIH3UKKFAD7PUNWHKJF5Y5KZFHR";"https://ct.automizy.com/8/SC46KIFANQF2SPGBUWBN3ZHX4XIZACY6XSOZ2JQJ43IOSY7M3TIXZT4BAL73C6HGEWJJUCG5UMCREABZAHV4HDMGWVO7CDLM";"https://ct.automizy.com/8/6YZ5Z4W2K76IPBAT3QKMWXQITVGQGNEVWZTQQVQBKIKXNYWFUNT4Z5ZKMPZFGMX7KXVGYN7OVWNS23OUQKAJJFGYCH6LIUZR";"https://ct.automizy.com/8/BLJLPTSQAFWEOXPJXMJ6CIHZAE2SLTD3YDKJ5E5RHTBN77Z73WLOFZIQSBMGYLOAGSLA2ZCOOAW2CKTV4VFCUE5INOR2YJGC";"https://ct.automizy.com/8/JGM54MFX3MXX5LOPTE2J4KRZUEKPNAX2AMXZQZ75HSDFNP6RD2FTU3L4AR6SKVSBEXAEKWLVM3GSSMJ72KXK4A4HBDI4CEBV";"https://ct.automizy.com/8/SLMPQA4CRWIPUUQ2CZJ2VTLONOVRHCBP7FZ3ZVMXMGBFWAURVYWKOEBKPVC6IAO7UTYFVF5DXGUEWQLQDPU25ERKC4TV7RQQ"</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>17 April 2026</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/GY3O7DARAOM27EKUJC3ONE6M3B4ZZSJVR6LZ64BOR2Z3Q2RR6H4R3HAEVBHZY7RJKHR3FXN776EKWBPQYOUY2SWKGCEECTUS";"https://ct.automizy.com/8/BJHLXIMDINPKPY2UA3ASOMPRXO3CXVMOTSV3FF662AQ5JQKUGBRFFDMOVDPGAAI55RCOXD5KXDTDBUTCF4NPHDCFQFXC657M";"https://ct.automizy.com/8/Q52IVQNBEJC3SZCUK5ODCB2DYSTW4CZERWKGXGQTKJMRXTIQSJYL5LMKBMRM6TXUILYXGZGGHMQOA3QV4XNNCMCHYCURYAV7";"https://ct.automizy.com/8/PMPWTAFLJLR2QIWZ7NUDGEGUI2RFH5ZVC5CCRZRCDPDKKWOTDLHMWUKBUQLAWS5VZWTUUUFMQSYO6I2U3PVCUOJJZPEYLC3P";"https://ct.automizy.com/8/GOOGOFHZH5ZYVLX4ESLWMHF5CRLOQKZJXX5IQ52AMDDBRLECPLTL2E44WAJCA5M7PGI7LWZQJHDAHC43EF3VYRHY4WSAERMU";"https://ct.automizy.com/8/UCFQ4FYVN2INWRNANY5KNQYZA2PDDOXLZD4HFPBSSGGIJRDFV4ZUOSQBRHBEGMJZZORFXVY3PEVECG6Q5TU64COR6PX33LXQ";"https://ct.automizy.com/8/4A33KXTQ7VHZKDRD5HRUJFLN3QA3SKYSQANOXNB55BFIT7GR3INBCGPIUREN4OLVOPME4WODUPTJS2DINE2MHUOTNCNVJVTS";"https://ct.automizy.com/8/GOWMB6UXPBN73MRLAD4X4QKZJFA2STGAMAYQEK6WHTKTWQWBQY2VAWU4HBGYSA6FPCRNATFD7Z4VCLGFNSN2PNIOB3VB3MFY";"https://ct.automizy.com/8/OLM5CPMQ3NHRHAW47Y4UCHU3FBMS3VBY6WOP3EMMNN4DLQKEUQ6WVJ36OU7T3NMAQE462XG6DO5MM3HQ4CDU33SM6OG7SRSF";"https://ct.automizy.com/8/A44UPDNK64AHVK6XKTOMBDLA2CLTDH7D3YOSZI7TQDART4XIMSWTG34KBTEWQGLBDKO2ROYKMZLLHAWR2J4IPCYSN4JZWFEV"</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>16 April 2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/ANFHRK7Z23TSASPYAARHQC644DJYB45PDGII3UBGZXHSY7OSVHXTQPGYP5BXAGI4U7ZURQGAEPVBD275UBFOQDMBIBWVSZYL";"https://ct.automizy.com/8/VU6RABOGCFBHXMMAIZ67RB55QHTW6JKYDM7ZI5S5LTDTIHSLLBV2FKRIPISBPZ3RWNTQXO5GVOZ2BP7CAINB2EYPRJZS6HFU";"https://ct.automizy.com/8/4BCIF6LTO325YUMD6HGZQXY3FR2RIU4UBKRCV5MKDP2DRLQSBRSETDNW2DKOPF5L5UMCCPKL2H5LYN3LVUCNQ3L2UKPHXBMR";"https://ct.automizy.com/8/GGUJOFZLTZNHAHYC2UHMJAGZDQLI5KNAFSRG57O2GV2L7P2BDKCQKV2BIDRAHH7JFMN6CWV6X5PX7LDIJMTZKQ3QOUT2FXB7";"https://ct.automizy.com/8/JWM76H42Y36JER7QSOUJOFGZAJ2SOYWMPNFTEPYHWXM5Q5ITZAGDJ4FU273ZNBIGBWXBS3MC732WRQ7SUPWZ34Q7OKKFPZSC";"https://ct.automizy.com/8/62TQEXY4CM2BYHBXB3TAE4IK7FWLM353TS32HSRUR2FV47CF3BJVCFGFIMBVLM5NU5DHFE7FBYDIV77HFKL7W2UUD6V5D7V2";"https://ct.automizy.com/8/HVFTTGWCIVIUDEZH25D7KKX3F42VOT56U2V7QGH5RIXQLY6DP52S4NRRG4BVZCJNUM22IZ2RW7UNUECLUT542YJG3CUOBJ6S";"https://ct.automizy.com/8/XPWVVSPRFGCENJ4UET4LUSK6VCJG72K7OOLIGQ7HSMXVSRRBQL25HCT5UEBRVKMBVQHMYUZVCZRRSDMKPOTXCRZY7XSZLQVI";"https://ct.automizy.com/8/S7MCDFSDJKX4NHNNSSZG5F47QYE4I2LTK4B5Z3ELNXBB5HLJ6RYSA7M55ZKQLVJCIP6B7Q2IQDQGYVMPFSHB6JPFQ5JNXITZ";"https://ct.automizy.com/8/57SY5ANLZKLHBKLZHVGMDF4EEX2USIHMKQMYMTNDRX46ABXCDICAEIB3HPHYD2VVUEBFSNLZWANOMSLDOP2E54GVUUQE6AEM"</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/ALERFO5EK4OCWRMP6OXKGMI4QFK5Z7YB4ETR7N3XQKWXXIYKGSZ6RCGTYB5DGNPCPMAM7UV43PRNLITQ5JE3UW4VTLSNFTAQ";"https://ct.automizy.com/8/WCBTRHVWVFZERL2PCCFZFOZJDX3L6JPDB6IAWQCXJ3RBCXO25NMNXDFGI2MZYH5YWTPW2NYU5ZOIISQHSCZZBYFAVLCB425B";"https://ct.automizy.com/8/FRC5RZCQ7KCMY6RSPAJXDLOUPIUBFUPNBIVXTI5GIZZOUTA7LVD6ACF6GTJ2X6NEDZZWV43GZMQ3E3IXAQAWTXURCTK2IBKC";"https://ct.automizy.com/8/YLB2Z27GX5OTTMHK4W3WXVC3RWTMGLP55IM545QSJA42TE227OF4LKBMKJQRXUHJ37ETHJA5WAZ6P6VBPM7NTJHIJGPRNPSK";"https://ct.automizy.com/8/LXHAOLQQM7GNRDEWRH3RPEAVQHWWCQ3HN2WDONRL6HROY74DXOLAVRW4NHMC4FTFTGDI7YZM57DKK4ADHHLY7W3JZO5446M3";"https://ct.automizy.com/8/BOQACJTR6777NE6DUAKU37BIOZACR3SD2O3443THLGKBLK34GCBWXT7KNTNMWSGMMPEC62OETWFRSXVFHNNQ2TP3S55L5F2Z";"https://ct.automizy.com/8/3INB2KXF6WPVOQNFKWT7KGUIO6OV7UO4KVGUT3EGYHN7BO7RJYCTTBFOOMO6PNIRLIVRL2UA7KRLZHF67MUPR23672WMEFOR";"https://ct.automizy.com/8/BB6ZED7FEMPVLMPWK7IUVFXWCLUUN3JALKY4M2NCCJWHQ2D6DROCINTYWI5WMWX4REHATKTV42GCTXZLLYUWMO2WLN7E4ZOZ";"https://ct.automizy.com/8/6GJLTSARNNRQPECPC5VRY3CQX7UL3CENUGC5MSFE2JQZPH5CPBM56SABLILUI623KYYJTQQV6IY3UGP33OBOZSLJI26ZOC4I";"https://ct.automizy.com/8/4QXPPWLZXOG4OABOYLUQE5R5GW47F6WTMFU4CNW2IQPIJYY3Y3DZ5OVOL27QPQLIHRC2DU7R727R2EVRFSMZC6UNUV76U3VM"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14 April 2026</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/UWYPEDLHXIQNILJJ4N4VIAY4JKINS6NRO4AXFT6NWEZRB5FR6LZ4TI622RZJNRFXWYMDY7ZODVTZUA4CQCCKT3M6OAKZ5QLR";"https://ct.automizy.com/8/GJQBMF2JFO3G2RWAWUPEACAR2AFPWBK2VCFX57PQ5RV6L23OMRAOCN4BX2P47FQT2G4BE5JYIQ5PIYR7EA6Y5XKJQDN6NPL4";"https://ct.automizy.com/8/365V2XXT7PAXLLP2GR2YSFVOMAT6QAYLZK3TMVX6WZAVR5HB5ATRTISHAUYOEJQLIZZE4QO7OPJHPH22YO7M3QQYZPO3GYME";"https://ct.automizy.com/8/3BAERRSXI35DJBP65IFAQACIDUL5WRH5ZS4EIABRFAC6IFJ74R7CLBA2P6NLWQG7NYTD774T57JS35256P3CBVUBNWDIYPTO";"https://ct.automizy.com/8/2MXDQYUJ6K3NODFRNSRUW25KDBUZRI6CZL5UKZ7FUIQBDBCL5KKOX3ADT2SVQH7ZRQ5QMMCK7YEQYAR3JVG7ENKYWYHI5BDZ";"https://ct.automizy.com/8/NV3HVFUORJGAHF4GIWGMOES5BUOUD4FRT6JEJHY47F4V4DJTNE4XOGZXXNJIS4CS3IOVQI77CTFNQJTDDFBFFQTTHCWXQDZC";"https://ct.automizy.com/8/PLRD2GF2SIOGOM6MSSRQYY5STITANJCKO73HOVMHRXPHP7RJVP5DUCWVMLT4EQ6YFVCAPL76MU67R73YPMECAPVKYZXMUNOJ";"https://ct.automizy.com/8/ZAUMMJWIO5L6HPI6HNZUNOSFGSPCE6EHW2R322ZDUSTBUMTCQWKLWDMG7FE7W2GCYVU6IWS6UHGAPT7PS4PN3PEAHGFEBZNU";"https://ct.automizy.com/8/4FTLLE7PFFKXBY6K6WNP6RF7ZVSSEDYB3DEFTOFW35FLUPTJ6QQBGTXY5LKODBCTNKFMRQJCWYSO35AWM64QA6S3DH5UD3LE";"https://ct.automizy.com/8/HX2I7EYZ6KFIWVMPADN7KSPBWC4TFVBQZEWGHBKEU2WHFB6DR3QB5BOC55QJLZ23VPLCPDHWROTHKQZRAL7SD6KIO4VZTLVP"</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>13 April 2026</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/6HX74IGP2GDJEJ7MMAQ4XNBPZQOOIDZMQX4IHVWI55C7F25NDDEUBW3L2V775BR2GDAADEBRGG654DJ6M2DYJEWE3WWR3ZPE";"https://ct.automizy.com/8/EBJAEJLPRDRI6C7XHK2ZNRWYLCKYDGBTL5WHROWYI7FXOUUOX42EKL52WSTVP2KA46JB6S7IEVQROOO2PIZFI35YQFRV5U6D";"https://ct.automizy.com/8/JINE2Z7VVITPFKWTKIWNF5A6ONCAENYJBC7OK5MX4WSJ3SOPSQJOVSCSNQG4ZIMPBEDGEDSWZX5H6ZIGDXQ4EQRTVXY5S5SG";"https://ct.automizy.com/8/6P6WQPBR4DCUILYE7GPOYMXY5JMHUOUWSNRLA5U3QDOXYTZPUE6ANVKM37BL37UVEYDZHPFJSBYOFNBKY2Z7UKAMHPSDZSRV";"https://ct.automizy.com/8/PL4I7UIG4YA4PWAVGYKD5LZ63ING7ECH6N55HF5AWTFKZVM3PQUEBDRM2MABZOL5FJNQU6CL6BYOHVYTN2FQJ7WJ2LLRYWJA";"https://ct.automizy.com/8/7Z3ET63GXY5E362U56PPYRKIXBMTKPWGUDZ74XZHIAMO5BOBFRJ2654ZTLMWVYZHTF4HDQPCTPTWKAJDMZFLVTOIGJBH7ELJ";"https://ct.automizy.com/8/GHWGE27PNFK5M7M45JB3VFZQSCPRSQIAOOYG5V3UZ7LP34XEY3JQUGCHTX7NHBZAPUEEAHJSL3M36M4IEFMBQFSB7H2MLL5F";"https://ct.automizy.com/8/IWUCM3X2E66MKVPK7DLH3IJIRYNS5OH75N5WE7P32BRAY2MNVL67EHDAF3OXA34QJIFKE3E6MADZZG32AJNDUAJMNUD4X3YI";"https://ct.automizy.com/8/GZ5JJSR6I577RDCC7VZBEV726FCGDBUFFGFL2XVYCXS6LBWJCJTSM3NYMLBH4AHXE7NSWAIDMBOR2I2DA6YKNSQLQUVDIQML";"https://ct.automizy.com/8/KDFBVPEODN5U4WIFN7K543AT4Z3KNMGYFWLEV7ULT56BO7DPIX633IMMW6EWCARFWMHMEVL7APPTFWVUELZDPNC3IAZQ3XFE"</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>29.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/2ALX7IAPODFZI6FSPML4GU3RYKRGYGTGYPWQQYY7KRLPXXSN7HIF63DYRXYW2TDOPERQXB7F3WM4ZM6WG5SCMXOMJX6O6MD6";"https://ct.automizy.com/8/LU7HYPPBGDN3WFDZCESLSH23K7P2GOGGQTBJ3VKYNTY6STYZ5BTGLPZXVL3NJW6HYJIUOXBSFVTYN6W5HAVYVXFP3WAD6U46";"https://ct.automizy.com/8/JZ7GU4I52ZZSYT2ITF2FQIDBIA36FF37YU35ZJMVGZT6HT4HAIQGWYGJWBTEP7ROP3GMOIWXWE37L6TKX4SXQE7ZCMPGZZ2L";"https://ct.automizy.com/8/JP6UNNT6RV2FHPOZH2BOIKJQQQFIYN4JARGZJ7OZ7KIPVXUSC66BN553KJ7WSOSS6DTNXSRR7EJRYP6QYID3IDFPVMUORBIG";"https://ct.automizy.com/8/3DSXIPDAXI6WFQ7XP2XHAPOJFJZWJLJZF33GBOXNNSB4EJ2AJOUAICBZVQ2RJBP3AU3X7QFRT42BAMR6A3VPI3ZU2H6P6E3Q";"https://ct.automizy.com/8/HHYZV7YOLBKR4UXAX4NLPVIXA326SF4UNKVXIOLOV3QFJD3SIIBP52LIKJHP4NHI5DRCU74Z25LPO6PGCAHJS3NDHZNRUSNL";"https://ct.automizy.com/8/R6NXLX6CGC3YSRNJYOPQA66FIEIOD7CEVSQWHM2EBO55PI3DU7XQFDMER2JRJHPDKCQACCYEC4DOROWM2WXHTSNRPFREB5QT";"https://ct.automizy.com/8/7YFM5MZGL6DSNGDXC4TUBPXMEBCJRSUXGM4BMSUBFIQIK3E6CEQSODAUOUBVZDFRJ3TG5LM3PX2TTDOQNBN7JWOSZESNWYZW";"https://ct.automizy.com/8/2B5DRLJT34O52G2VSSTSXJITDBRH7OYJULUCN2LKBC5EZTGV2APYXSKFL6YBUOWTMSLF2XOBQBME6K72R35UKU6B5CMBSECW"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>28.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/2MAAQCLPPGVNGPGSJQTEJTGLUDNN3GK27TD67IIX6OYNHPWM5AE35CK3TIOUD6FPK7ONVRUAELM37Z5ZE47WH2PFL7GTOH3Y";"https://ct.automizy.com/8/GAKOJ5QI56E7VWSOIV7CEWALVR7FHAQWQUKXXH6VXSHCOFVROP2AEHDRFEHN6HNDK6ZCTG23M4NDRVJ4W6UDUCLH3LAEMMP4";"https://ct.automizy.com/8/AYI5DWYRFNJIZM3QGUGWPHDNKFBH7PCSXADPUC2FS2LB23VUHXHJQM2GZYMBOCUGE6LVDPM5SFHOS2RYOYNAIX4ZJEO43Q35";"https://ct.automizy.com/8/MZTXTNLNAFYXHXZBHMDQQGAO5RJAOXGC236HUOIMQSTTUKP2HWUTXD7YFWFT6SBCO2ZQOKYY2UX6A4HNABQTCPP3EXCYQLHR";"https://ct.automizy.com/8/5W3NGAW6BWBE72YQAO6OQVTGGFHRCOORDK4X52GEOJ4N55EOHTPMEQVRBIY3YNJM7VYOVAR65KSXI26COG6X3NMDTARJHMDB";"https://ct.automizy.com/8/L2QGZXRNYRKLRTWYOQREXF32TLGPU2IQO6E3JDTJODNC2FXMZDBESYC7CNSWB72GTM5SNRVUBMR2R4LBJHV7JMUYIMYQ5N2I";"https://ct.automizy.com/8/XPC7NZROUG26VWMDGHJHMUCNIRLDXKI73TYTQJUBAHIGY5LGG574RA6DL6A3V2PE2TBPNR2D2BNGI76AYEQEXM32SVRFQMMR";"https://ct.automizy.com/8/OXWRCZGEUHL7P6IFBRENW6KONVXATJSPSDKCCBUQ4MCAAQAC6MJKMQLLE2VIRQ3APTXEMF7ZXB3M4DYCTT3ZK652HNY3X6EV";"https://ct.automizy.com/8/QSK6LZDWFQEU4RWRSQU4S56BKWYSD75XM6MMVNQ75XR4B3VDZTNTHLK5LKLELXOJ27RTOSUSRNT3I47E6P7JAY2QMAHXKX2X"</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>27.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/V6CHS4ZLXDEGVXSY7SWO3REIWZI4LSSGTS2AJ3742YFBMVXNG6V3FSM4C2BAXTPEYIRJU67JELTDOCBRUU5ZJ2OGSAPXMXXU";"https://ct.automizy.com/8/S6IT5LRJGWDFU5JEBV2OYENHGALQGFSYQIVR4S2HU55ZEDOBS2WN6OBGUY74TZA5MVYOQRIR4YPEB6EG4FUQMUG5KPWPYKWJ";"https://ct.automizy.com/8/6XR6I4LHR5HPEQVKBONCYIAPEE54RQDK2W5WD5HST4ZS54QN5HB2YXBAVCP2TF5XBVWYTKJQ7JB5NDE2CEKQSDPQPUE7KQRM";"https://ct.automizy.com/8/53YD57DB6JLU3CTAWQIW5UEFCGALAJMX66LA6G4SVFJXMCSCP34WW5EAE4FS4XPGE2EJ7PUPKAKOJER2UFLKZDNL2EL3VAMN";"https://ct.automizy.com/8/NXLUSN34SLOBQIBZBUHCZXIE4DVXE4ZYDLGEPPQR7WOKZTHKLTQSU747ORFQDPIJFR6WP2DEFESE3JE4DO63MDOJPPDNLOUF";"https://ct.automizy.com/8/7FNA25MITIQCQGJNWRYICMCS4JAUJAMBPYEW3DJEXUNSI72Q3V5SN47B4VRWMNHIOWXFWBOVQIOEQBGX3K6ZHWDVTQOESHYS";"https://ct.automizy.com/8/LUV5IQCIH3VDYH4CZE4KIXKROJ6GLZ3TQQCKV6Y4J3CDOUCNEN7ZAA3SVYIAW57MWJ54RWLFGJ7QTH2XPUZSHI4ICS4GCHNF";"https://ct.automizy.com/8/4J4B5XQWSVWGGF25QIBJBOBNYJCAUROPDFLGZAR6AMW4T2ZQWTRLHUVYKHIUUELQ3M6YAFX55TRGFHQFZ2ZR7ILCQDJCAQXP";"https://ct.automizy.com/8/6BVKYZX3Z36EVRF4LJMPTPAOYOZEIEQVZU4HOITJBMX6WFYCJZLOKE2UYDFDVRBH5AT6J5OVBYXOMJY2M3JXKBTKUFHJOJV5"</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>26.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/FYDKLBV3K6RB6P7FUQDFGRQRMZI6B6743ZV2OADWOFIXVFY6M6WENVYI5BSWELQKI6IRDHQHIFLKD5I3PWAFXPO2OOL2VLXK";"https://ct.automizy.com/8/Z7OLZLWO5B7SNK6CC2YSMV2XX2PG2P4X33OZAW7ZMGGZIYXWKSJIAPU3JSIJ3H6MOKXKVJJT46TAIXCDC2WVPN4HLO4HKE3E";"https://ct.automizy.com/8/RR7KIOYXTLTK6DN4VEFUG3WGEIABL3FNKTFCRFG3TYBOKFDIAS4MT2YPGSIVYJKAYM53VOGMVVBDGKCNYKMPG4KYB6T4OLI5";"https://ct.automizy.com/8/DTEFSI2MGE7ZB7ZFCCGLMX3IAFP6GPDWQVHZ3A7XCA6H53FXTFAZVFFGBBLLYJSBB4GIVQWSESB2FKJRZPLM7RA6PMTBRQRS";"https://ct.automizy.com/8/R2NU4PRHFNF5D4NDXMWTVNU5VMCXJEWZMSWFJWLQUBSLZW3GUD45FH5XMHXSJWC7E5FHSCBJWVE54HOVG7KY73THUJW3O72Z";"https://ct.automizy.com/8/CNSPHREDCLPEMQGBPU3VKHFOKLWOMMV3TZRZBD326YSJQ66BMMST4HNI6Z4NAWJWUWD6OEL6G7JT3DLAB5D6ER526GF6J2VM";"https://ct.automizy.com/8/A52KHBTKMNECXEVMHMTSVFFXBT76KEAURRVWJ6CCH3WSYIRQERGKKZYSRXPQGMK4SQIEJFFZ6Z2DM3ZWWZYLDPSWO4JZJ6PI";"https://ct.automizy.com/8/MHOKPAFCCVHIJUWGBRCDZRYP3LYH4CPJ3CSAT3RA2LWWORFQ3RZONBK5TJT235FEEH7GVKET23KQNO4ZY32TXPMXBLXBDSPW";"https://ct.automizy.com/8/CX7ST6ZG7ZZCMTG7IOPLA746W6G5BK47XNVPEFSXW7CLRFDGAKG6HLRUR7BQWOSJUSHOY6SV7COXBZ6E4QNQQS4RC366DNTI"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>25.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/DBNUR7JV2COLKWD72UTNSJESB6LKZYTMJWPOJB4RBHDM7B5SWCB66NYQDCPSJ5I26HHPYD2S75Y522NXZZC24EZWW4RB4SSX";"https://ct.automizy.com/8/7IHJQBPQC2LDIIKLWQIFPVOK73MEGK6PRMIPYUSFTUTIO737GDARNPKCDE5ZBT7LQUZQ4RL6VLRDEA5C7QHQH3B3UBF3UOJW";"https://ct.automizy.com/8/BUD4DR5W3G3CMXXHYX3RWQDNAG3BY2FRR2RYFXXFUSD4S3IIJXVKYZ43XXXMZSOIYEVGQPW6BNX4JQSSZFLX35YX75HOAJ6R";"https://ct.automizy.com/8/MK3Z2NQ72G6MUA2LXYYQ6R27H4E7Z2KGUTQYUEXKL3NNY6KVMNTACAKOIOAOAIIWNKWMITCEZJL67ZK6TRKS3VEDFTYU3MAZ";"https://ct.automizy.com/8/6Y7RJVGUIKNF3EMLXP2GTAAT2KUIHTZG5LCMO3BSLYCNXXA4SRMQETBLAB52I4QORPUMRQZXAG6P77G6NY3THFURXKF4ARYQ";"https://ct.automizy.com/8/KA3T52UTJGHUUQ344MBRV2R77RQYHRE4WBDZSGBVWPZBGY6S6SGJONIDURSB3O5CQO6YL4MGJB4XPI2S2LP3W23MV2FP5TT7";"https://ct.automizy.com/8/BTGULPTQMAUNMAH6GAUPUT6I2ZI5DKZVRYQTVJXXNG3ZXQC6UE2QWPYO7Z6ASPW4Y4VDR64JSHIWJATYGOPKX3ZC7SOBJWN2";"https://ct.automizy.com/8/OVKTTNSANC7POJOSSVUKNQGZCRNNRVRVRXEAK3RGUH3P6ZIF3AKEMTGKU42LYGYI7AWF2SPSBQB5H4X7H4NSTIKGU5AAMEWY";"https://ct.automizy.com/8/LX4ELDH47GKDH7YOVSTCAVSTIB5VWQ3ASULJL7WJ5U6JD2UYMZKUCHPEEPZDRACXAJTF6LHX6FHLTBGIWYB46GUZN3V22KTX"</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>24.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/U5B7AKN5525XAWDZYNPJCWONZOYH4OTFYLQQ7J7CH36BI7ZS5I3Y526GWQMZSPSHV3XV3JB47ISXPQICCDXFJMYQB6OPKUNH";"https://ct.automizy.com/8/D4OAZ3UO7AHHDJ45ZCMHM54RGR5AUOJ7CN73OYFL2FDG24NWSVGO4KSPNESHHSKCPLXPDUALCRE5RKRV77YTFZBPB7FOGQ3B";"https://ct.automizy.com/8/R5EWOKHTWYQ6WLMNG65CBMEJXCQJOCREMIUSL45QAX3PTR63XUZLY5VAZEUPRSJTLQMSU2K4RT6QJPSDM3XJ7OCL5JU2UY6U";"https://ct.automizy.com/8/VSPDRDNXP4N37C4I7ACVCRO2DRS62UKQOC3O4OJ6J6L3MBTPNQ4XSTUZX7UITLNJ4KTVZ6TRHYDN6PYZ45XZOBJHTNPUGNET";"https://ct.automizy.com/8/RGEOWSODTHI64DMJKNFWHUBIBGGS7MYVE7KENFWYIQEBQPJIMO66TUGHUGOPUKZP2DSVU4SJGMRI6Q4UBGXF2YFZWM5ESL7S";"https://ct.automizy.com/8/V72CDJNV22BY5QAWPXQKZHOKAS7GS5K4PHCEIQRPJDX5AOO2XCM46KNUCWUUC4FKQR6R3A4ZQ3TMJYUDUCVVGYTCRIZPRBXL";"https://ct.automizy.com/8/ANWDCQ7CEO26NEBFTOWZSCPFSDAQEKEVARAR3WX4LQH74LUHDPYT2INAVSJA52T5L6RVNNIUQ4MMRKCSDLB2YMT7O2DZX474";"https://ct.automizy.com/8/IKIXPSX5HJWBPROYGR4PEEUWG234LZ4OITGGZEVUEXQMJPNNLKMGLYFIFNAMSR7RKKLDGHJYFASHJ5I4XD6XGEMUYKFZUQHM";"https://ct.automizy.com/8/Q52JJRVB5FYBL2LOZCZBVDXSRDYDDHS4WGQT7RNGJ5DZR4SGFGT6KCEKZLXUZM7GPGO2UCM4FI5EPEXQCDGRNBZKMTL2MKMO"</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>23.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/BPL2ZU3XXDVNM7ML42NT7T5GJ7QPLJACS7GYP7D3MAZETFST4E25RVGOOTUNLPGK343ALCEFGUCZEPS7IIOBPFC6LKDVI3GG";"https://ct.automizy.com/8/J4SQOCTJFRWEGH7NYSQEFGFYVRL26KCWWOQIKFBFFX3VQ4IHTU433YLDEX4B37PEJEMYCKAIPEX7LV6GGJK52KG52S6EEWYB";"https://ct.automizy.com/8/5RO772HYA3RMLR5IIO4VDLJLSFZYPMFXXTXZG2KNF6AXQTM6YGMKVU7S4FIYRT4ROJNXPILCOIYA3KM23HS4RIJRGFKROGHA";"https://ct.automizy.com/8/M2WDOZERRIRIXBSQ5NAUKHQAX55VQKPNJ5CKYK2Q5MOIFWHM4XOWXQFUPNSMK3CSR562PR662ODKDYC3AWI5VPBBTJU2SFW3";"https://ct.automizy.com/8/YXZTHB3XZZN3U4DNRNMVQ7JXOWLSTMQJ6HV5X5PEK6CC34WCAEGGR4WKTZ4WLI32ICEUK4UC2U5PZJIPY67GVRBMT6W47M5W";"https://ct.automizy.com/8/Y3UUEB4WHJBZBUGPG4XCCWHAP2T7AQTOOG4CFGD5DDLPMQZ2TLFZ7IZLCNZODHZZ6OQALWEKHEVS3NMVAVEP7OCLAHUNPPNV";"https://ct.automizy.com/8/G5KNSBPNOY7EW62KIZX7S662BDQ3HS66DJGX2THJSUY2HAJMVFDBXZO23QYJKUAOVVMYFNKCFXLQNWGOZW3NOU7FZKFQRCID";"https://ct.automizy.com/8/IAJKEBCK67TJZ7WDIIH4OZXHE26VCKT5EDRLWVDZLORHSNUTKK7CPCLYVG43GNOGHS2VSII5IT6APOEH3S27TIUL4MD55X2F";"https://ct.automizy.com/8/YR7OZY5XXIGBGCOTH2V46SHNPGBIQ44EGPDSRFDNFGL2QQ3XHVLFUPZIDLEKQPRUUWVCL6DNEI5KSLTZNTNGMMKM3ERQ3W7E"</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>22.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/FQUGMRDRRUHBUGKHWRH4KW4QZABK4LNZJGQQOLPMIQNZ3VUPZQMJZZY7V6HKK2S6KQRWITSIA545PVT34P47HQOCYGPEB6XK";"https://ct.automizy.com/8/PXUSCIF23AJGRMQB6LHURXMLGUVVFICN22CZWKIPODAACWQXHLCORWXBGY2T3QBXHR2KJA7UVQI5IKCH5HLUZSQ5LGQOUAZW";"https://ct.automizy.com/8/QOTVCLNUEXXOU2T6PHJN4KGDCGZ4T22LHC2ETKMOLXNKRFTGKUWP6D2QOCK6VSFCZGF54LLGD73XYEVMUG6M7N4S662ED64F";"https://ct.automizy.com/8/3JP6OQZ6ASI7J3AVWUEH2V4E4RPDJ5JIEML2ZLP4YBCQHHO4BNZMCEJZ2EJ2IREAYTNF4M6ZPO7LKHO7IXY2OGE377T2YWU3";"https://ct.automizy.com/8/VTX4FFSJVR5D4XURLHTDZSLRQ2SP72UITMDNFZYSPQPYMKZPRPBV3Z4NLGOYI7C4MVBPC3C6OVWMMB5GJVZ4Z7FE6ACU3OI4";"https://ct.automizy.com/8/SQPLTC2BARNCJN224XRDONS56O5HJSDOSVV6RNZQLININMHMF7ACIB67WP7K54G55B4NC4UHNXTHTRV3UBDEJJTZMEFVEWXB";"https://ct.automizy.com/8/JH52GC2LSQRJ6WYUMZEPFXVPNR6YKWAGVS6WX7USJWUYL22R6BSOFLSEARYOJHPPUHBWQLCP7WJII6DGKUUIWTZ7IMHDKXN3";"https://ct.automizy.com/8/LU63RXKFZ56A5ZDGGUVCQYMAFQKFTBPJCO5YIARIE4GJUEYTC47TH2TQ5C2ZOKOSRWNIHE5GQPZCPYIAYMLXAQNHH6DTPNS2";"https://ct.automizy.com/8/HUBPQP5HPVUKEKL3WQ4JZJKVOTYBYB54QFJQZBSAJIGJY527ENVPFHFVOZNKWP65TP4RLNYVAGCE3EG4KFQNACQ6DT6DOBWV"</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>21.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/DG44LSWWACBXK732EQOBKCPTK3P74SASHU5MHGF7JRQL5GEY3VAKI7ZNVLT2EG75CRIZBWJVQSWWTUMYC6DOHNFSP5FIV3SZ";"https://ct.automizy.com/8/YADZRRQM5YFCYEPQP44MLD4X46EVKIP4OXOQU77MIPPDDBEBA5FDMGL3XLUJHHSVBCDQ6UMHY3ACDALT3WRNXKCGECYFPKY2";"https://ct.automizy.com/8/GDK5GZSSV2PXYAYB3OTI6HLMFIWEP7AYQWF3QX3GACX2R7Z7EJDRD4YFFUR6VO5Q4BZZAGY2PJW767L6KTYLFAUQL3CKRM4K";"https://ct.automizy.com/8/TVMXOFO5XTY53U4TNPVRFVKL6EBNTL2I53KDDYM7JTNPACSAFYHU32PBDPXF3PD6CLT6LRTMXVN5KCPWUXAZB7JRTPCHLVEP";"https://ct.automizy.com/8/XCBVI4C55Q2HXKCAVTROJOQR7XZSJVDDESIKWJ3CZAFZCLOGT5N4JMKS7AQ2CWHTFFWEASIIB64ARFREMDKA2AQZIXH2E3TK";"https://ct.automizy.com/8/UUXNGAQTQL23OFHCWMFHKE5EFED6AC7PES45X5ZSTNTQ55MOIG3QWIRYJWANI75VKYF7W5V2PBEKUNWPXU4PJZF4N54FGXIA";"https://ct.automizy.com/8/FOMVBANA33HTBY4ZRUMUARSFMTYIEONQF7HHNYH53XULJWHBKURUNDF25HTO3DWQORUW7KRQWMLHCKCYVLYCZVPJKQQRN63L";"https://ct.automizy.com/8/GSAV42OHLNAJBLSN7EJQ7YL3QHMC3VDNMME2WPLUQ6EK4B5EJGWB7VNQBFNPJWQD4QC7JTOGRNM3URFZGQ65DBDO6W26WEOH";"https://ct.automizy.com/8/SMA3GMQXUQQA42JUCSEB7NAWC222DOW7C2IDA73DPHNW7JTXJYOXH3CGNF6DSE2XF4OJK6E4UEEUGN6PF6LVDTQCPKV6JB7Z"</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>20.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/52MYMU77HNZQBCJG53VRM7DLWFLQ3W4LP5AWUQSPLM73TVHUCKXMZPHLQ5Z6AQP5NEAU2HJ6CDX6BCA6FDLFMPJTYQA4JYQH";"https://ct.automizy.com/8/CVILTOIJDLR4ERLRH2EGWQ4JOBSFDITKS6DWO6CQGLGOH2G2LYM2MKRSHAG2LOCK7LD6XTY3BAGF5F7Q3MBIRSVIVR4QVRID";"https://ct.automizy.com/8/KVUFZL3H4JMYHNOKMMW2FWHNNXEDXJDBJ3TJTCUFOXGELPXPUV6FPS2OKWSUA773OCMOF5YJJDS4XPS73KSZ7UYEE7MN6437";"https://ct.automizy.com/8/TIYEFUWBJXH2WJ2OHPKDWWUNGXRM6EKNOBQIQ3DLGO2VSVPF3VIXKZABF26QDHPA22HEARGTQSLRR7SV66CSTAAZRFGQ7MZ6";"https://ct.automizy.com/8/EGH7I4CWDHKDFQJ3EYLODPV2R3TWJLVAWTC6XURJ5WO4GOLIYYP4X42CTDJTGOZEEGQZOLYS4ECFNFMYXSAWLBEEOEBOXGLC";"https://ct.automizy.com/8/DGEYEY5T4OSKLSX2I7E2GSPLSLHIXEUMFWR57VT4PORAJTOWXQ44EUOG2HKD7Q2FYSNWGPUBQA34H4S736DCJWCCVQI3FYYG";"https://ct.automizy.com/8/3GYKPGCDLUH2AJGLPHYGVKKYMVFWZITVFMJ32OT6NKPFOAJCC6QPPZDFNHZVE26OMBDXBE7BH4KNSVV7VSSGLHCUSZLJOTQF";"https://ct.automizy.com/8/PEJRA4FCQX5K2YA2AAFNPFJ5PXIQPEU2BL55RAVPCT32RMVIME7IOGR5IP5H4MVDPZKZAZBVSY5LWEBYV57I2SRM7KQYXLAL";"https://ct.automizy.com/8/TKDSDTISTAYXXGXZOR5B2HQ4ALJWURUVSMKGZD36TRMGMTQPU4VTPGF6UUXMGJ26RTELQBXPIONIOJWLNCPOU5NVWIR6AOS2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>19.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/KHKBRB44AUAKFI444EDPNESHGGED5FSB4MBLV7ZXJMUEGMHX4CEVD5KYJ63Y4ELNWWR7GOFKM5PIZEG2KKO5A3E36CYWA3C5";"https://ct.automizy.com/8/YNGG27R6DEG4BWSFERCWW3ZC2N2ESAFI43M76QWTZ32JSUVWIMJIDKJW7ERWTWMRTWOUCO3UUM5PWQEEOGXAV6GBGPR2OFIG";"https://ct.automizy.com/8/FLTLIZFZDWCUGNWBHLPIFEYNSXLWUVQOE5UKGUAQCTJWBOYZFJC4IDCVGAWLLI5UYGJHBAUIFZOS6I63IP4Z5EXYL5VP44OQ";"https://ct.automizy.com/8/DFTCXKWTEV6C3I3DBPWUUXRW57N4B5GM2RMNSSLCGH7QFVB4OL2C2AP24WMQIB7IS7ENMW7MSXO2Z5R2YPSBVKGGEIANGUN5";"https://ct.automizy.com/8/2FZZRUSZX7A7OSY7BNFXYPVNMUK4VNGLILTANDOSLWSNCWJE5WVUJYQM5NCACSITFLERNW4GXTBJFKEJV7RCC74SD5TZ3OHV";"https://ct.automizy.com/8/7BUNKYOSWQ4XMDMYATEYONZ7BBSRHKRROLSM3SAP2QOD5L7STMCOUPFXIP6A5Z7BQA7IXSSIUJDMXCC6XOSYF3LLYVS27XMQ";"https://ct.automizy.com/8/Y4BWNJL5XBO2SVDSVBZCF3CEZDFXZ7UPQB6NCJ2HWODP2EW7JOJWJO3CWHNWYKZN5DMF4UTA3CXY42PPQ5LZRCACRJ7D3MMI";"https://ct.automizy.com/8/MVZEBJZECAFQXJIBIE46YHIBCD4YV64EFA6N5TWV7BHVHSCVF2RXSZVV6S4C52FGOY4X2GHIWCHZTG7CKBO57ETNCD723NQC";"https://ct.automizy.com/8/IGHDGX6YCF4XSVAQJVVILCX4BEMR4TN47QJ4MY63TTJR6FZI5TKMSKELNWDUUVZMZ75UCXIXP5WGVYYORIFFHLOGNDCAPHWU"</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>18.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/5C3JPE5AWD3R723K64J3MMW2XDPPJITK3ZXZ5267JH6535X2Y2LFPNOQQM3LKQ5V24VIF6BH3KMJYMFSJ74NMXAWUFS5H5H2";"https://ct.automizy.com/8/6CSS6Z5VSCNIBYGLEHAKDNLJME6RWRNUDD4GJBJCTV6RCGMUHZBO4AJGBSVAJOK7RNHHXLKZIPIQWS5LTVN5RD35EDMXLSPQ";"https://ct.automizy.com/8/VUZO2NOBK52EYGCC5NYRWFS3A6EXN4ZTIEA46PVKDM5K23U6N5LKQZHO3YKUED5TBLKXVIL5C7OBS3IY55WIULDGYBBRMNIZ";"https://ct.automizy.com/8/KUS6XI56WAHQXAAHU2BDQRRGSCWNVICR3COIUWQN52HIAD33H4MJQEIIHQJNT3ZMXIVO5655UK7GTH66CF6ZXYXH75PMSC24";"https://ct.automizy.com/8/UMQBCQIZ3UXG5OGPDWP7Y4LSAYQXPZ6LPJZCPFFXEONVUYG64H5RCRPDA5PONAKI3CVWDMGGGZIAX6XYDOL3GTZ72C7LDBRI";"https://ct.automizy.com/8/SSAHAIIG7ND4NNX3J7PU65NZPJCXBAH53Y73263XNBMEUINV6G3TY26LTELTTNVYGD4C7XLJZAOW4V6IYR2G2UYYMVFEFD7S";"https://ct.automizy.com/8/JL3FFKLTTOXPHXUYSEZLUEJINPBVO5AWO6LCCB6F7IKURG7TGB2V4ET3R6LGPCUYY4FTIU3PHIKXYCJYHW2QRIBLA3JEBPVI";"https://ct.automizy.com/8/QFAUPXNC4CMVYVQYXHFPLWHZC6JCVKDZFGCG447FVHCPJ2NDBYLFJNVLHHX6WKWRUJAS5HUYYUY6KRCAUE4KP664ZW3KHVLU";"https://ct.automizy.com/8/Y4WLYT2TN5N5WQKTVJ3OGUQAD6KOXCU2WFZARZ2DRCR2HOHOBFOWXEIREKNZSGXDHGTE5ZELQJI2UN4TTQELBUFO3MQQ2EEL"</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>17.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/BBHTFYHJ4H2MDPNEPOILOPIMVUQKP7SYYUC7TRUY6WFQMHRVXLXEOLS2TX6FYIOKSH46C7MALQLZQYTQMFVRXO2TAK4AYXLV";"https://ct.automizy.com/8/A3GWVDVCFT7TQOSXG24JJZDRVDKZUK6DT3KWAKRGEWHE75G6WQHUSRN6ETHLCAOI6FVGV254436AWD5Y6TR2IANZ7UBNMOIX";"https://ct.automizy.com/8/STPCZDQIXAFHCAVR3QDYTX5P553XPZLOLBZPKRYOOXHUZIJWDDPKY5AUHO24LPML65RKSNGGFHGLCL5IBKIAHN7BVRCY4TI4";"https://ct.automizy.com/8/2O23ASUMSLITYBCDG4FEGRCYKXJUH3EMNGOXJAFDLQXYVH4P6H2N2P7QDGQ4W3H6US7UPG2Y7UTS4XSBBQGV3ASLIBPAF7SO";"https://ct.automizy.com/8/BQTW3DKRWEO34GFH56LORP6BS7B47FLFEYJRB6CATDKBBHHJ2WUMEZQ6HOY6ZTC24L7QYWSAG6XVTU5U3JSBVVBWUXGEMXQG";"https://ct.automizy.com/8/RLOCE44DRR5PE7EAH2Q2TFAA2GHNZ5UFKQNIHJYCAKYZIBMJZTEHQV22UTKFU7S6GKPJR5COIYZUFX7FGYZBKT24HEWW5SH5";"https://ct.automizy.com/8/HCJWGBEQY5M2ID5ZDQNSWAX5W5N43Q5V5KWTXL3ZWPUMCGI545O2IXMT5HSM4FL3C7M4ARENMBVF36ORUHDBGSV63DW6NJ5D";"https://ct.automizy.com/8/ZEHBT33ACR4O4CYNE7CBMPA3DCLGMQHNQB4M374KRRKS3BWVJWKJV2LIC5TJKQ63JM5UVNTUJRMAPQOSULBM6ZZU5L6AYN6Z";"https://ct.automizy.com/8/HQW7PEACHUVGRQSNALPODMN4ZJ3CA4XCMY6KC7JIK66ZSNXR2MPT3QOLIVHDUWH3FWYN4OIC2PMRIR2GKK3MCP3EENBFNMCQ"</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>16.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/YOTPR5OHFAFCLR7WOFF2LV7KROZEAOXT4VNXQN2S7UYYQPCXBDG2BSUEOQV22JFGBI2LGU3W6F6MNPJAOB76L5ND7P76SZZL";"https://ct.automizy.com/8/Q7TPUSZGDBMUUUIN6S3F22UAFICPVVX4QBMF25SFFVCGSTVUL4PJB663HOIHDIPYBVGYLWLI43GSJSLCSHICCVP6HTWBXHMM";"https://ct.automizy.com/8/GQRMK3WVTUKKKFK4BMLRDVJDC37ZZUYC5ZS2GBOHVZTB475URD3JRAZO4RT3FGGCWQTS5E7UDGLOP3HHSJIUYB42OXJRIU6X";"https://ct.automizy.com/8/LF2U6HJOFSJF7MUY3XYTRIZPIIEDXAKBXPA4ELJQV6VGE3FR4BA7CS6JG6YKTYKTFIUKJTO6WXJJD7QJ46C4ZSQKGIIFCMPM";"https://ct.automizy.com/8/LJ67HEOMZCQG5ND3G5AJWNV225IJ3CD2GPJQOV2SULVIS2J3L2AS7AXQLODGI5WY5QUYOHGHWRAXHTLVBJCXB76MNNQRJ43U";"https://ct.automizy.com/8/YWELSEUMWZ3EDQ4YKHOYTGJZSOEG6ELW7I2B7TOBAHAOA3MYEYGEUBFJ67QO7KRLTPQIWCTYHFVLUDLVMYPEKLTKLELKGZND";"https://ct.automizy.com/8/7NNAAOS2PM2PRCHRBRJ4JSTIIITZAUKVWFKDCXADYEZUQLGCNG5UERMF5OVPOTTTLISJYTHSBQNEPCCYWLF7462XQ4MRIKEC";"https://ct.automizy.com/8/U2LY55EWL7CLUMTBJVA2445RL5CHI5OI4UDPXD4UAGWHNRO6FXBBJB4EWXZQCGCN277ABOP3B552JM6KK7S4QQADXL3OYGVW";"https://ct.automizy.com/8/QAKSHW2FANK7UAK7D7PRYJAXBN76SP76UV7YOZFXGWPV5Y3LCPXGG4XL6YBWQJHSXJIQFAX2TBEAPCDIA56KYIBK6LQO33ZC"</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Origo</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Origo napi hírlevele</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>15.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>"https://ct.automizy.com/8/4WHZ2APIXDTSUCRQFXWGSCVLI5L6WKJ5GTGQHNJ626QAEUDNMIBYWZQTBGCOM4UEVPFJ7SMI5T3LO5YE6ASJMW3V7NTF47UU";"https://ct.automizy.com/8/JGCZMC2LGJI6ZGCUW4ZCLYU2HEMZW2ZWQQSNP3D7PEUT4XY2OSZ7N3SUFGUAOQFSQCZRU4244SSVVZCCQH6H2QGT6NNNSHKS";"https://ct.automizy.com/8/HMGLYBYQOTFUGHZJOQGPGZNMYPFREGMA6TXFZVZ3CUSS5S3XLQYV7HS253BDMNRCN36C7HZ7SMF72BXEY7AFU4HPJEJSNM46";"https://ct.automizy.com/8/RXOJX6CEEHU54HEBLME3NFE5OCNTNUONMICBGLLJMGEOGFIAKXPUJLJWWYK6XB2BXF5DH7FT2CFMLL7QJ5ZHPM7FQCMXXIIQ";"https://ct.automizy.com/8/WFIYMDNM7SFMUQ54LHXBPHKPETSPEA7IKTEF5FHPQMJYE6N3Q2RMNSQLIGJEMVDWMPVNEE5NVFXFN4ANPEYNRVRZX7SZFS2K";"https://ct.automizy.com/8/PYPLH4GYOJZG662KYYZQJAY2SAFY2Q7MXAPLEKHROZDWKFF4W6HIPMW534GFPKSJHYBHJ7GBX6MI5DV7RAC74VVT7ZKMIMHF";"https://ct.automizy.com/8/QIT7RN6ORXUS45JMKUSGTSRDQCHBF6FXI7DFZLE2EWHWVZNVLCZX374LRMYCQJY2IMDTV5U2ILX6UJFAT6TS6M7VXQNDDJHW";"https://ct.automizy.com/8/OYFWFYXSNSCDKMB5JMNOE3OIYWUYVJGVMG6JRJQ4B4SW7HXZ3IIVUY5GPJV3BVUBBUNJKLMOWXKBLZMJJQG3OKKLCLSHCD7J";"https://ct.automizy.com/8/E2T4UHB4AEVMNZO2ESL2A5UOFZGLG3X6S4RUIOF5YUCYOZM7VIJUTOA4DZCGDKASOUBHIQHPSSEYRRIQ3LHSZI4NN74QSXER"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Developed and tested link filtering+extracting Der Standard
</commit_message>
<xml_diff>
--- a/research_data.xlsx
+++ b/research_data.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.77734375" customWidth="1" min="1" max="1"/>
@@ -1954,6 +1954,644 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Abfertigung, Feuer im Lesachtal und Good News</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>24 April 2026</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_27&amp;ems_l=9073610&amp;_esuh=_11_ea6addb532084f0908f25cca4bd830160a9dffe94ce5b0cc10ed0af739d15be7";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_23&amp;ems_l=9073610&amp;_esuh=_11_f5e63db7dc4ec87497b67f626d94c26e5de448cc4326d5ebef42902547a6c026";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_31&amp;ems_l=9073610&amp;_esuh=_11_a4c120a373a1c1ef328c14d2f4c50537bd7034eab84ba75853bf6a10ce1c6f16";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_43&amp;ems_l=9073610&amp;_esuh=_11_24cfb4386da97f270d415f7b97a27d655f7466079227a2c90a3e73866ea3be48";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_35&amp;ems_l=9073610&amp;_esuh=_11_6ded492f67d24312b4cb86c2ec70690effde606c1230233e6fe8ac6ea67c2ccc";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_17&amp;ems_l=9073610&amp;_esuh=_11_2b854323cd6afe0ce549e31bf6867a6ff1445678b6054d664a502f45b083db6c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_19&amp;ems_l=9073610&amp;_esuh=_11_5222e23926baefb2c14b714f2e1df9c111e10a8c53c7b34f7abfa6e752954633";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1221_7398480_1_39&amp;ems_l=9073610&amp;_esuh=_11_f29f2cd88744d855afd85cf1927a06d53b34e18e502996f4da3ded4778aec8dc"</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Irankrieg, Tesla und ORF-Stiftungsrat</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>23 April 2026</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_43&amp;ems_l=9071921&amp;_esuh=_11_470aca6c75e48fb643c8be450f74d06a1f394ff289be5eacd029d3d4d936e686";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_39&amp;ems_l=9071921&amp;_esuh=_11_3ed1cbc44a79cea7e3886b48908abdab80e628083453699ea272f983afa9c102";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_35&amp;ems_l=9071921&amp;_esuh=_11_4c8dcb71c36fdb392f2ac6caa4d231fa3c3b9d5694ea8d91ffede40da12b3afb";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_27&amp;ems_l=9071921&amp;_esuh=_11_f489bd303ee72a2a4c12b624f686dad9080a7dfea7eea3ff709f0bc689d805f1";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_19&amp;ems_l=9071921&amp;_esuh=_11_f4c5438d48ebaa7d07851df70f44411666ac42e4dd4bab0f5825a8860d0625b4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_23&amp;ems_l=9071921&amp;_esuh=_11_6885620b9db37e28720a2afe6a23b31800ca0dce3b9666fc32f1e922450dc7dc";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_31&amp;ems_l=9071921&amp;_esuh=_11_72ece7ae4c6d022167e39a00117106c7787e873d12ef636b1631cd72c3395050";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3219_7396941_1_17&amp;ems_l=9071921&amp;_esuh=_11_e59d8b0a0bc385192645abf7af124f4cc8e7161bb8129c71eca4731358feb06a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Wöginger-Prozess, Ungarn und Abfall</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>21 April 2026</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_35&amp;ems_l=9068411&amp;_esuh=_11_72020b3fad56d463ffcc926f7386e51c7041ed5488031bc2db329e122cb5fdca";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_39&amp;ems_l=9068411&amp;_esuh=_11_bdf0a1647a76b2d2540fe59365578eaa581ef2985eb9dc914acda4ce435905cf";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_43&amp;ems_l=9068411&amp;_esuh=_11_481b073b9b8db801391c33f2a0c2f4ad5714cab5894a11140976a184b7dcd32c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_31&amp;ems_l=9068411&amp;_esuh=_11_3193ba1d1bfe394c9f5cbdc3cac480212804ca5ad36b8c4e4a10ffaf5a59325e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_23&amp;ems_l=9068411&amp;_esuh=_11_6e1270965600f770d63bdb1334d7d728c610400686b4e43868e6afd183120f86";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_17&amp;ems_l=9068411&amp;_esuh=_11_afc1bd21b1360d3adf175abd23087588123601eca7ce90d7609acb8f702c7c4e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_27&amp;ems_l=9068411&amp;_esuh=_11_98d2daee09b02e39654ff5f34bed25aabc1c65fa8578827b39fdad61cc16db12";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2499_7393703_1_19&amp;ems_l=9068411&amp;_esuh=_11_287b9c4fdd19cf1552a56b62c21bcc1b04c944c79b0f9e581f662f736600a2cc"</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Operschutzstelle Zara, Iran Krieg und vergiftete Hipp Gläser</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_27&amp;ems_l=9066653&amp;_esuh=_11_433f012702842b28b36f55ddf55ebda07ff270bb744402b849a54b0b8f612c04";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_31&amp;ems_l=9066653&amp;_esuh=_11_1a76b8e8d49532c75ea615c35dfafda4a9a3a6e0ce11224b6a843abbcdea717e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_39&amp;ems_l=9066653&amp;_esuh=_11_38a835e6a7fccec364b30d40de0114e7dfd366909577bdb1381de5def9dc4218";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_43&amp;ems_l=9066653&amp;_esuh=_11_90df9a5a72d1e8571e43d73adb7dd3aab57c202e48f2689374bf725d5adcbca9";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_17&amp;ems_l=9066653&amp;_esuh=_11_c6b36d55294ab580d6e04345b1e5d769dbd62f5572e49bb7527d4c1b84fb138a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_35&amp;ems_l=9066653&amp;_esuh=_11_7aa9558b68fadab205a57d469fe0111181dad0a7b839864f772e9855c83296d8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_23&amp;ems_l=9066653&amp;_esuh=_11_d1114ddf6d1bc7b72d1dac772e540d18c6faf9a5bf9b0643a92d44e896c594d4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2983_7392052_1_19&amp;ems_l=9066653&amp;_esuh=_11_bc4e63a0b6ab02489e3f1f957db4adabc090d5c6259e60bfc3f8fcdc4ecf416a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>FPÖ-Finanzaffäre, Good News und Atlantikströmung</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>17 April 2026</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_31&amp;ems_l=9062105&amp;_esuh=_11_91f7dd49293f54a96b0c247d05af41dba7196e02667df4e2aa55db6df12004a1";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_17&amp;ems_l=9062105&amp;_esuh=_11_08cca55570c272311fcfd94ef8b7d4cab0bf87d79d528657531be8e7d355dcd1";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_27&amp;ems_l=9062105&amp;_esuh=_11_cf5e77b34d3a22f63cfc8c94901d2b00ec4d737d6403b9d03b31d7d7498de79a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_23&amp;ems_l=9062105&amp;_esuh=_11_b84295ed3691ea90f836a2fd2ac0817f76f797e933556715a97d5a76af04215e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_35&amp;ems_l=9062105&amp;_esuh=_11_8290ea60e48ebba1d4f62d42c76a76cd141091b9cd0770ee150edf484df38fd2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_39&amp;ems_l=9062105&amp;_esuh=_11_591f30f2f77b2106af49d03c33f3000b4be089b0364e7dde954e1c7c3a1840ad";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_43&amp;ems_l=9062105&amp;_esuh=_11_5f0db8a0df85fbc4ab2d77edb786ab49abbb5215160144f0d3ee7838c77113f8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2563_7387971_1_19&amp;ems_l=9062105&amp;_esuh=_11_2417f5db00a9b06c23aa5bf8a737756e8723b1007fa46bdc885ac41f2a43a310"</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Flughafen Wien, Familienbonus und Café Central</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>16 April 2026</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_43&amp;ems_l=9060338&amp;_esuh=_11_bd0e2767bb867143aa31cd39f3b89ce4749086a27b63063c2a282205fddd66f8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_39&amp;ems_l=9060338&amp;_esuh=_11_02a669dfa2bbcca73d688dafe444b0092e728452a641d12c8f04c3780cbc29e5";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_23&amp;ems_l=9060338&amp;_esuh=_11_c8a6487eab350b014d552d07582326acb0f2fe0057d7d6dcc13d98714fa9fdbb";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_27&amp;ems_l=9060338&amp;_esuh=_11_becac073a1f824c756e6df52e39c835f2ed6b7ab7ae13f76212415ba18b30013";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_17&amp;ems_l=9060338&amp;_esuh=_11_d19effed68b2208abc4efbaf57515938239847fa91cb8b39435b1d1d596d4b0e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_19&amp;ems_l=9060338&amp;_esuh=_11_1ddb17c33fb868807b6675595f4b81a9f5720a51a72771311db74aa42a84e7c6";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_35&amp;ems_l=9060338&amp;_esuh=_11_b6a8a3778eb1f6bf1f2851b2b63d897c0add2e45237501736ebe9f80e6799df2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2298_7386356_1_31&amp;ems_l=9060338&amp;_esuh=_11_5493fb54c8a9183899128292734208d024290fc98d24de726bb8e3a113fccb0a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Nahost, Raser-Fahrzeuge und Ö3-Jugendstudie</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_17&amp;ems_l=9058586&amp;_esuh=_11_a62ae6005d1da59d4efa1e633184519e4738c2af34b8affeaff2c6d5e17dc57c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_27&amp;ems_l=9058586&amp;_esuh=_11_ca47ec9000b0cf59bc1cafcb0a6203df438f65ac65d67f8844acf45c34d72a85";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_43&amp;ems_l=9058586&amp;_esuh=_11_c022d106fc308ce46f7026309a150174fb17d50adad5face73b2a09d0ca29690";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_35&amp;ems_l=9058586&amp;_esuh=_11_4faf4558ae28fc23499744a26d3a4de35cf1380584ec4f3031f3d76816439809";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_39&amp;ems_l=9058586&amp;_esuh=_11_46f0ef1920ca9094bbd1d57eb35124f293c622797ef0d31971046c70e5fa76a8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_19&amp;ems_l=9058586&amp;_esuh=_11_0c2fdc20362270e48a8358560c65fa7d0c2840eb05b37f93265e6cb862bb86ff";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_23&amp;ems_l=9058586&amp;_esuh=_11_48c335e6a78821210454a3ec23a939501c490b8a9c699faea5a6b0956d02a13b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1492_7384766_1_31&amp;ems_l=9058586&amp;_esuh=_11_8f89c0bea92bb5c74cd526a7479300fa481e205fe0619650873bfa32e50b6c66"</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>OMV, Iran und Arbeitslosigkeit</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>14 April 2026</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_39&amp;ems_l=9056766&amp;_esuh=_11_a3c76734f7f1ee1728d30f2eb52457b2721f23e28de43892862f0c5136f7d2fc";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_43&amp;ems_l=9056766&amp;_esuh=_11_e63e4a6e6cbac171bcf593008bf108d15ff006e01135f48f4703a699813e356e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_19&amp;ems_l=9056766&amp;_esuh=_11_bfa7b9e2c87f05e354b80f8dc933ad8eb6e45f422fbfd122adaf79d2624f0a16";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_27&amp;ems_l=9056766&amp;_esuh=_11_b2f19b048a728db093132d1c6d2d811d62fbf5ab3e90329973dbb0b3bfad1b81";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_31&amp;ems_l=9056766&amp;_esuh=_11_95c64174aaf02563651dfbba16f8278c665a210c7335500527b2ddfa200df5ee";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_35&amp;ems_l=9056766&amp;_esuh=_11_541d7a90cd52170a3c68ef263a949765ae903b70b23d326bcffa24dbd323eba2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_23&amp;ems_l=9056766&amp;_esuh=_11_44688c89957da8201ef6d91622aa861cb46d35c286ac89afc050f897e7537876";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1003_7383164_1_17&amp;ems_l=9056766&amp;_esuh=_11_32fe274a4c2418d7f4fd3ccade837d23f2fbd35049c552d65e984e85fa2ef91b"</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Ungarn, Keytruda und Telefonieren</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>13 April 2026</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_43&amp;ems_l=9055185&amp;_esuh=_11_d2aa612612aeae4fd4b810da18b1ca5ca1d3206455a46db1b26f9673852f38ad";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_23&amp;ems_l=9055185&amp;_esuh=_11_4f7b525ec21b7d1411097bf0e82135b1df698382fa0a7d0202c6c75b9b349635";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_35&amp;ems_l=9055185&amp;_esuh=_11_985bc341131480f8cd90c059536f831869da65438aa0fa3c24073ea80568fc1b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_19&amp;ems_l=9055185&amp;_esuh=_11_4499143450398736f2e69fdd3eb8d81015c16cb9bdcbeadb3143e97f7b26f9db";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_39&amp;ems_l=9055185&amp;_esuh=_11_2341833ae0462700fa0ecee9d36ba0794c0a6fea782a7f39af3839da8d10fbdb";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_31&amp;ems_l=9055185&amp;_esuh=_11_5714d5b394abcfb97434be6c8f5930c2d4dcde29cc7f0ca58a43091770d2c8d1";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_27&amp;ems_l=9055185&amp;_esuh=_11_0889c2a574e8216c1b9ca70fd2c09d93974c8e65b520a9bcf0ca493d310ed083";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1109_7381661_1_17&amp;ems_l=9055185&amp;_esuh=_11_b069bf7e4f7ac63e676d1ad62b54947571c68ada28f5cfdd89c779c0cd9f261a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Wohlstand, Scheitern und Schachsport</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>10 April 2026</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_17&amp;ems_l=9050726&amp;_esuh=_11_af750b4587a9c21491be18d9afa419dec90cbe223b37091b99b34ee39af561d7";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_19&amp;ems_l=9050726&amp;_esuh=_11_ff6625897758d9396fa3505518a2a6835fdf7fe1b7b6559bc8bcf15ff70d4992";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_27&amp;ems_l=9050726&amp;_esuh=_11_33b7353f3f0ba063ea43d3ce6f60151c432453e5ff5deceb388ec3dee0656277";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_39&amp;ems_l=9050726&amp;_esuh=_11_ad79e2f222acf288f72f6354d0971e963c7504eac00d4b3b6e2ac04e4294130f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_23&amp;ems_l=9050726&amp;_esuh=_11_4d303cb680970ddfeff51f86020d36388de2342ad6e3e855262e374f6e0aad3c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_43&amp;ems_l=9050726&amp;_esuh=_11_3f466679721ea778c84a9df6bdf7a8cc62398eb583f31c163bf95f8e2d6b5006";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_35&amp;ems_l=9050726&amp;_esuh=_11_340add3398ca266cc07bb3f456c9cd39b586dde247e53028b846c00ffe1b2ce8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3972_7377781_1_31&amp;ems_l=9050726&amp;_esuh=_11_bbc87d3b9c38c3cd187f47bd0c69d1463187fae7f828ebad762a1b5e0d579151"</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Raser-Autos, Goldreserven und KI</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>09 April 2026</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_35&amp;ems_l=9048945&amp;_esuh=_11_d380a1d71d967dc1b506754c0a1bc41fbe671d2d72c26c85b0fe2e1bc9fdcbf8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_19&amp;ems_l=9048945&amp;_esuh=_11_30622507b70bfa26d5a106846db56b8414ee333c5be3e24f05c6338d29c802a4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_17&amp;ems_l=9048945&amp;_esuh=_11_e2cb372a05c457838430def3fa9255bed9578f857c399552c06748684aebe0d8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_27&amp;ems_l=9048945&amp;_esuh=_11_ce0e10b1e12bd37a25c92fb39ce95ce4b5e918a05d7ebe770ed7a0b67cb1ae25";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_39&amp;ems_l=9048945&amp;_esuh=_11_8e20e577e6105925705100de243e23270a01151efbef26f11dc48d2c3ee0dd45";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_43&amp;ems_l=9048945&amp;_esuh=_11_f056ba9dac809e9e0d6972dad3c32cfa099082c8d0b1f46d12314751e19987a9";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_23&amp;ems_l=9048945&amp;_esuh=_11_c0c64de3dd187745ab04e5b10373cc4438c91864209a9799ce88df0f758d20c0";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_871_7376022_1_31&amp;ems_l=9048945&amp;_esuh=_11_d5387f190c395379895a57e3a05681b48196ab869377f077007bbee50b403d6a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Irans Regime, ORF und Psychedelika</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>08 April 2026</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_27&amp;ems_l=9047239&amp;_esuh=_11_6cde6b9514a67be48399d6539240953c62a2085a323b3661590c2d5afe3f5726";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_43&amp;ems_l=9047239&amp;_esuh=_11_1adf67b8cc0d33ba4ecb8a40dc7e5e58e58465b478744751e2fe262667d9139e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_31&amp;ems_l=9047239&amp;_esuh=_11_5b40aeeaf26c2dd0d96b4e3a3d06a4c5fdad91de422ee30ef5eebbea0420d23c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_23&amp;ems_l=9047239&amp;_esuh=_11_969234d973bfb0bbf60d0026be0dde18b12c8358b71f11b29b23b55ad8f453ac";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_35&amp;ems_l=9047239&amp;_esuh=_11_5ecafdab2ee4aeedca9c468000b3994a542580a786803c95adc18ed035c45721";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_19&amp;ems_l=9047239&amp;_esuh=_11_457db752e5b4df665a8400ae5b2a8dd29e485f088349dc15961a46d738e7853a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_39&amp;ems_l=9047239&amp;_esuh=_11_0a5d7aa030c1b911e6507a9561b2a6425731bc051af3a6aec1e59130934bfa69";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1668_7374464_1_17&amp;ems_l=9047239&amp;_esuh=_11_c147f0e638811f2a2cdc6478ad14ae3b9fec1888c8fd328591e8f2798a083d4e"</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Iran, Windenergie und Artemis-2-Crew</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>07 April 2026</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_17&amp;ems_l=9045435&amp;_esuh=_11_b907c5b4ff9a8f8f50035dd011b286f952bc052b932eb250150d411f41a39ba9";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_35&amp;ems_l=9045435&amp;_esuh=_11_618217f8ff45633d3f9d0a8a5ea2d1560feb5c007bb27dd8d458a02e52cfd188";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_23&amp;ems_l=9045435&amp;_esuh=_11_525c717a3afbf23552e37ef3e06c943d9a49caf5715deadf0a57bd99392b37c5";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_43&amp;ems_l=9045435&amp;_esuh=_11_c7f2ee920cb5cba0dfd085f7f23c05b6aba3915fce49ecb28ced2948a56b725d";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_31&amp;ems_l=9045435&amp;_esuh=_11_912589b513f9c8bd8720924b58b9308645cb1449414825ec885c47b19d269b70";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_19&amp;ems_l=9045435&amp;_esuh=_11_a96c459322d2a0e871af4bb5f6f29e0c3ff2fef3274c494a03e9726f61006fd8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_39&amp;ems_l=9045435&amp;_esuh=_11_ac8a4e2829b4d5b8dc0607f617dc97b4b2b0d466b0ee6f7ccb9948cc08423924";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_328_7372820_1_27&amp;ems_l=9045435&amp;_esuh=_11_88097d413800d1489d50a3bbad26bed31ef98f9be354af8d611690299669eba7"</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Energiekrise, Pensionsversicherung und Kirschlorbeer</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>03 April 2026</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_27&amp;ems_l=9039634&amp;_esuh=_11_54ee179a0ef80455eb9c6a59a63dda83ff0fedb72d47cd7ced0cd05c67f352d2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_23&amp;ems_l=9039634&amp;_esuh=_11_e23b8dc167385c17044e245a92fdeb91ec90eb0bcc7f3fb0437802c2dbb1ac23";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_31&amp;ems_l=9039634&amp;_esuh=_11_b21814f88927d85933830e83fd5df4049c128360c9dcb76c7ae4943e5d6dccb0";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_43&amp;ems_l=9039634&amp;_esuh=_11_158ca1b075ca61f049d7224b346c011fa4e438e3d4dedf715c1f6d0317f391a4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_35&amp;ems_l=9039634&amp;_esuh=_11_6230f63d14c5bcd29fde590ea0484c1e92f30a19e239b013e4d11dada2864f19";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_17&amp;ems_l=9039634&amp;_esuh=_11_3de5e2d3b1f3c212820af8a692d41c950eca7e40ccb580f15ecb73484731f6e6";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_19&amp;ems_l=9039634&amp;_esuh=_11_755128b48361651e5d24ff29c3176f141bf58d50b4c47b2c6c2b0be9c77e78eb";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4508_7367603_1_39&amp;ems_l=9039634&amp;_esuh=_11_c14c868149c5347674e7943201d4f4fbc2d401881a4a4f88da92082ce1296b2e"</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Ölpreise, Steueroasen und Schulpflicht</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>02 April 2026</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_17&amp;ems_l=9037890&amp;_esuh=_11_b3890978c99ca7f2ff80f5357d0ae25baacbc140a7161324330ae013586568cd";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_39&amp;ems_l=9037890&amp;_esuh=_11_86fb7c6986f32e3f675f6f341348b129a6736a3bcda049b7c5d340dc7b1075ae";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_35&amp;ems_l=9037890&amp;_esuh=_11_d3ae0b6c3090f1f0fd3d8ae9ce780799a0ef08ea2978007ccbbdf64b0089812b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_43&amp;ems_l=9037890&amp;_esuh=_11_f364257cba1f2a6905817935e9717055683442beabb3395cc44f4513db889912";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_31&amp;ems_l=9037890&amp;_esuh=_11_840f89b0e33df795d7498023945e6acaf6e4249d76aaa2a866c2d9a690ea5573";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_19&amp;ems_l=9037890&amp;_esuh=_11_2d7c4fc596748d8146c17721c2d94373479c08b8b4caef6b1957ab4d817dbda7";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_23&amp;ems_l=9037890&amp;_esuh=_11_e7681de371674a3d3eea6203df0b57cb7d10a34295afce21e7db32fafae9234c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1262_7366167_1_27&amp;ems_l=9037890&amp;_esuh=_11_dedbdacf338ad7deaebaa263121b2bc377175efc2396b1ac2d6781894a4c2ca5"</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Iran, Spritpreisbremse und digitale Übergriffe</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>01 April 2026</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_35&amp;ems_l=9035935&amp;_esuh=_11_69209c056db7e3c067a80c6e1fa5f04d3ed2f51e7723fed747719ff32e1c28b8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_27&amp;ems_l=9035935&amp;_esuh=_11_398fccffacbd57c57982c3ca3dbf3b086181c976f1c6b07ccc95c175b925da60";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_17&amp;ems_l=9035935&amp;_esuh=_11_d0310bce1101d0f8c859a29ddff906b96ed2d6ae26d2d3ad3ae96d69d2f58426";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_23&amp;ems_l=9035935&amp;_esuh=_11_898783c128cf34b5520319b58b7bcb8e97e5c1a68b6e4956169ed9e167961392";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_39&amp;ems_l=9035935&amp;_esuh=_11_a76712205082e65e131e27934e53f86ab5b40c39888300e44717dfe8753b2220";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_43&amp;ems_l=9035935&amp;_esuh=_11_87794c735990de965ee58d56067197eefddf42bf6b3dda3c15bcae2eb0133083";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_31&amp;ems_l=9035935&amp;_esuh=_11_336c0e9febedf2c23ab36c76e01c70a43c304120d13c3b9dbcd24c24c517f2a4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2780_7364323_1_19&amp;ems_l=9035935&amp;_esuh=_11_6137a4137581fbc648f5e6eac4c51ed3a2ea98ede9f9e197084831ffef307f11"</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Inflation, ORF-Spitzengehälter und El Niño</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>31.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_17&amp;ems_l=9034255&amp;_esuh=_11_9ea945b5b743f0b25ec377a35064ef117afd2f677089e5cbb049abf42aae936c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_27&amp;ems_l=9034255&amp;_esuh=_11_a15a2f5823747003c93763a5e5e798afe050416126d1b236cb23f329e31c51e2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_35&amp;ems_l=9034255&amp;_esuh=_11_eb94e87d99deaf70134d37fccee5ac414ce36dfbf2c4346c06956b1101256dcd";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_39&amp;ems_l=9034255&amp;_esuh=_11_8e4f0094a8c2789784333e88c3faff88e377b8351c718913ca9537b5c7d9995c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_23&amp;ems_l=9034255&amp;_esuh=_11_969ac63e772e3aa4a2d36fa71929c034a49dcc8f242dc8efa502c492467b46ec";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_19&amp;ems_l=9034255&amp;_esuh=_11_4004125c7943b6ceef3c7fabc18156fa56fcaa55466aee824830c0075391738b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_31&amp;ems_l=9034255&amp;_esuh=_11_afc999280d398f8cd5008575c4fd80475304cec53d14b7b4232d3fedd029e4d2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1995_7362748_1_43&amp;ems_l=9034255&amp;_esuh=_11_cc23545351698f06f111832e9d7b372fe3aaf31ccd5015fff3df9198d070b4e3"</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Irankrieg, Pilnacek-Buch und ISS-Notfall</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>30.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_19&amp;ems_l=9032819&amp;_esuh=_11_c4b5c135675cec9a50345e088fcacb95942876be763aeb089ab2ed68eb07284d";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_43&amp;ems_l=9032819&amp;_esuh=_11_4cfa8f513ffa668d511b32338bb0788006979f791744eeb9380a72ef22b0a418";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_27&amp;ems_l=9032819&amp;_esuh=_11_d6bfe00ec235d91a1edeb1baf6135c530afdfa9e178a18f6821f33ffc47de889";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_23&amp;ems_l=9032819&amp;_esuh=_11_2ae670fa6e91343af9fca1523be05be4531617a2d76a906d19cb61051130d8d4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_35&amp;ems_l=9032819&amp;_esuh=_11_d553f507b0621d01be81fdfa81b522a18ecf6975d8cffb62f3088a8aed24fe96";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_39&amp;ems_l=9032819&amp;_esuh=_11_2d546b358323644c8ac83b766a16e144ba8de275ae95d0626cc3aacb930627e2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_31&amp;ems_l=9032819&amp;_esuh=_11_a6dfb3fb77f5ed18bd0879b83f811d74435dfdfa9ebe02f23001e2cd0714cfac";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1454_7361165_1_17&amp;ems_l=9032819&amp;_esuh=_11_284f44784fc8c82dcc0502a155f5e3d89832c26b098a1504c41c7d22fc54cf80"</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Wöginger-Prozess, Social Media-Verbot und Hundemärchen</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>27.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_23&amp;ems_l=9028023&amp;_esuh=_11_d7e1336aa0c065e78fa9bfb3fcfbc7f78a48a8d80505ac298ae34cf0caf967da";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_17&amp;ems_l=9028023&amp;_esuh=_11_a85a5f38b109a4f432ad98e85a499ca57e12f4b54a8e81f83782e20451079e09";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_39&amp;ems_l=9028023&amp;_esuh=_11_a4da3a222f988db00b229f254d3e344474f88f9825315aac7ef8fa47d1801e3a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_35&amp;ems_l=9028023&amp;_esuh=_11_c3d1351d43f33281ddeee1f6c4c2e7c113d7103947498b2e0be38ac0c54084a6";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_27&amp;ems_l=9028023&amp;_esuh=_11_fbcc509c5c651e7a6d36b7477d3c942b425f83dabed5fce908e74d8085e2fbe6";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_31&amp;ems_l=9028023&amp;_esuh=_11_e90caf7bb246899b610020a270736a02363e19dcc4ee16331ccfea5351dc9087";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_19&amp;ems_l=9028023&amp;_esuh=_11_0671cfa43117ef813f598daefe48ea8019e0f9d773c5ade110e8390aceb1aa75";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_1814_7357057_1_43&amp;ems_l=9028023&amp;_esuh=_11_cc4e59c8bf5f40e9cb4fad560a8e6d14d4e15a2d1594ac370871907364ce59e4"</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Social-Media-Sucht, Goldmarkt und Ring-Radweg</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>26.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_43&amp;ems_l=9026324&amp;_esuh=_11_3ad78158740a0ec36b31bf8620cf7db53be1c0083273a27d2d8434c060a578c4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_39&amp;ems_l=9026324&amp;_esuh=_11_42f020d8743a81ed93720832949554d4c9902d9913e98e09332dd942eea120cc";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_19&amp;ems_l=9026324&amp;_esuh=_11_6f7f55531d18285cc52873465d4d991009339e4cb15083daa77c66b7d9eaa994";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_17&amp;ems_l=9026324&amp;_esuh=_11_64e497bd97a791ab63835d2ed1c3baf20722df84ddfb819d6093ca6403732a5b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_35&amp;ems_l=9026324&amp;_esuh=_11_90e54fbf19ae7028cdf26b9923900afa3d1b98941c2f82cd876d59950b08b41f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_27&amp;ems_l=9026324&amp;_esuh=_11_f0d2d2901b1b33be647ba923317d2be72e61e2cf140411beee1fae269409842a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_23&amp;ems_l=9026324&amp;_esuh=_11_50615ab85b052286c2f4aa1d671ed0343af4ef8d2f08bb70fbe74af71e8a202f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3963_7355519_1_31&amp;ems_l=9026324&amp;_esuh=_11_23a9d3871fb3d54f6b48b9914c5cee159e0a81721012314a3dee5803fcf187c3"</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Spritpreisbremse, Ungarn und OpenAI</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>25.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_17&amp;ems_l=9024639&amp;_esuh=_11_506c2729a792b76b9137a4a8e4c8dca15f7497e2a240e10970ce33346f921c6f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_31&amp;ems_l=9024639&amp;_esuh=_11_64ae9aa9c7aa877c92351ddd1bf449896a5a7995d239b5b458d64fc24d51d5b7";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_35&amp;ems_l=9024639&amp;_esuh=_11_24f2af7f27d1de22eb8c0ae034b738e386d8a89ea6e4160219b28aefbf7f5052";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_39&amp;ems_l=9024639&amp;_esuh=_11_d713fe3b8a0a20674c9fa5fce750d6f54f92185fd861243afb71b4e8aa7649a8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_19&amp;ems_l=9024639&amp;_esuh=_11_fb8633f7b37707902e97d7aebf92df00add33e264bbf8b0225ea680e04ea648f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_23&amp;ems_l=9024639&amp;_esuh=_11_98919b722271b98e7876d7054952f00301e67bb850f88a0674bab7b264690edf";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_27&amp;ems_l=9024639&amp;_esuh=_11_fa8af88d518e5d82a91d596276be2b5ac248beecb69b3baaa95fd5f51d4a242c";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_929_7353970_1_43&amp;ems_l=9024639&amp;_esuh=_11_b09294975c0bf1cab699163bdc09f182ccad6d4e6e63d2cbc0444840f50ad595"</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Wöginger-Prozess, ID Austria und Pottwale</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>24.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_19&amp;ems_l=9023233&amp;_esuh=_11_29e76c5b9c9aa68f3c3461a303b1dec78aff96e112923fe21197af8b0a4796a8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_39&amp;ems_l=9023233&amp;_esuh=_11_9767bf957b28a8ac965edc42d4dce4fce81d8b552fe4e1616ba74cd24f256d60";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_27&amp;ems_l=9023233&amp;_esuh=_11_bb36b5f428619d443ed16b44b1f308bac6e181526ec1fbc2cbd77f6a655d356f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_17&amp;ems_l=9023233&amp;_esuh=_11_a5ced5481297dfe4ddcf04b8ca98989fd1bedd9a1cf77abb524052f3838bc5e5";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_35&amp;ems_l=9023233&amp;_esuh=_11_d8c4eaa2be59f42665ff082bad62702690362e94fbc9cd1923ead24f6d96777e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_31&amp;ems_l=9023233&amp;_esuh=_11_918155d0c5dbbfa511afb2f6906bb658552de468b1aad358b585d5cf6a969902";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_23&amp;ems_l=9023233&amp;_esuh=_11_37c981ae50354573aa2c55e5e6fbed53a07a18fa3da12e5e1bc5e6dd09ea05a4";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3136_7352637_1_43&amp;ems_l=9023233&amp;_esuh=_11_5e14206f7e7538aaf47d35011c3c32bd8c1b926aa984be4e184fc0f394fab484"</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Erbschaftssteuer, Männer auf Social Media und neue Schule</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>23.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_43&amp;ems_l=9021706&amp;_esuh=_11_eaff23e84cc5cc31b2ac89ce290428d54a29484c3be8c5c991c007037a5bed05";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_39&amp;ems_l=9021706&amp;_esuh=_11_8a215dfe377a9a3a28ec7c2da7fe58d671e7e70da090e0acca66eebfb5f8821d";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_23&amp;ems_l=9021706&amp;_esuh=_11_c1b783e3d782242859f888c2a4bbd8f692e1ab1e54464846b4a678408147e2e2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_35&amp;ems_l=9021706&amp;_esuh=_11_f13c82cb94e4af527308493efe89a67de6e09b3b70b298a74dbbf79cd6d9fccf";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_31&amp;ems_l=9021706&amp;_esuh=_11_3a8293f72a8663c4af4ea3fccbc5c5dfc0456c204ae31eaa87c89a4eaf4faf4b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_27&amp;ems_l=9021706&amp;_esuh=_11_ddb4e9d4d37f098e6675e6042326955be7b0f496a16bdbca0aa1ebc893b3c062";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_19&amp;ems_l=9021706&amp;_esuh=_11_3c1c80fda97388e3b37854b75eaac07d527d8269b997f90d56962713ff312643";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_649_7351148_1_17&amp;ems_l=9021706&amp;_esuh=_11_2ec959c6cbd3ab71fe358d6361185508ec8f2e4eae4db2cee2f10bc73edb2257"</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Darknet, Cholesterin und Deepfake-Pornos</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>20.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_35&amp;ems_l=9016994&amp;_esuh=_11_3f3687e8a51ddd085f2f8a8146252c1b1c3053898c6c7be7365af89748c3c4de";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_43&amp;ems_l=9016994&amp;_esuh=_11_c38fd75dbbd5cf9e54b8a721c88e57a3958ca990b1d006c8c57577071d45eb8a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_39&amp;ems_l=9016994&amp;_esuh=_11_492d9f384081647a266ed64cc546ce5626058c61b1a541bdd7aa4b33707f8769";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_17&amp;ems_l=9016994&amp;_esuh=_11_7dc1f6fda74427d5c58cf49fcf44cdd31ce5f2c62232cf57b679dd1b8f494398";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_19&amp;ems_l=9016994&amp;_esuh=_11_04614d48a32bc349c84c6dc79f884dd19489b63d15d32dc960857c0bf8070e0e";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_31&amp;ems_l=9016994&amp;_esuh=_11_c048d3b46bf3c29f208739feb0713940a9406b888cfaece6d348a530deab5b29";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_27&amp;ems_l=9016994&amp;_esuh=_11_516484358a96074c65ccf1b0001db62b2f4c21eaa28c4af42ddac6aa97c1b594";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3573_7346909_1_23&amp;ems_l=9016994&amp;_esuh=_11_b1d7826e61475b8ef1b7178f62b2267e4260d76196d5335572e45c97d9c422be"</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Irankrieg, Wöginger Prozess und Vorwürfe gegen Christopher Seiler</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>19.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_17&amp;ems_l=9015313&amp;_esuh=_11_e180ef9b571383fbe3823f415ce8747801478de3071fe6c1d8289ae0287c4a1d";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_27&amp;ems_l=9015313&amp;_esuh=_11_6ed1cb20f7d64eec3f3f4f7a134a60f7d91918b209c801334b6b407fbc32c087";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_31&amp;ems_l=9015313&amp;_esuh=_11_ab6792858e91d19d906425982a8188926b85b7455b511dd10f94f4fb118d8921";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_43&amp;ems_l=9015313&amp;_esuh=_11_1604e77eb2590d1dff0260928653c014cf4324ba4e8d808949b206ffbda6c7f0";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_19&amp;ems_l=9015313&amp;_esuh=_11_dd40ce8242aab32f4d6a2e18c34533a56bcf1d0f233d69206fdf619d08617604";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_39&amp;ems_l=9015313&amp;_esuh=_11_c95452104be2c92042dbd3f51a90e31e16d98893de06d0f7654872659cbb8d13";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_23&amp;ems_l=9015313&amp;_esuh=_11_6046e20232e6673f461e5757a5b44380ef3cbe035d27db6e3eb41d35d196d4a6";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_2698_7345481_1_35&amp;ems_l=9015313&amp;_esuh=_11_6a9b14dfc48d8ac2f9f0afad6b9f066755a210ae5816098f23b172db4a13964e"</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Spritpreisbremse, Polizei und Moldau</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>18.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_39&amp;ems_l=9013615&amp;_esuh=_11_43a735705ed391a19b478c866545280692af88edfba285b1c480fab229c21541";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_43&amp;ems_l=9013615&amp;_esuh=_11_ab700ca272085edb4708a2ff822aae8de1b59ba05229e7e98cc14c8c9235531f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_19&amp;ems_l=9013615&amp;_esuh=_11_e001514ea791e53fc2fb9e7943968b7ecf7a3a3433818d9980377d66e77adf30";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_23&amp;ems_l=9013615&amp;_esuh=_11_6e0b934b61513fe7df79ffa530794df7395658410134744c0335b023ceabd462";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_27&amp;ems_l=9013615&amp;_esuh=_11_2c29773763abadde708a75cebbb75284a60dd09e74e8b2bd88956acb197176d1";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_31&amp;ems_l=9013615&amp;_esuh=_11_cbc55a46f3a21c216e91bcc1f4839273e3315470a98d3a550ee66a431dab89bb";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_17&amp;ems_l=9013615&amp;_esuh=_11_0f5e3eb2fb81b836635f4a295dae1a5901df07b90f4e3d477057f5c168ac9c4b";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4223_7343880_1_35&amp;ems_l=9013615&amp;_esuh=_11_6f6c4afdc7fbc1e2c8587b60e5d770cdc9e0f65625e4dd1e707d1ac0adcb5df7"</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Irankrieg, Fake-Bombendrohungen und Skispringen</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>17.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_17&amp;ems_l=9012008&amp;_esuh=_11_a8dadb61362f35f06fb863a6dea6be0831ddddee3c1b6d211ca1e7a8d3e67c93";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_27&amp;ems_l=9012008&amp;_esuh=_11_ae1e733f41e7be2088752cd05321d5e4f0ddbb6fcac54a30c34e300308241c9f";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_43&amp;ems_l=9012008&amp;_esuh=_11_6a7f92c7738841b42765869acd339afcaaa139a75f009673bafa13028b44e4bd";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_35&amp;ems_l=9012008&amp;_esuh=_11_a00fff471b2680bc588a0dcacd076927a0de24b648aeb24b156ba9ef8a227765";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_31&amp;ems_l=9012008&amp;_esuh=_11_9b0319357ffff37a01315e095f6b98ba4f386d2d1c63384c2e5084ca47fd0519";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_39&amp;ems_l=9012008&amp;_esuh=_11_b467a4ef711af972be8b3298da392f309bae2065fd441dd0bcd1fe6ded2e3b62";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_23&amp;ems_l=9012008&amp;_esuh=_11_379b729beb1ae52fb706b040833a7c18d66932a66e018ef293b74b8490f32dbb";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_834_7342369_1_19&amp;ems_l=9012008&amp;_esuh=_11_c4ee93222b0648e5d3971cddc7bb67e515ce6c01d9125c79043c7ffa1c6b7c84"</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Irankrieg, Banksy und Oscars</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>16.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_19&amp;ems_l=9010513&amp;_esuh=_11_cff012ec34da097f624f2aae4768bbc6e8899fb951769c4b0248ad57b09d28e0";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_39&amp;ems_l=9010513&amp;_esuh=_11_d5844c60c4d9069ff0fc85f0dd678480427f8d82d54a34615ca9638d772cbfde";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_31&amp;ems_l=9010513&amp;_esuh=_11_beb09554c3ae2835c5a7f5221eed344ac7e709a80e6f93778f8b10f2e882971d";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_43&amp;ems_l=9010513&amp;_esuh=_11_a580e1e6f493b0e3b47dab7cdc67fb4f0ed68d42c8a0de3c125f17cf17071cef";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_35&amp;ems_l=9010513&amp;_esuh=_11_0172c2f7e99c53c32dea0da3f5cfb0b5c0ede70778fc9ccf0bc4602e47238e4d";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_27&amp;ems_l=9010513&amp;_esuh=_11_aea24a5deaa3fe1c732ea48618cd9785f167dd52e3c527dcd75d23cc568790e1";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_17&amp;ems_l=9010513&amp;_esuh=_11_43422539f126e63b13a560db98cf857d61bdabeec4d28245b879fe307983296a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_3477_7340887_1_23&amp;ems_l=9010513&amp;_esuh=_11_12f0a7b87671a323ac25cfcac303400676e1a50735f6d1880d42e52a5ff7dd6d"</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>DER STANDARD - Daily</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Iran, Gletscher und Pornosucht</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>13.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_31&amp;ems_l=9006246&amp;_esuh=_11_48aef7e7535fa7be02383e2eca3d7b1aa69d9ebe601533a8147421949ab92088";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_43&amp;ems_l=9006246&amp;_esuh=_11_58c71893337f36cd09adfccb2481004a38c911f05fc4b681b5a19833da456bd8";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_19&amp;ems_l=9006246&amp;_esuh=_11_279e3f9f76200fa64528f0c2cd75a925bdd362423906361328edae0afbd01f16";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_39&amp;ems_l=9006246&amp;_esuh=_11_f7088868799fa752cb8f2e9653415e86e37c089055e4e115508ce2604b649fb2";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_17&amp;ems_l=9006246&amp;_esuh=_11_4aa83ad270ac841201755cefa4aafe95ab40da1ad9c7a45e68303efdfb37f41a";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_23&amp;ems_l=9006246&amp;_esuh=_11_0826ace0426bb4b29c266c4e79923fb163baa72307b5a3269679ea9686e8f601";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_35&amp;ems_l=9006246&amp;_esuh=_11_91c2b1e8486a0c38bf545523a23cebbcafd57cc470124816454eaac02e7ede57";"https://click.dst.at/u/nrd.php?p=yk3W5wVgNt_4446_7337237_1_27&amp;ems_l=9006246&amp;_esuh=_11_ec845ecb06cb8d7ec80d9937d19283db68ca501ebfc6e8cf52b31737fe124ea5"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Developed and tested link filtering+extraction heute
</commit_message>
<xml_diff>
--- a/research_data.xlsx
+++ b/research_data.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:E142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.77734375" customWidth="1" min="1" max="1"/>
@@ -2592,6 +2592,996 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Supermarkt knallhart! SB-Kassen nicht mehr für alle</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>25 April 2026</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=926dd90caf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d43f075618&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3658d15e21&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2ccc701661&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=de281ad520&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0e47ab6b82&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7c42bac479&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=df8dcef42e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a911874663&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2a817b3612&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>98 Prozent blind! Trotzdem schickt PVA Serafin arbeiten</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>24 April 2026</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=734ee0e6dc&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c96b61b525&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=750d911e9e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=99bdb0d3ed&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=de0f44c757&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7625b7723d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=21b4f40e82&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c3bb7c4992&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a7d7a876e8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3bf1f7be30&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Neuer Spar-Hammer: Jetzt kommt ein "Trump-Budget"</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>22 April 2026</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4b10baa2d1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0b3e59c1d1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c0481d8685&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=18844cd01a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3471042830&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=feb2204349&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b8f69955b1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5db0fe1d94&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=90831235dd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bc29a82d69&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Mehr Geld für alle – jetzt kommt neue Zusatzpension</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>22 April 2026</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=82f0c3062f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9970b4f2ad&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ff6b0df5f9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1095d1526b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8bca2014c0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=345d15dc3c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=461937c6f9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ef0cfcef70&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=dc3b38ce81&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=26972f293f&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Kopftuch, Scharia – "Staat muss klare Grenzen setzen"</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bd2724f3b1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=aca5d3af38&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=854de5d028&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ecd57253fd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2c28e01eac&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f6d8dfd41a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d7d1d1a86d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=44167b602d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=67f26dc440&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a77985c0ee&amp;e=494d210687</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Rattengift in Babynahrung – nun Suche nach zweitem Glas</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b6781cbb3c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=400c8d9023&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1b75ef87e1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=33907e6a86&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=30b43a1907&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0b01be6d12&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ef9c97ac1b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1b0c2035cf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=be319d09f2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=db0ade7bd7&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Erstes vergiftetes HiPP-Gläschen in Österreich entdeckt</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>19 April 2026</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=78d03cd266&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=74e7d2ffe7&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7f7f8e0a7b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=01f5aac671&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=81d3b3e0cd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9f185e15b9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=61fdd95568&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=be98c13e5f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=379cba39d6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d0de11aa8e&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Junger TV-Star verprügelt Polizisten im Wiener Prater</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>18 April 2026</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0ca496b6f0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9d8cbae326&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2242718860&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7264548cae&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9dedfd0829&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fb8eb2c073&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=50b5e110f7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6139312fed&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c95ae4ea38&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=102a95e208&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Wienerin bricht Medizin-Studium ab, wird Influencerin</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>17 April 2026</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9ceb4c9b74&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fcd00459dd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2cbfb2d452&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9a4de0ca7f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ce94acd171&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ec9badd4b2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=845f79947d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bdebe863e2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f2a15f69e9&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=497febeed5&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>"Massiver Druck", Anzeige – Ex-ORF-Chef erzählt alles</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>16 April 2026</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ac24b83484&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=00a7fcae8f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7269e2945e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=09f86784f4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=00f9147d1d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1f2edb590a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a078bf06b9&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=91beda6da3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e654e5f81f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d191e4137b&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>"Stehe vor dem Nichts" – Böller zerstörte Annas Wohnung</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=11a1b301de&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c474225deb&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ec3cbbe557&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6b323145b8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=65bbe1e62c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1974736635&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6efea35aff&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fb8b5c5073&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9c488c0e45&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5b81173f67&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Nicht in Deutschkurs: 5.000 € Strafe oder 3 Wochen Häfn</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14 April 2026</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e433a835dc&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=dfcdde93c0&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=59b2248881&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0173c94031&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=872f9402ea&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0cf6f1f706&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=738bd71eca&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0affd791ec&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6842b119e4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=221ff4ad03&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Justizwache-Beamtin war heimlich auf Porno-Plattform</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>13 April 2026</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f6527570af&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=96a177c0b9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ceb09176cf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=29f47453f4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d564cecc70&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=52bd1383ba&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fa27c5daaf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b30a90ead0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8f02c8ec00&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=79976c04ff&amp;e=494d210687</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Autoverkauf wird Albtraum – Wiener verliert vor Gericht</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>12 April 2026</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b4c127f8b7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4356acad95&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=82ceff2cbf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8c63f5f18b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d7066effe8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=59068ca153&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=27e47ebbca&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e6a2e486de&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=978a1106c9&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8bd8386b39&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>"Sind Tiroler" – Geschwister kämpfen gegen Abschiebung</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>11 April 2026</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e6c9dac150&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fe05995443&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=22e6e9bb30&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=05a578fe7a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9c2891d7f6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=18fecee83c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e8e88dc9b0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6ded7cd5ad&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6ae28d2224&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5deaaa3189&amp;e=494d210687</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>"Tut total weh" – für PVA aber nur "leichte Schmerzen"</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>10 April 2026</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c2e7db705a&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=92d35b8bfe&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3d89c9290b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d4bcebca24&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b755ec41a3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=db145fec0b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bdda594178&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d2677aed6a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=50af67e9f8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4fa5dd105d&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Kein Spital konnte helfen – AKH rettet Oberösterreicher</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>09 April 2026</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0336cc4f01&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5c77d1840f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=be487f0b6a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cd180086bf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fdc1419bf6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=48ec5d8b63&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5c9cfd4541&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2fcfdcbfd1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f76c327f2c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bd2c67c1c9&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>USA und Iran verkünden zweiwöchige Feuerpause</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>08 April 2026</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3b2d3c0e65&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5dad384de5&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=95c223bf38&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d007dd876d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d5f6ad8ee3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e6060977d7&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4f60be5712&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=52fd6d8e8b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e2c53636a8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=be6c70c4a2&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Preisschock: Sechs Stunden arbeiten für 50 Liter Diesel</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>07 April 2026</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bfecc0e07b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=01e4c93c1d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d726546346&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b0fda8a7b0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5df87bc1c7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1d988644cd&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7b0281e8fa&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=af4f8edf7b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e68da673e0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=07acfaa950&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Video! Mega-Ansturm auf Tichy-Eis am Ostersonntag</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>06 April 2026</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6bb9045b42&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=34021c8eba&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f5a4d7fe9d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=409597c77e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9d045c34e4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2011561f48&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a717f1cc40&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8e038c6450&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=da190b5bf1&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a3bedc5f41&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Wienerin verkauft Audi – SIE soll jetzt 28.000 € zahlen</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>05 April 2026</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1f6a191671&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7d64830a0b&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=76381accd3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=016b7421d5&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e65f6e6ce6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a568894c56&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7385fceceb&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=80fce265dd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9cb8d478a1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b1c4771747&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Kanzler Stocker nennt Kickl "völlig verantwortungslos"</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>04 April 2026</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=777e6e6312&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9ad01de17b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=228c95cd59&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9521b02512&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=19e7c094a7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=96b62ac6f0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2a0e198296&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1775cd1e2c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ec90ee1496&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1a5e1c7391&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>"6 € haben oder nicht haben – das ist nicht zum Lachen"</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>02 April 2026</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e1c598c23e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=033ba2c908&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6d642e9f72&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e88b067a7f&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=94de52b4ef&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9cbbc38351&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=41605dd60d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2a87b6a043&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=48a7d658fa&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=326ff90bf8&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Öffi-Essverbot – Securitys mussten 1.200 Mal eingreifen</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>02 April 2026</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a904ec8266&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8be348bd31&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=00aeea82ba&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9d82e9c01b&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=07d6c49e45&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f870a31e34&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=03d88b6043&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cd8fd76038&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6c3fa49842&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4f413735c6&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Die Gagen-Kaiser im ORF – jetzt kommt alles ans Licht</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>01 April 2026</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4363bf3167&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d4fc51fedf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=01c36e52b0&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0f728b9e6a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3840f6d67c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d6d5b29ca0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ab7db24c4e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cbff753568&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=32b1f2cd3a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=64d152e415&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Neuer ORF-Gagenkaiser casht mehr als Bundespräsident</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>31.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0b2e5f687d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=813702afd7&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=72c7fb2394&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1b71f30fa0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3db42e7ee8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d7df0370c9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=dc5d14f8fd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f05504748e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3077f4af61&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8edfefdbb2&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>"Wegen Ölkrise" – Taxler verlangt dreifachen Fahrpreis</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>30.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=98e12a0d56&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2073220835&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c4612eef19&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e1f9b77dc9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=73a7889224&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=70e615423e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=edca770b65&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a8265e96c0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9f1499b9ce&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5220308642&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Ex-ORF-Moderator soll 13-Jährige vergewaltigt haben</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>29.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a16e884b5a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1ea1147a41&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=122c11826e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a0d64a1c10&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7270f7f2f4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=aec29105b3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2567c5e37c&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5e4c79e995&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b8f98c591f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=be18f690f5&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Geheime Zahlen: Wo Kickl abräumt, wer ÖVP stabil hält</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>28.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3a683f221c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bd7efaf044&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=47a545aea3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=03c5fd63ea&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cd9ce5929f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=66dee83028&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=17260db95d&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=db0c674ddb&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b925a85993&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2826d52a9d&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Neue "Heute"-Umfrage ändert für Kickl-FPÖ alles</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>27.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ab392de9f2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=233f52143a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=800de8db29&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=383e8dc0e3&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bb5c4ff49c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b7c2438e02&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e2a01d4a4c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=721c5dbf91&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=94bd904dfe&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a206c115e1&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Neue Sprit-Regel gilt für alle Autofahrer in Österreich</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>26.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d5c0188419&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1d6ad82757&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=80045d112b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=43ee3080b9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3efdc15646&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d996834464&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5b7e71d46b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9bef71a94d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ff901c4f17&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0d17907c0b&amp;e=494d210687</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Tank-Tsunami sorgt für neuen Ärger in Österreich</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>25.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6992a6f849&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=90d3914e0c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bb97b30a03&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4a9451e52a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=94defba9cf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=16ee8eb492&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=3a038c8ac1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d5852bd64c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1ae4174ffd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9a71ad2599&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Geräte defekt – Wienerin klagt Vermieter auf 10.000 €</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>24.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b27288cffc&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7f13c3510e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b112d7dfdb&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1cdc5dd7c4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=83ab9de3bf&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=34754f0f44&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9780cf0354&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f7d8c7bc16&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9d49dd4745&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2499099083&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Doskozil: "CO2-Steuer aussetzen!" ++ Streit um 10-Cent-Spritplan der Regierung ++ Neue Regeln für China-Shop Temu</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>23.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f620f8819a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5c5087ba60&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a5409b1e84&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7a4bbca7df&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ab3c2dd56f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=10fb33c8f0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bdb1e73dfb&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5a384c0eab&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=afbacf0889&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=886624d10f&amp;e=494d210687</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Doskozil: "CO2-Steuer aussetzen!" ++ Unternehmer erfindet eigene Spritpreis-Bremse ++ Neue Regeln für China-Shop Temu</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>23.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e3bfa2f772&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0f0548626b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b8b54450f2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1e0022b93c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e79cbd7306&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=269bd992de&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b992e81031&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a18f7103f6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c47750f436&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=dc0da627c3&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Doskozil: "Der ORF-Sumpf gehört trockengelegt" ++ Trump stellt Iran ein Ultimatum</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>22.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c86af1f967&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a35b906d23&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=196bdf271e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ad593e3075&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=dbc96ce62c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=17f02e339e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5a135e9945&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d8ac6d01d5&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=26f520b6cf&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Kickl zerlegt Spritgesetz, bringt eigenes Modell ein ++ Diesel-Irrsinn! Plötzlich kostet er nur 1,20 Euro</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>21.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f107f516d6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=077dc601a2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=63f2f58238&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=24c594fb29&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=700b1ee681&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=56da403a79&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bf833540f2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=11a5129ebc&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=1f92d512ac&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5a3b76bb0b&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Auto-Pickerl Neu: Was sich ändert, ab wann Reform gilt</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>20.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c305b73737&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4b2832a331&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d72656dc78&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5c71e4ebde&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=616464903b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=265d74cbe4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f07a3fc01e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5de7dbf338&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4e3bfb7233&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cc62245781&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>"Müssen uns gegen die Islamisierung im Land wehren"</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>19.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7327503ba9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=93c10432fe&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bc53e3447b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7c181dc17c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bb91bf2f10&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=9502c2acc7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6f93fe47e9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=ec66333ed9&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=abc0853d4e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=93b7f90537&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Seiler: "Ich habe ihr Kokain auf die Lippen geschmiert"</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>18.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6c37c03030&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a030176f01&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cc1a38cdf7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8b6e872e72&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=db7625fbe0&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5fcc614c73&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=03013d89d2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c07a210a4e&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d8ab2f506d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=dedb39b9b6&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Krieg, Blackout, Katastrophen – jetzt Warnung an alle</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>17.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5b4a5651b6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=74e016301b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cacf4e9319&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=d347db0e59&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e737708761&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8f221e55ec&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=29156f616f&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a8c1760c4d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fdc2e4fb2c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=91cc3a8ecc&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Kickl auf Platz 1 – aber Stocker ist ihm auf den Fersen</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>16.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=f6a9a443f1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=a7a8627ce7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=66e5893313&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fdddeb4347&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=918ce067dd&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=52e44daca8&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=98ff9836cc&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=662daca294&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=c77ec8a671&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fd1148a6ec&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Braucht der ORF wirklich eine Milliarde Euro jährlich?</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>15.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=49913a82f4&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4de7daa933&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0fc0337c09&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e293fdb620&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0c5a12977d&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0a738cfd34&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=4cc5ef8426&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fe114db49f&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=e39b221c3a&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=8b89df5569&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Eis-Chefin verrät: "Das ist unsere beliebteste Sorte!"</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>14.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0a4760690b&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=7147f26c53&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=aaa2cdfdc8&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b70a1c0dad&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5e58b23bfb&amp;e=494d210687;"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=2100440897&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=bd1714e5c6&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=abb5e774b7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=cc864a6d16&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=fa57d2da2c&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Heute.at-Newsletter</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Millionen nach Autodeals weg – MMA-Kämpfer im Visier</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>13.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=611d8affa1&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=6048029547&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=293a59e28c&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=616342d287&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=35c5ca0979&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=08f2bd6fac&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=0fe98649de&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=37025e46d2&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=5b15a956d7&amp;e=494d210687";"https://heute.us15.list-manage.com/track/click?u=e85da083a4e95214379d07dd8&amp;id=b1a8bdfd42&amp;e=494d210687"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Developed and tested link filtering+extraction blikk
</commit_message>
<xml_diff>
--- a/research_data.xlsx
+++ b/research_data.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.77734375" customWidth="1" min="1" max="1"/>
@@ -3582,6 +3582,666 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Tönkrement a házassága a TV2 híradósának</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>24 April 2026</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvZ2Vkby1neW9yZ3ktYmV0ZWdzZWcvZjB2MngyeT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTI0/69b31bd04d2f0e8d990b13ddC8308890a";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3N6ZW50cGV0ZXJpLWVzenRlci12YWxhcy1tZWx5cG9udC1rdXpkZWxlbS9xcmM1NWsxP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjQ/69b31bd04d2f0e8d990b13ddC5885ccfc";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3N6aWpqYXJ0by1wZXRlci1iZXRlZ3NlZ2UvZnRxcXcyZT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTI0/69b31bd04d2f0e8d990b13ddC9412ff3a";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hlcmNlZy1lcmlrYS1tZWdhc3p0YXItenN1cml0YWctbWVzdGVyLWJlamVsZW50ZXMvZ3luZHljeT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTI0/69b31bd04d2f0e8d990b13ddBff9c613d";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2lkb2tvemktdmFsYXN6dGFzLXZhcy12YXJtZWd5ZS1zYXJ2YXItc3Ryb21wb3ZhLXZpa3RvcmlhLW1hZ3lhci1wZXRlci9zYmhyZzN3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjQ/69b31bd04d2f0e8d990b13ddB87685b63";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3N6ZW50cGV0ZXJpLWVzenRlci12YWxhcy1tZWx5cG9udC1rdXpkZWxlbS9xcmM1NWsxP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjQ/69b31bd04d2f0e8d990b13ddD5885ccfc";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvbWFuLXN6YWJpbmEtdmFsbG9tYXNhL2JyeDMwazc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yNA/69b31bd04d2f0e8d990b13ddB5a6df772";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3gtZmFrdG9yLW1lbnRvcm9rLTIwMjUtc29sZXJlLWJ5ZWFsZXgvdDB6aG5xOD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTI0/69b31bd04d2f0e8d990b13ddCf0e8f5d5";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90aXN6YXVnLWVsdHVuZXMtaGF6YXRlcmVzLWJlbmNlLXRlbGVmb24vNjFobnJ6Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTI0/69b31bd04d2f0e8d990b13ddBdde08e27";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90aXN6YXVnLWVsdHVuZXMtaGF6YXRlcmVzLWJlbmNlLXRlbGVmb24vNjFobnJ6Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTI0/69b31bd04d2f0e8d990b13ddDdde08e27";"https://link.blikk.hu/click/45365694.12966/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2EtbWkta2lzLWZhbHVuay1wYWprYXN6ZWctcGlsaXNzemVudGxlbGVrLWtvbHRvemVzLzVyMzhxODA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yNA/69b31bd04d2f0e8d990b13ddBd9d3c024"</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Kómába esett a fogműtétje után a családapa</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>23 April 2026</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvdGVzY28tYnVkYXBlc3QtYmV6YXJhc2EtYXByaWxpcy12ZWdlbi93eTVkNTlrP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjM/69b31bd04d2f0e8d990b13ddC01565767";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9tb2wtYmFyYXRzYWcta29vbGFqdmV6ZXRlay11anJhaW5kaXRhcy1iZWplbGVudGVzLXN6YWxsaXRhcy9ranpuYmZ4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjM/69b31bd04d2f0e8d990b13ddB8bb36a30";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9tb2wtYmFyYXRzYWcta29vbGFqdmV6ZXRlay11anJhaW5kaXRhcy1iZWplbGVudGVzLXN6YWxsaXRhcy9ranpuYmZ4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjM/69b31bd04d2f0e8d990b13ddD8bb36a30";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3N1dGktYW5kcmFzLWJhbGVzZXQvbDVsNDl6OD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddC09df8e47";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9rb21hLWZlbGJyZWRlcy1pZGVnZW4tbnllbHYvemY2eGplOD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddB9ee076cf";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hhbGFzei1qYXptaW4tdmFka2VydGktYWRlbC1wYXJiYWovNTJwZnM0OD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddDca534681";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hhbGFzei1qYXptaW4tdmFka2VydGktYWRlbC1wYXJiYWovNTJwZnM0OD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddCca534681";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dhc3Bhci1ldmVsaW4tbWVnc3pvbGFsdC9zeHFrZTY1P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjM/69b31bd04d2f0e8d990b13ddC8babbffd";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvYmxpa2stdHYvc3pvcmFrb3pvaGVseS1iZWRyb2dvemFzL3czZDc3ZnI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMw/69b31bd04d2f0e8d990b13ddB85b3c655";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3NhcmtvemktYWtvcy1yYWN6LWplbm8tZXR0ZXJtZWstY3NhdGFqYS1nYXN6dHJvLXNob3cvODZ2Ymx5cj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddC1bca364c";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90dXotaXZhbmNzYS1ha2t1bXVsYXRvcmd5YXItcmVhZ2FsYXMtbmFneS1lcnZpbi82OTRjZWdrP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjM/69b31bd04d2f0e8d990b13ddC02afadd1";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9rb21hLWZlbGJyZWRlcy1pZGVnZW4tbnllbHYvemY2eGplOD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddD9ee076cf";"https://link.blikk.hu/click/45335437.12534/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2VrbGVyLWx1Y2EtZXhhdGxvbi1odW5nYXJ5LXZlcmVzZWcvcDQwOGtzaD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIz/69b31bd04d2f0e8d990b13ddBc738cbfd"</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Tóth Gabi és Tóth Vera testvérháborúja</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>21 April 2026</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3N1bHlvay10YW1hcy1vc3N6ZWhpdnRhLWF6LW9yc3phZ2d5dWxlcy1hbGFrdWxvLXVsZXNldC83NGVkNDBwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjI/69b31bd04d2f0e8d990b13ddB1e3315fc";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9iYWxvZy1sZXZlbnRlLWZlbnllZ2V0ZXMtZXJkZWx5LWVsb2FkYXMtY3NhbG9kYXMvenpyZHBuaz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIy/69b31bd04d2f0e8d990b13ddCd8938e06";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvdGgtdmVyYS10b3RoLWdhYmktdmVzemVrZWRlcy9xZTNsY3MwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjI/69b31bd04d2f0e8d990b13ddDda822d7f";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3N1bHlvay10YW1hcy1vc3N6ZWhpdnRhLWF6LW9yc3phZ2d5dWxlcy1hbGFrdWxvLXVsZXNldC83NGVkNDBwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjI/69b31bd04d2f0e8d990b13ddD1e3315fc";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9iYWxhdG9uLWhldml6aS1raWZvbHlvLXRyb3B1c2ktbm92ZW55L2p0emRuanI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMg/69b31bd04d2f0e8d990b13ddB7bc85605";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9zemV4dWFsaXMtYWJ1enVzL2gybDJqNXI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMg/69b31bd04d2f0e8d990b13ddC4008e610";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvdGgtdmVyYS10b3RoLWdhYmktdmVzemVrZWRlcy9xZTNsY3MwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjI/69b31bd04d2f0e8d990b13ddCda822d7f";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvdmlsYWdwb2xpdGlrYS9vbGFqLWRvbmFsZC10cnVtcC1wYW5pay8yOHYzMWxuP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjI/69b31bd04d2f0e8d990b13ddC5b7816b5";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hhdmFzLWhlbnJpay1oZXRpLWhldGVzLWtyaXRpa2EtcnRsLzZ5ZzJtZnE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMg/69b31bd04d2f0e8d990b13ddBac4ba213";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvdmlsYWdwb2xpdGlrYS9kcm9uLXVrcmFuLWJhcmF0c2FnLWtvb2xhai12ZXpldGVrL2N3azhudjc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMg/69b31bd04d2f0e8d990b13ddBc95b6698";"https://link.blikk.hu/click/45319596.10051/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay90ZWNoL29rb3N0ZWxlZm9uLTIwMjYtcHJvYmxlbWFrLXRhcmhlbHktYWxrYWxtYXphcy80bjdleDBkP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjI/69b31bd04d2f0e8d990b13ddB3b92c7f9"</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Mihez kezd Gáspár Evelin a kormányváltás után? Megnéztük, milyen területeken van tapasztalata</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>21 April 2026</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZWx0dW50LWd5ZXJlay1hcGEta2lza3VuaGFsYXMvOTlqMjRuMD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIx/69b31bd04d2f0e8d990b13ddD2ba88420";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9rZXJvemluaGlhbnktcmVwdWxvLW55YXJhbGFzLXV0YXphcy9jdjkwZzZxP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjE/69b31bd04d2f0e8d990b13ddB2c44cf68";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL29zenRlci1hbGV4YW5kcmEtZmlhL3QxMHpoM2w_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMQ/69b31bd04d2f0e8d990b13ddC6cf6485c";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3VqLWtvcm1hbnktYWxha3VsYXMtb3JzemFnZ3l1bGVzLXRpc3phLXBhcnQtbWFneWFyLXBldGVyLXVqYWJiLW1pbmlzenRlcmVrL2xwMjN0dHg_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMQ/69b31bd04d2f0e8d990b13ddBb720edd3";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dhc3Bhci1ldmVsaW4ta29ybWFueXZhbHRhcy12YWxhc3p0YXMtMjAyNi85eXkycTJ2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjE/69b31bd04d2f0e8d990b13ddCb4c01419";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9pbnRlbGxpZ2VuY2lhLWlxLWJlc3plZC1wc3ppY2hvbG9ndXMvajUyMXA4dD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIx/69b31bd04d2f0e8d990b13ddC147f78c4";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3phbWJvLWppbW15LXphbWJvLWFycHktaGFqb2themFzLWVsZXR2ZXN6ZWx5L3N3MWQ5OWQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMQ/69b31bd04d2f0e8d990b13ddC808c2185";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZWx0dW50LWd5ZXJlay1hcGEta2lza3VuaGFsYXMvOTlqMjRuMD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIx/69b31bd04d2f0e8d990b13ddB2ba88420";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3VqLWtvcm1hbnktYWxha3VsYXMtb3JzemFnZ3l1bGVzLXRpc3phLXBhcnQtbWFneWFyLXBldGVyLXVqYWJiLW1pbmlzenRlcmVrL2xwMjN0dHg_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMQ/69b31bd04d2f0e8d990b13ddDb720edd3";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21hcm9zaGVneWktYWxmcmVkLXN6YXJ2YXMtam96c2VmLWpvc2gtam9nZGlqLzg4MTdyNm0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMQ/69b31bd04d2f0e8d990b13ddC59fdf0f8";"https://link.blikk.hu/click/45290883.8355/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2FsZXJpYS9sZXp1aGFudC1iZWxncmFkLXJha3BhcnQta2F0YXN6dHJvZmF2ZWRlbGVtLW1lbnRvay10dXpvbHRvay1tZWdzZXJ1bHQvbTI5cndzNT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIx/69b31bd04d2f0e8d990b13ddC539e22c9"</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Kiborult a bili: egymásnak esnek a sztárok és a politikusok​</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>20 April 2026</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21hamthLXJha2F5LXBoaWxpcC1rb2NzaXMtbWF0ZS9mcGV4ejIyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjA/69b31bd04d2f0e8d990b13ddCf0bbb59b";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hhemFrb2x0b3plcy1rdWxmb2xkcm9sLXN6dGFyb2svcWMya3M5Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIw/69b31bd04d2f0e8d990b13ddBb4f8bf73";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JhbmdvLW1hcmdpdC1lbWlsaW8tdGluYS1iZXRlZ3NlZy1sYWJhZG96YXMveTh6eHB2Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIw/69b31bd04d2f0e8d990b13ddDee79e910";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2plc3plbnN6a3ktenNvbHQtb3JiYW4tdmlrdG9yLXZhbGFzenRhcy12ZXJlc2VnLXN6ZWxsZW1lay9neDlkcDFwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjA/69b31bd04d2f0e8d990b13ddB7d9886c1";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9rdXR5YS1lbGV0bWVudG8tcmVmbGVrdG9yLWF1dG8tYWp1bHQvMzF5ZHJneT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIw/69b31bd04d2f0e8d990b13ddBa0ac3496";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JhbmdvLW1hcmdpdC1lbWlsaW8tdGluYS1iZXRlZ3NlZy1sYWJhZG96YXMveTh6eHB2Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIw/69b31bd04d2f0e8d990b13ddBee79e910";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9vbmtvcm1hbnl6YXRvay12YXJtZWd5ZWstZm9pc3Bhbm9rL3g3bTFkeXo_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMA/69b31bd04d2f0e8d990b13ddC38ac4231";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2FsZXJpYS9wZWtpbmctZS10b3duLXJvYm90LWZlbG1hcmF0b24tcmVrb3JkL3Q5Z3BqMnc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMA/69b31bd04d2f0e8d990b13ddB68f685a4";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9lcnN0ZS1iYW5rLWplbGFzaXR5LXJhZG92YW4tbWVnc3pvbGFsdC1vcmJhbi12aWt0b3ItdmFsYXN6dGFzL2tjOHJxOTQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMA/69b31bd04d2f0e8d990b13ddC245bfd38";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9waWxpc2ktZW1iZXJvbGVzLXN6ZXJlcGphdGVrLXN6b2xvLXV0Y2EtaWdhemdhdG8vNXZmMm1tcD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIw/69b31bd04d2f0e8d990b13ddC7c2eb20f";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JvcmJhcy1tYXJjc2ktYXJ1bGFzLWtvY3Npcy1tYXRlLXZhbGFzenRhcy83YjdkY3c1P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMjA/69b31bd04d2f0e8d990b13ddC83e694c8";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9vcnN6YWdneXVsZXNpLXZhbGFzenRhcy0yMDI2LXBsYWthdC1sZXN6ZWRlcy1hcmFrLzJ2cmw4dG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0yMA/69b31bd04d2f0e8d990b13ddC1b04687a";"https://link.blikk.hu/click/45277506.3674/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2JhbG9naC1sZXZlbnRlLXN6ZW50a2lyYWx5aS1hc3Zhbnl2aXota29jc2lzLW1hdGUtZmlkZXN6LXZhbGFzenRhczIwMjYvM2d3NzUxbT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTIw/69b31bd04d2f0e8d990b13ddB4a4e2d5e"</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>A Mol-vezérrel tárgyalt Magyar Péter, megtartja a védett üzemanyagárat a Tisza​</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>17 April 2026</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9tYWd5YXItcGV0ZXItdmVkZXR0LWFyLWJlamVsZW50ZXMvaHI0d2gzbD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddE155e27e8";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9tYWd5YXItcGV0ZXItdmVkZXR0LWFyLWJlamVsZW50ZXMvaHI0d2gzbD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddC155e27e8";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21hamthLXBhcGFpLWpvY2ktYmFyYXRzYWctcG9saXRpa2EvcWIwaHByND91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddDf2d231db";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvYXV0by9rcmVzei1zdG9wdGFibGEtc3phYmFseS9reHR0OHl2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTc/69b31bd04d2f0e8d990b13ddB6ba0d923";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21hamthLXBhcGFpLWpvY2ktYmFyYXRzYWctcG9saXRpa2EvcWIwaHByND91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddBf2d231db";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9nb2QtYWtrdW11bGF0b3JneWFyLW1lcmdlemVzZWsvYnFqcXd5cD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddCb5d75758";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2FudGFsLWltcmUtcGlyb3NrYS12ZW5kZWdsby1lbWxla2V6ZXMvd2tld2d6Mz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddB4f2f1c33";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9tYWd5YXItcGV0ZXItbW9sLXJlc3p2ZW55cGlhYy1hcmZvbHlhbS90bmNmeGI5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTc/69b31bd04d2f0e8d990b13ddBeea7403d";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3JvbmFpLWVnb24tYWktaGFtaXMtdmlkZW8vMWUzcnhwZj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddBf0c1c18e";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9maWt0aXYtZm9nbGFsa296dGF0YXMtcG9sZ2FybWVzdGVyLWhhbGFzenRlbGVrL2s0YmIxd2Y_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNw/69b31bd04d2f0e8d990b13ddC5d8bc3f8";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci1maWRlc3otdmFsYXN6dGFzLXBhdHJpb3RhLWludGVyanUvbWtocDNkMT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE3/69b31bd04d2f0e8d990b13ddC95614c96";"https://link.blikk.hu/click/45250255.10350/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9lbGV0bWVudGVzLWJhbGVzZXQtdHVya2V2ZS1rZXJla3Bhcm9zL21jbGtwaGI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNw/69b31bd04d2f0e8d990b13ddB7f9caf48"</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Kudlik Júliát akarta menyének Antal Imre édesanyja</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>16 April 2026</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2d1bHlhcy1nZXJnZWx5LW9yYmFuLXZpa3Rvci1taW5pc3p0ZXJlbG5vay12YWxhc3p0YXMtdmVyZXNlZy9yejJqOTZ5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTY/69b31bd04d2f0e8d990b13ddBf864926a";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dlc3p0ZXNpLWthcm9seS1zenVsaW5hcC1nYWxhbWJvcy1sYWpvcy8ycmZtaGN4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTY/69b31bd04d2f0e8d990b13ddBc2a78112";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9rdXR5YWstbWVndGFtYWR0YWstbmFneWtvdmFjc2ktcG9sZ2FybWVzdGVyL2ZjNmU4MjE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNg/69b31bd04d2f0e8d990b13ddC58c12266";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3JhZGljcy1naWdpLWVza3V2by1zemVyZWxlbS93M3c1Y2g2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTY/69b31bd04d2f0e8d990b13ddC198bc335";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9zenRhcnN6dG9yaWsvYW50YWwtaW1yZS10aXRrYWktaWlpLXJlc3otdmVsZXRsZW51bC1sZXR0LXRldmVzLzlxMWsyYzU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNg/69b31bd04d2f0e8d990b13ddB7ab0b526";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2FudGFsLWltcmUta3VkbGlrLWp1bGlhLWthcGNzb2xhdGEvZWtxNXduOD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE2/69b31bd04d2f0e8d990b13ddC3340392d";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3NlYmVzdHllbi1iYWxhenMta29zc3V0aC1yYWRpby1tYWd5YXItcGV0ZXIvbGZ6ZTR4Nj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE2/69b31bd04d2f0e8d990b13ddC3d7fddb1";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dlc3p0ZXNpLWthcm9seS1zenVsaW5hcC1nYWxhbWJvcy1sYWpvcy8ycmZtaGN4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTY/69b31bd04d2f0e8d990b13ddDc2a78112";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvamVsbGluZWstZGFuaWVsLXZhZ3lvbmFkby1sZWdnYXpkYWdhYmItbWFneWFyb2svY3luaDV4dz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE2/69b31bd04d2f0e8d990b13ddBd13bbf80";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvamVsbGluZWstZGFuaWVsLXZhZ3lvbmFkby1sZWdnYXpkYWdhYmItbWFneWFyb2svY3luaDV4dz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE2/69b31bd04d2f0e8d990b13ddDd13bbf80";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9zenVsZWptYW4tY3NhbGFzLXN6dGFyLWxlaHV6YXMtcmVuZG9yc2VnL2Y1czdsZjI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNg/69b31bd04d2f0e8d990b13ddC55fb8743";"https://link.blikk.hu/click/45221559.7091/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC92ZWdyZWhhanRhc2ktZWxqcmFzLWFydmVyZXMvdGRnd2JkMz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE2/69b31bd04d2f0e8d990b13ddC42e828d8"</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Bodrogi Gyula megmondta, meddig él majd</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9maWxta2xpa2svc3VzdS1hLXNhcmthbnktZmVsdWppdGFzYS1kdW5hLXR2L3ZqczVtcmQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNQ/69b31bd04d2f0e8d990b13ddB4f36674a";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JvZHJvZ2ktZ3l1bGEtc3p1bGluYXAtdGFuYy10b2xvc3play8ydmJuOXRtP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddBe35059be";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay90ZWNoL21vYmlsdGVsZWZvbi1pbnRlcm5ldC1zZWJlc3NlZy9qcWptYmVmP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddBc13f1a49";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3BhcC1yaXRhLWJvZG5hci1hdHRpbGEtbnl1Z2Rpai9seXpiN3dtP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddDf5022e42";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvdWpwZXN0LXN0YWRpb24ta29ybWFueXZhbHRhcy9tZXhsOWpyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddCda20555f";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNQ/69b31bd04d2f0e8d990b13ddB3d22f71b";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9lZ2VzenNlZy9lZ3lzemVydS1tb2RzemVyLWFsb21iYS1yaW5nYXQvNnc1cnE2OT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE1/69b31bd04d2f0e8d990b13ddB01862fe7";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3BhcC1yaXRhLWJvZG5hci1hdHRpbGEtbnl1Z2Rpai9seXpiN3dtP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddBf5022e42";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2R1ZGFzLW1pa2xvcy1zaXJqYS9qN3Q0anMxP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddBcd9c68f6";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2xvdmFzLWFubmFiZWxsYS1tZWdoYWx0LXJlbmRvcnNlZ2ktbnlvbW96YXMtaGF0aXpzYWstdWphYmItcmVzemxldGVrLzY2Y2w5YmY_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNQ/69b31bd04d2f0e8d990b13ddC7a85a7a4";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9ldXJvcGFpLWJpem90dHNhZy1ldXJvcGFpLWJpem90dHNhZy1tYWd5YXItcGV0ZXItYnJ1c3N6ZWwvOXd2amtneT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE1/69b31bd04d2f0e8d990b13ddCdcf0cd60";"https://link.blikk.hu/click/45209402.5819/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JlcmtpLXBhdHJpay1kYWdhbmF0LW1hbmdvLW1hcmdpdC9rdHNrcngwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddB60b765b8"</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Blikk új sport sablon teszt</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>15 April 2026</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45209394.11606/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQva3VsZm9sZGktZm9jaS9kb25uYXJ1bW1hLWJldG9yZXMtYm9ydG9uLWtpbnphcy95djBiZzh4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zcG9ydC13ZWVrbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNQ/69b31bd04d2f0e8d990b13ddC51d46120";%20lelki%20egyens%C3%BAlyr%C3%B3l;"https://link.blikk.hu/click/45209394.11606/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvZ3l1bGF5LXpzb2x0LWxlbW9uZG90dC1tZWdzem9sYWx0L3J2eXZncGY_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXNwb3J0LXdlZWtseSZ1dG1fY29udGVudD0yMDI2LTA0LTE1/69b31bd04d2f0e8d990b13ddBd3823449";"https://link.blikk.hu/click/45209394.11606/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvZnJhZGktcHVza2FzLWdhbGVyaWEvZ2NiMTRubD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3BvcnQtd2Vla2x5JnV0bV9jb250ZW50PTIwMjYtMDQtMTU/69b31bd04d2f0e8d990b13ddB28c73801";%20%C3%A9s%20szerintem%20neked%20is%20nagyon%20tetszene.%20R%C3%B6vid;"https://link.blikk.hu/click/45209394.11606/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQva3VsZm9sZGktZm9jaS9saXZlcnBvb2wtcHNnLWVsby1lcmVkbWVueS9oMzltMmowP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zcG9ydC13ZWVrbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNQ/69b31bd04d2f0e8d990b13ddC4d31e7a1";"https://link.blikk.hu/click/45209394.11606/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvbGFiZGFydWdhcy1uYi1pLXRldmVrb3p2ZXRpdGVzLWpvZ2Rpai8wdjBjcHdyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zcG9ydC13ZWVrbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNQ/69b31bd04d2f0e8d990b13ddCb3b914c8";"https://link.blikk.hu/click/45209394.11606/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvZ3l1bGF5LXpzb2x0LWxlbW9uZG90dC1tZWdzem9sYWx0L3J2eXZncGY_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXNwb3J0LXdlZWtseSZ1dG1fY29udGVudD0yMDI2LTA0LTE1/69b31bd04d2f0e8d990b13ddDd3823449"</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Ezt tervezi Magyar és Orbán a választás után</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>14 April 2026</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9iZXQtcmVzenZlbnlhcmZvbHlhbS1vcHVzLTRpZy1ncmFuaXQtbWJoL2xrY3c4Zmc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNA/69b31bd04d2f0e8d990b13ddC0b8de4cb";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvZnJhZGktYWxsYW1pLXBlbnplay9uZDl3cGU5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTQ/69b31bd04d2f0e8d990b13ddB088f16f5";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2RlcmktamFub3Mtc2lyamEtZXZmb3JkdWxvLTc1LXN6dWxldGVzbmFwLzhuejF5eWw_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNA/69b31bd04d2f0e8d990b13ddCcf6b81e3";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL21hZ3lhci1wZXRlci1zYWp0b3RhamVrb3p0YXRvLWhldGZvLzcxa3o0Zjg_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNA/69b31bd04d2f0e8d990b13ddBa862f5c3";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3BvbGl0aWthaS1zemVyZXB2YWxsYWxhcy12aXNzemF0ZXJlcy9wdDFnMnp2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTQ/69b31bd04d2f0e8d990b13ddBb93bdb16";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9oYWxhbG9zLWd5b3JzdWxhc2ktdmVyc2VueS8zZGN5bGJnP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTQ/69b31bd04d2f0e8d990b13ddBf750e64a";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci82NXR4emxyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTQ/69b31bd04d2f0e8d990b13ddB85bf5ec5";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3BvbGl0aWthaS1zemVyZXB2YWxsYWxhcy12aXNzemF0ZXJlcy9wdDFnMnp2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTQ/69b31bd04d2f0e8d990b13ddDb93bdb16";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9kdW5hLWVsdHVudC1maWF0YWwtYmFsbmEvanQ5NDNjZD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE0/69b31bd04d2f0e8d990b13ddBd35a1f49";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9hbGFnc29yaS1oZWx5aXNlZ2VrLWluZ2F0bGFucGlhYy83NjhnZ3cwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTQ/69b31bd04d2f0e8d990b13ddB4d337b48";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL21hZ3lhci1wZXRlci1jc2FsYWRqYS1maWFpLXZhcmdhLWp1ZGl0LzkwMjhzemU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNA/69b31bd04d2f0e8d990b13ddC89e698af";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dhbHZvbGd5aS1qYW5vcy12YWxhc3p0YXMtZXJlZG1lbnktb3JiYW4tdmlrdG9yL2ZrcndkZ3Y_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xNA/69b31bd04d2f0e8d990b13ddB05218ccd";"https://link.blikk.hu/click/45183009.11629/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2Vja3Uta29ybWFueWluZm8tZ3VseWFzLWdlcmdlbHkvMnJ2eHo3eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTE0/69b31bd04d2f0e8d990b13ddBee9e09b9"</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>​​A Tisza nyerte a magyarországi választásokat</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>13 April 2026</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3NjaG9iZXJ0LW5vcmJlcnQtZWhzZWdsYXphZGFzLWJsaWtrLXZhbGFzenRhcy9nczB5bGpkP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTM/69b31bd04d2f0e8d990b13ddCff495032";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2Vja3Uta29ybWFueWluZm8tZ3VseWFzLWdlcmdlbHkvMnJ2eHo3eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEz/69b31bd04d2f0e8d990b13ddDfa57116c";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2Vja3Uta29ybWFueWluZm8tZ3VseWFzLWdlcmdlbHkvMnJ2eHo3eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEz/69b31bd04d2f0e8d990b13ddBfa57116c";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC92YWNpLXV0aS1mZWx1bGphcm8tdG9yb2stYW1va2Z1dG8tZHJvZy1hbGtvaG9sLzdoZzRnc3g_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xMw/69b31bd04d2f0e8d990b13ddCa6f0389d";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL21hZ3lhci1wZXRlci1iZXN6ZWQtZ3lvemVsZW0tdmFsYXN6dGFzL2ZxMmpsOWw_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xMw/69b31bd04d2f0e8d990b13ddC72f9cf63";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90aXN6YS1wYXJ0LWJ1bGktYnVkYXBlc3QvbGtzcjgxeT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEz/69b31bd04d2f0e8d990b13ddCc4a1dbd1";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2FsZXJpYS92YWxhc3p0YXMtMjAyNi1maWRlc3otZXJlZG1lbnl2YXJvL3M2ZDU0bjA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xMw/69b31bd04d2f0e8d990b13ddB6776ba9b";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci1ncmF0dWxhbHQtbWFneWFyLXBldGVybmVrL2huejg4cTA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xMw/69b31bd04d2f0e8d990b13ddB6384a97d";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90aXN6YS1wYXJ0LWJ1bGktYnVkYXBlc3QvbGtzcjgxeT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEz/69b31bd04d2f0e8d990b13ddDc4a1dbd1";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hldGktaGV0ZXMtMjAyNi1lbHNvLWFkYXMvNWY5YjdseD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEz/69b31bd04d2f0e8d990b13ddBd24def9c";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2FsZXJpYS90aXN6YS1wYXJ0LWVyZWRtZW55dmFyby12YWxhc3p0YXMtZ3lvemVsZW0vOXlxYzNqbT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEz/69b31bd04d2f0e8d990b13ddBfc8062d4";"https://link.blikk.hu/click/45171410.7881/aHR0cHM6Ly93d3cuYmxpa2suaHUvYmxpa2stdHYvdmFsYXN6dGFzLTIwMjYtZXJlZG1lbnl2YXJvLXN6dGFyb2staGlyZXNzZWdlay8wemNuZWxnP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTM/69b31bd04d2f0e8d990b13ddC798fdf65"</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Hét év börtönt kapott a Megasztárból ismert énekes</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10 April 2026</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9lbHR1bnQtc29tb2d5LWZlcmZpLWZpYS1ob2x0dGVzdC9zenBocTBsP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTA/69b31bd04d2f0e8d990b13ddC529f2378";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3VsZm9sZC9lZGVzYW55YS1tZWdzem9sYWwtZ3JvbmxhbmQtc3pha2FkZWtiYS16dWhhbnQvbGZkNzBnbD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEw/69b31bd04d2f0e8d990b13ddCa93a846e";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvcmV2ZXN6LXpzdXpzYS1neWlsa29zYS10YXJneWFsYXMvNGtxNjBndz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEw/69b31bd04d2f0e8d990b13ddBdb82c70e";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2Vsc29mb2t1LWl0ZWxldC1ib3J0b24tZmVrZXRlLWRhdmlkL2U1Z2RocHY_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xMA/69b31bd04d2f0e8d990b13ddC8122a298";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbnl1Z2RpamFzLWNzYWxvay1hdXN6dHJpYWJhbi90c3owaDF0P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTA/69b31bd04d2f0e8d990b13ddD746c8396";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbnl1Z2RpamFzLWNzYWxvay1hdXN6dHJpYWJhbi90c3owaDF0P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTA/69b31bd04d2f0e8d990b13ddB746c8396";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21hZ3lhci1zenRhcm9rLWJvcnRvbi1yYWNzb2svNXp0Y3FyeD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEw/69b31bd04d2f0e8d990b13ddBac55a10d";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvb2xpbXBpYS1qYXJhZGVrLW1hZ3lhcm9yc3phZy10b3BsaXN0YS8zZGJ6M2M4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTA/69b31bd04d2f0e8d990b13ddDc5230e88";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvb2xpbXBpYS1qYXJhZGVrLW1hZ3lhcm9yc3phZy10b3BsaXN0YS8zZGJ6M2M4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTA/69b31bd04d2f0e8d990b13ddBc5230e88";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC90aXBwZWsvbWFnYXNhZ3lhcy1oZWx5ZXR0LW1vZGVybi1rZXJ0L2x4ZDlxMDk_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0xMA/69b31bd04d2f0e8d990b13ddC88aba7c5";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvc3RhZGxlci1qb3pzZWYtYWthc3p0by1ueW9tb24tdmFneXVuay80d3d6emZzP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMTA/69b31bd04d2f0e8d990b13ddCd3390caf";"https://link.blikk.hu/click/45147013.1183/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2lzdHZhbi1hLWtpcmFseS12YWxhc3p0YXMtcGFydC1maWRlc3otdGlzemEtYnJvZHktc3pvcmVueWkvZ2tnMHNnaj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTEw/69b31bd04d2f0e8d990b13ddCc4785915"</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Orbán Viktor elárulta, kik az igazi barátai</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>09 April 2026</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9lbHR1bnQtY3NlY3NlbW8tdG9sbmEtdmFybWVneWUtdGFtYXNpL3I0Y244MTA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOQ/69b31bd04d2f0e8d990b13ddC625a0a3d";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvb2xhamFyLWNzb2trZW5lcy11emVtYW55YWdhcmFrLXRhcnRhbGVrL2hkbDhzNTU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOQ/69b31bd04d2f0e8d990b13ddB6646b3c8";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3J1YmludC1yZWthLXNjaG9iZXJ0LW5vcmJlcnQtcmFrLzI3bW5scW0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOQ/69b31bd04d2f0e8d990b13ddD09965c87";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2thcmFmaWF0aC1vcnNvbHlhLWd5dWp0b2dldGVzL25nMnE2aGg_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOQ/69b31bd04d2f0e8d990b13ddC685ede48";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3J1YmludC1yZWthLXNjaG9iZXJ0LW5vcmJlcnQtcmFrLzI3bW5scW0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOQ/69b31bd04d2f0e8d990b13ddB09965c87";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvYXV0by9lcmRvYmVuLXRhbGFsdC12b2xrc3dhZ2VuLXQxLWtpc2J1c3ovemRlMjYwNj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTA5/69b31bd04d2f0e8d990b13ddB0ac0ae9b";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9kaXN6dGF2aXJhdC1iZWhhanRvay1rb3ZldGVsZXMvMWdiaDNlcj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTA5/69b31bd04d2f0e8d990b13ddC026a1125";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvYXV0by9lcmRvYmVuLXRhbGFsdC12b2xrc3dhZ2VuLXQxLWtpc2J1c3ovemRlMjYwNj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTA5/69b31bd04d2f0e8d990b13ddD0ac0ae9b";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2Zhcmthc2hhenktdGl2YWRhci1mZWxlc2VnZS10ZW1ldGVzZS1taW1pL3oyYjY1azA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOQ/69b31bd04d2f0e8d990b13ddC40afb063";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9vcmJhbi12aWt0b3ItYmxpa2stdGFsay1pbnRlcmp1LXZhbGFzenRhcy9wazVxZzdtP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDk/69b31bd04d2f0e8d990b13ddC9df92164";"https://link.blikk.hu/click/45119002.7522/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JlcmVjemtpLXpvbHRhbi1yb3Nzei1zem9rYXMtc3p1bGV0ZXNuYXAvanhqZjA5dz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTA5/69b31bd04d2f0e8d990b13ddC381595dc"</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>J. D. Vance: „Sokat tanultam Orbán Viktortól” – Exkluzív interjú</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>08 April 2026</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvdmlsYWdwb2xpdGlrYS9qLWQtdmFuY2Utb3JiYW4tdmlrdG9yLWFtZXJpa2EtYWxlbG5vay1pbnRlcmp1L2MzNGM0dG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddC3ea61a9a";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3dvc3NhbGEtcm96aW5hLzBsNndjbG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddB283d3559";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9tb3RvcmNzb25hay1jc2Vjc2Vtby1kdW5hLXZlc3plbHllenRldGVzL3cyNGNmZnk_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddB4c3788a7";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvYnVkYXBlc3RpLWJham5va29rLWxpZ2FqYS1kb250by1zemFsbGFzLWFyYWsvd2Y5ODE1ej91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTA4/69b31bd04d2f0e8d990b13ddB5ccf0f95";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3ZhZG9uLWphbmktcnRsLWhldGktaGV0ZXMtdmFsYXN6dGFzMjAyNi9laHYzcXQ2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDg/69b31bd04d2f0e8d990b13ddB3d59e4ce";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9sb3Zhcy1hbm5hYmVsbGEtbmFneS1vLWhhbGFsL2RubjRya2Y_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddC0d17e29d";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2thcnBhdGktcmViZWthLXBhcmphLXN6ZXJlbG1lcy9mcWhsdjI0P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDg/69b31bd04d2f0e8d990b13ddC17852486";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2VrbGVyLWx1Y2EtZXhhdGxvbi1iYWwta2V6LzVzbHR3NGQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddDfdaf9df9";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2VrbGVyLWx1Y2EtZXhhdGxvbi1iYWwta2V6LzVzbHR3NGQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddBfdaf9df9";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9tYWd5YXJvcnN6YWdpLW9ydm9zaS1lbHV0YXNpdGFzLzZ6aDAwM2M_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddC18b75c0f";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvdmlsYWdwb2xpdGlrYS9qZC12YW5jZS1mZWxlc2VnZS1wb2Nhay8xeTV4bXhtP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDg/69b31bd04d2f0e8d990b13ddBd358cbad";"https://link.blikk.hu/click/45104936.13251/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvdmlsYWdwb2xpdGlrYS9qLWQtdmFuY2Utb3JiYW4tdmlrdG9yLWFtZXJpa2EtYWxlbG5vay1pbnRlcmp1L2MzNGM0dG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wOA/69b31bd04d2f0e8d990b13ddD3ea61a9a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Megszólalt a Blikknek a fogászaton halálba altatott mérnök özvegye</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>07 April 2026</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9mb2dvcnZvc2ktYmVhdmF0a296YXMtaGFsYWxlc2V0L2c2bHJmZHQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wNw/69b31bd04d2f0e8d990b13ddCef812549";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvYWxhcGl0dmFueWktY3NhbGFzLzB2Y2c0MHE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wNw/69b31bd04d2f0e8d990b13ddBe86552d6";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2xvdmFzLWFubmFiZWxsYS1ob2x0dGVzdC1tZWdoYWx0LXJlbmRvcnNlZy93M3Roc2N3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDc/69b31bd04d2f0e8d990b13ddCcfb4a113";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9mb2dvcnZvc2ktYmVhdmF0a296YXMtaGFsYWxlc2V0L2c2bHJmZHQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wNw/69b31bd04d2f0e8d990b13ddDef812549";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQva29zenRhZGlub3ZhLW1hZ2FzdWdyYXMtcGxhc3p0aWthemFzLXBvbGl0aWthL2JxejZmM3o_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wNw/69b31bd04d2f0e8d990b13ddBed8ad4e9";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9lbHRvcnRlLWZvZ29ydm9zLWZvZ2h1emFzLWFsbGthcG9jcy92MHF2Z3h3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDc/69b31bd04d2f0e8d990b13ddBaf4a1ca4";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3Zvcm9zLWF0dGlsYS10YW5rY3NhcGRhLWdpdGFyLW5ldmVybW9yZS1wYWx5YWZ1dGFzL2N3c21oZzk_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wNw/69b31bd04d2f0e8d990b13ddCc5b4f926";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9raXNjc2liZS1rZWx0ZXMtYm9sdGl0b2phcy82MHltN3E1P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDc/69b31bd04d2f0e8d990b13ddCaedb3594";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvYXV0by9wYWxpay1sYXN6bG8tZ3VydWx1bmstYm13LXgzLXRlc3p0L2pzMTUxajE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wNw/69b31bd04d2f0e8d990b13ddB5a44850d";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2thcnBhdGktcmViZWthLW9yb2tiZWZvZ2FkYXMta29uZ29pLWRlbW9rcmF0aWt1cy1rb3p0YXJzYXNhZy9jNzVndnNlP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDc/69b31bd04d2f0e8d990b13ddDf0b3bdb3";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2thcnBhdGktcmViZWthLW9yb2tiZWZvZ2FkYXMta29uZ29pLWRlbW9rcmF0aWt1cy1rb3p0YXJzYXNhZy9jNzVndnNlP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDc/69b31bd04d2f0e8d990b13ddBf0b3bdb3";"https://link.blikk.hu/click/45077130.11601/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9lZ2VzenNlZy9ub3Zlbnl2ZWRvLXN6ZXItem9sZHNlZy1neXVtb2xjcy1saXN0YS9ieHR4NnpkP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDc/69b31bd04d2f0e8d990b13ddB1393ae40"</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>A válásáról beszélt Nagy Bogi</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>02 April 2026</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3VsZm9sZC9vcm9zei1kcm9udGFtYWRhcy1rYXJwYXRhbGphLWVsbGVuLWFyYW1zenVuZXQtaGlyemFybGF0LzBzYjYyNnE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMg/69b31bd04d2f0e8d990b13ddB139bd99e";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvYmF0b255dGVyZW55ZS8xcXZmdmdkP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDI/69b31bd04d2f0e8d990b13ddB3c9b0ae5";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9oYWJvcnUtYmVmZWt0ZXRlcy1hcmFueS1hcmZvbHlhbS1lc2VzLXBlbnotZ2F6ZGFzYWcvc3h6ZDIwMT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTAy/69b31bd04d2f0e8d990b13ddB175fbe61";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL25hZ3ktYm9naS12YWxhcy1oaXJuZXYtemVuZS9kZ3dkbXJ2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDI/69b31bd04d2f0e8d990b13ddDc0d3c865";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHVodHRwcy8vd3d3LmJsaWtrLmh1L3BvbGl0aWthL21hZ3lhci1wb2xpdGlrYS9vcmJhbi12aWt0b3ItYmVrb2x0b3p2ZS1oYWpkdS1wZXRlcmhlei1sZXZhaS1hbmlrby1oYXphc3NhZy9keG41NzBnP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDI/69b31bd04d2f0e8d990b13ddBa4103399";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci1iZWtvbHRvenZlLWhhamR1LXBldGVyaGV6LWxldmFpLWFuaWtvLWhhemFzc2FnL2R4bjU3MGc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMg/69b31bd04d2f0e8d990b13ddBb24756b8";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2tvY3Npcy16b2x0YW4taGFneWF0ZWstYXJjaGl2dW0tY3NhbGFkL200bjBqNjE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMg/69b31bd04d2f0e8d990b13ddBebe3d449";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3ZhZGtlcnRpLWFkZWwtamFrYWJvcy16c3V6c2FubmEtZXhhdGxvbi1wYXJiYWotdXRhbi85c3dnMmh4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDI/69b31bd04d2f0e8d990b13ddC0c4b7b51";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9idWRhcGVzdC1sYW5jemhpZC10cmFnZWRpYS1sZWdlbmRhLXZhbG9zYWcvM250a3htbT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTAy/69b31bd04d2f0e8d990b13ddC66f829a9";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL25hZ3ktYm9naS12YWxhcy1oaXJuZXYtemVuZS9kZ3dkbXJ2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDI/69b31bd04d2f0e8d990b13ddBc0d3c865";"https://link.blikk.hu/click/45016183.12697/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2tpYXJhLWxvcmQtbGFrYXRvcy1sZXZlbnRlLWVza3V2by92MmNkdmZwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDI/69b31bd04d2f0e8d990b13ddCe159a48c"</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Hiénák nyerészkednek a Demjén-musicalen</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>01 April 2026</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC92YWxhc3p0YXMtcG9saXRpa3VzLWJpemFsb20tYnVkYXBlc3QvYzN5ZzF6bD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTAx/69b31bd04d2f0e8d990b13ddC47ad07b1";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dpZG9mYWx2eS1hdHRpbGEtbmFneS1mZXJvLWFydWxvL3BwZHowdjA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMQ/69b31bd04d2f0e8d990b13ddB585c059d";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZHVndWxhc2VsaGFyaXRhcy1hdHZlcmVzLWNzYWxvay1taWxsaW9zLW9zc3plZ2VrLXJla29yZC95OGwya2QwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDE/69b31bd04d2f0e8d990b13ddB48c9340d";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dpZG9mYWx2eS1hdHRpbGEtbmFneS1mZXJvLWFydWxvL3BwZHowdjA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMQ/69b31bd04d2f0e8d990b13ddD585c059d";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC90aXBwZWsvYmFuYW4tdmFyYXRsYW4taGF0YXNhLWFsdmFzcmEvc2V6YnQ0dD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTAx/69b31bd04d2f0e8d990b13ddB14fd33c9";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hvZ3lhbi10dWRuZWstZWxuaS1uZWxrdWtlZC1tdXNpY2FsLWplZ3ktZWxhZGFzL3Q4ZGQ4dmc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMQ/69b31bd04d2f0e8d990b13ddD9ccfb824";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZHVndWxhc2VsaGFyaXRhcy1hdHZlcmVzLWNzYWxvay1taWxsaW9zLW9zc3plZ2VrLXJla29yZC95OGwya2QwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDE/69b31bd04d2f0e8d990b13ddC48c9340d";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYXV0by9kYW5pZWwtY3JhaWctZGVuemEtbWFya2FuYWd5a292ZXQvejVqcTR2cD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTAx/69b31bd04d2f0e8d990b13ddB420cb0b8";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9zemlqamFydG8tc3phbmtjaW9zLWxpc3RhLW9yb3N6LW9saWdhcmNoYS9udjJjc3loP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDE/69b31bd04d2f0e8d990b13ddB2cff1f9e";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvaW50ZXJuZXRlcy1jc2FsYXMtc3ppbmhhei1rb25jZXJ0LWplZ3llay1idWRhcGVzdGktbm8vNGVmM3d4Zz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTA0LTAx/69b31bd04d2f0e8d990b13ddBf2da7376";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay90ZWNoL3RlY2gta29ueWhhaS10cmVuZGVrLWJ1cmtvbGF0LWNzZW1wZS1hdGFsYWtpdGFzLWZlbHVqaXRhcy9zZzZsdHBrP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDE/69b31bd04d2f0e8d990b13ddBaaa62b1c";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9iYWJvdC1tYWxkaXYtc3ppZ2V0ZWstdXRhemFzL255cnNlZ2Q_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wNC0wMQ/69b31bd04d2f0e8d990b13ddC86a6e956";"https://link.blikk.hu/click/45000255.1624/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9tb3pnYXNrb3JsYXRvem90dC1hZG9zLWF1dG8tbGVmb2dsYWxhcy83azJ3eXZ2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDQtMDE/69b31bd04d2f0e8d990b13ddCa4975806"</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>A tudtuk nélkül élő adásban megy egy család magánélete Egerben</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>31.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkva2luY3N2YWRhc3pvay1lbGxvcG90dC1ncmFmaWthLWVncnktam96c2VmL2h3ZDNsNzE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMQ/69b31bd04d2f0e8d990b13ddCc6f8593b";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JvY2hrb3ItZ2Fib3ItbWVnYXN6dGFyLW1hbmlwdWxhY2lvLzU3MmtiNm4_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMQ/69b31bd04d2f0e8d990b13ddCf17ebde5";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvaHVzdmV0LWVsZWxtaXN6ZXJib2x0b2stbnlpdHZhLXRhcnRhcy9yMzJkY2d3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMzE/69b31bd04d2f0e8d990b13ddB12967a8c";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2tvdmFjcy1hcm9uLWFwYXNhZy1uYWd5LWR1ZXR0L2p0NHd6cHg_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMQ/69b31bd04d2f0e8d990b13ddB5be44205";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2V4YXRsb24taHVuZ2FyeS1uYWd5LWJlbmVkZWstYmF0eWphLXNlcnVsZXMvaGh4ZTJxZj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMx/69b31bd04d2f0e8d990b13ddDbc6d9626";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2thcGl0YW55LWlzdHZhbi10aXN6YS1wYXJ0LWhvcnRheS1vbGl2ZXItc3phemhhbG9tYmF0dGEtb2xhamZpbm9taXRvLzdkMmZqbmQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMQ/69b31bd04d2f0e8d990b13ddC169ccaf4";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2V4YXRsb24taHVuZ2FyeS1uYWd5LWJlbmVkZWstYmF0eWphLXNlcnVsZXMvaGh4ZTJxZj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMx/69b31bd04d2f0e8d990b13ddBbc6d9626";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9nYXN6dHJvL2JvbHRpLWh1c3ZldGktc29ua2EtdGVzenQvbGc5YzgzeD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMx/69b31bd04d2f0e8d990b13ddCf04a7cdf";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2F6c2lhLWV4cHJlc3N6LXZvbWJlcmctZnJpZ3llcy10aXNjaGxlci1wZXRyYS1zZWZlay1zZWZlL2YzbGJyZWU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMQ/69b31bd04d2f0e8d990b13ddC1c49fd41";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9iZWJpb3ItbWFnYW5lbGV0LWtvenZldGl0LWVnZXIvY21yM3ptaz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMx/69b31bd04d2f0e8d990b13ddCd8fe1018";"https://link.blikk.hu/click/44972127.383/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2tvdmFjcy1hcm9uLWFwYXNhZy1uYWd5LWR1ZXR0L2p0NHd6cHg_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMQ/69b31bd04d2f0e8d990b13ddD5be44205"</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Ezt tudhatja Orbán Viktor páncélozott autója: a szakértő szerint indokolt lehet a védelem</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>30.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9kcm9nb3Mtc29mb3ItYW1va2Z1dGFzL2JoNDFxYmQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMA/69b31bd04d2f0e8d990b13ddB938be394";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9vcmJhbi12aWt0b3ItcGFuY2Vsb3pvdHQtYXV0by1zemFrZXJ0by9qbmJmaG14P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMzA/69b31bd04d2f0e8d990b13ddC80ebdcaf";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci1iZWtlc2NzYWJhLW9yc3phZ2phcmFzL2N2c201MnA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMA/69b31bd04d2f0e8d990b13ddB4a2f701c";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2tyYXVzei1nYWJvci1taWtlcy1hbm5hLXBhcmthcGNzb2xhdC1tYXJpY3MtcGV0aS9rOHI1NnhoP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMzA/69b31bd04d2f0e8d990b13ddC487aa842";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC91dGF6YXMvaHVzdmV0LXV0YXphcy1rdWxmb2xkLzVjanBxMno_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMA/69b31bd04d2f0e8d990b13ddCdca930ff";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci1iZWtlc2NzYWJhLW9yc3phZ2phcmFzL2N2c201MnA_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMA/69b31bd04d2f0e8d990b13ddD4a2f701c";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21vbmlxdWUtY292ZXQta29yaGF6LWluamVrY2lvLzhtN3E3a2Y_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMA/69b31bd04d2f0e8d990b13ddC27e5ceb8";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3N6dWpvLXpvbHRhbi1sYW55YS1tdXNvcnZlemV0by10ZWxldml6aW9zLzRkYjA2OGw_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0zMA/69b31bd04d2f0e8d990b13ddC64ceb548";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9jc2FsYWRpLWRyYW1hamEtaGFtdmFqLWF1c3p0cmlhLWd5aWxrb3NzYWcvZW1xZ2Rqdz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMw/69b31bd04d2f0e8d990b13ddD18f206a1";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9ub2ktbXVua2FlcnAtZmVyZmktc3pha21hLWthbWlvbm9zLXZpbGxhbnlzemVyZWxvLWJ1cmtvbG8veHE3cjJ0aD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMw/69b31bd04d2f0e8d990b13ddC7d7df299";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9jc2FsYWRpLWRyYW1hamEtaGFtdmFqLWF1c3p0cmlhLWd5aWxrb3NzYWcvZW1xZ2Rqdz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMw/69b31bd04d2f0e8d990b13ddB18f206a1";"https://link.blikk.hu/click/44958727.8951/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL29yYmFuLXZpa3Rvci1wYW5jZWxhdXRvLXVrcmFuLWZlbnllZ2V0ZXMva3N4enR0NT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTMw/69b31bd04d2f0e8d990b13ddB1d016823"</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Itt a nagy európai benzinártérkép!</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>27.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9iZXRlZ3NlZy1kYWdhbmF0b3MtYmV0ZWdzZWctcmFrLW1lZ2Vsb3plcy8wamxsMWo3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjc/69b31bd04d2f0e8d990b13ddCca575b49";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9sZWxlay9odXN2ZXQtdGlwcGVrLWNzYWxhZGktZHJhbWEtZWxsZW4vMThxNW01Zj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI3/69b31bd04d2f0e8d990b13ddB28ca60d0";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei91emVtYW55YWdhcmFrLW1hZ3lhcm9yc3phZy1ldXJvcGFpLW9zc3plaGFzb25saXRhcy9kajByOWt5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjc/69b31bd04d2f0e8d990b13ddC01ebf092";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9idW50ZXRvZWxqYXJhcy1mb2dvcnZvcy1lbGxlbi9zZ2poajBxP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjc/69b31bd04d2f0e8d990b13ddC44c7f9f9";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei91emVtYW55YWdhcmFrLW1hZ3lhcm9yc3phZy1ldXJvcGFpLW9zc3plaGFzb25saXRhcy9kajByOWt5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjc/69b31bd04d2f0e8d990b13ddE01ebf092";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9sZWdpZG9zZWJiLW1hZ3lhci1naXppLW5lbmkvZ2gxcjZ6bT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI3/69b31bd04d2f0e8d990b13ddDd1bde5cd";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9jc2FwZGEtbnl1Z2RpamFzLW9zenRyYWstbWFneWFyLWJldG9yb2sva2JrNGZ3Mz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI3/69b31bd04d2f0e8d990b13ddBf6a3a5f0";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9neW9neXN6ZXJlc3ota3JvbmlrdXMtYmV0ZWctbWFneWFyLWtvemxvbnktcmVuZGVsZXQtYmVsdWd5bWluaXN6dHJlZXJpdW0vaHdqYzJ0Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI3/69b31bd04d2f0e8d990b13ddB0204a9e4";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9lbXUtdGFydGFzLWJhcm9tZml1ZHZhci1oYXppa2VkdmVuYy83dnczY2h6P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjc/69b31bd04d2f0e8d990b13ddB7c339c29";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JvcmFyb3MtZ2Fib3IvazI3dzg4cT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI3/69b31bd04d2f0e8d990b13ddCf497b319";"https://link.blikk.hu/click/44933492.5731/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9sZWdpZG9zZWJiLW1hZ3lhci1naXppLW5lbmkvZ2gxcjZ6bT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI3/69b31bd04d2f0e8d990b13ddBd1bde5cd"</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>A halála előtt tudta meg Jákli Mónika, hogy megcsalja a vőlegénye?</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>26.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2pha2xpLW1vbmlrYS1yb2RlcmlrLXVqLXN6ZXJlbGVtLWJvcmFyb3MtZ2Fib3IvMnExc2w0Yj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI2/69b31bd04d2f0e8d990b13ddBbfb30525";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2ZpbHV0YXMtdmlrdG9yLWV4YXRsb24tc2VydWxlcy12YWxsa2l1Z3Jhcy9ydzQxZTNmP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjY/69b31bd04d2f0e8d990b13ddBfe6d7dd5";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3VsZm9sZC9vbmx5ZmFucy10dWxhamRvbmpvZy1oYXJjLzB2NWpreGs_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNg/69b31bd04d2f0e8d990b13ddCe3a62547";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9uZW16ZXRrb3ppLXN6dGFyb2svcGFsdmluLWJhcmJhcmEtbWlsZXktY3lydXMtcGFzaS9xNjVyNnB3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjY/69b31bd04d2f0e8d990b13ddCb3c4d33d";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3VsZm9sZC9yZXB1bG90ZXItcmVwdWxvZ2VwLXV0YXNvay11dGtvemVzLWJpenRvbnNhZy81eHRxYzBrP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjY/69b31bd04d2f0e8d990b13ddC51e4dc93";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9vc3p0cmFrLWNzb2QtbWFneWFyLWJ1dG9yZ3lhci1hZGEvenE3ZmxtOT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI2/69b31bd04d2f0e8d990b13ddC4e6c826c";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2pha2xpLW1vbmlrYS1oYWxhbGEtbWVnY3NhbGFzL2pobTJmNmo_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNg/69b31bd04d2f0e8d990b13ddC7d23f4ec";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9tMy1hcy1hdXRvcGFseWEtYWxyZW5kb3ItY3NhbG8vZXdmMzllcz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI2/69b31bd04d2f0e8d990b13ddC5b805d9b";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2ZpbHV0YXMtdmlrdG9yLWV4YXRsb24tc2VydWxlcy12YWxsa2l1Z3Jhcy9ydzQxZTNmP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjY/69b31bd04d2f0e8d990b13ddDfe6d7dd5";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dhbGxhLW1pa2xvcy1iZXRlZ3NlZ2Vyb2wtb3N6aW50ZW4vbHhxbHhrNj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI2/69b31bd04d2f0e8d990b13ddBcb7abfbb";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3N6aWpqYXJ0by1wZXRlci1rdWx1Z3ltaW5pc3p0ZXItbGVoYWxsZ2F0YXMtdGl0a29zc3pvbGdhbGF0LXZhbGFzenRhcy0yMDI2L3NncnhkM2U_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNg/69b31bd04d2f0e8d990b13ddBc20eae96";"https://link.blikk.hu/click/44903138.12233/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3N6aWpqYXJ0by1wZXRlci1rdWx1Z3ltaW5pc3p0ZXItbGVoYWxsZ2F0YXMtdGl0a29zc3pvbGdhbGF0LXZhbGFzenRhcy0yMDI2L3NncnhkM2U_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNg/69b31bd04d2f0e8d990b13ddDc20eae96"</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>A humor kiságyúi</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>25.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hldGktaGV0ZXMtMjAyNi1lbHNvLWFkYXMtbXVzb3J2ZXpldG8vNDd2c3Q1bT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI1/69b31bd04d2f0e8d990b13ddCe0f69941";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hhbGFzei1qYXptaW4tZXhhdGxvbi1lbGh1bnl0LWVkZXNhcGphL2xxcG52cG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNQ/69b31bd04d2f0e8d990b13ddC357c30f1";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbGFrb2stZWd5dXR0ZWxlcy1qb3pzZWZ2YXJvcy10YXJzYXNoYXotb3JvbWxhbnlvay9zeTJlaDIwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjU/69b31bd04d2f0e8d990b13ddD4a67aa14";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL25hZ3ktYWRhbS1oZXRpLWhldGVzLW11c29ydmV6ZXRvL3d3c2VwOGQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNQ/69b31bd04d2f0e8d990b13ddBf9061d19";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay90ZWNoL2VydGVrZXMtNTAtZm9yaW50b3MtZXJtZS82ZHpibmVmP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjU/69b31bd04d2f0e8d990b13ddB1bab730e";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvZ3VtaWNzZXJlLWFyYWstMjAyNi1ndW1pc29rLW11bmthamEvbnFlNnl6Nz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI1/69b31bd04d2f0e8d990b13ddC73888fbd";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9iYWxhdG9uLXZpenN6aW50LXN6ZXpvbi1lbG90dC92eGN2NzE4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjU/69b31bd04d2f0e8d990b13ddC22bee2a0";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2d5dXJjc2FueS1mZXJlbmMtbWFjc2thLWtyaW1pL3pseGJteXI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNQ/69b31bd04d2f0e8d990b13ddDb329e9ea";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbGFrb2stZWd5dXR0ZWxlcy1qb3pzZWZ2YXJvcy10YXJzYXNoYXotb3JvbWxhbnlvay9zeTJlaDIwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjU/69b31bd04d2f0e8d990b13ddB4a67aa14";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9rYW1hdC1jc29ra2VudGVzLW1uYi12YXJnYS1taWhhbHkvZjdyZ3Jubj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI1/69b31bd04d2f0e8d990b13ddCb49d1334";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2xhemFyLXN6YW5kcmEtYnVkYXBlc3QtbHV4ZS1sYW55a2VyZXMtdmlldG5hbS8ycm5uOHl2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjU/69b31bd04d2f0e8d990b13ddC4a4abcda";"https://link.blikk.hu/click/44887820.6550/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2d5dXJjc2FueS1mZXJlbmMtbWFjc2thLWtyaW1pL3pseGJteXI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNQ/69b31bd04d2f0e8d990b13ddBb329e9ea"</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Ezt a 10 hibát ne kövesse el az szja-bevallásában!</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>24.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvbGlzenRlcy1rcmlzenRpYW4tbmItaWlpL3NkODgwZDc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNA/69b31bd04d2f0e8d990b13ddB04b0d320";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2RlYWstcmViZWthLWhhemFzc2FnLWVsc28tbGF0YXNyYS1rb3pvc3NlZ2ktbWVkaWEtcHJvZmlsLXRvcmxlcy9wZHhnbmJyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjQ/69b31bd04d2f0e8d990b13ddC6b1db672";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2VrbGVyLWx1Y2EtcGFyYWxpbXBpYWktYmFqbm9rLWV4YXRsb24vcDlxOXg5eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI0/69b31bd04d2f0e8d990b13ddDab173080";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2Zhcmthc2hhenktdGl2YWRhci1neWFzemEtbWltaS1oYWxhbGEtZmVsZXNlZy10ZWRkeS9seTd6YjNyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjQ/69b31bd04d2f0e8d990b13ddCdd330fec";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvdXplbWFueWFnLWtvcmxhdG96YXMtaW1wb3J0LWxlYWxsdC9ocnNxc25rP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjQ/69b31bd04d2f0e8d990b13ddCbe13f951";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZWx0dW5lcy1lZ3Jlc3N5LW1hdHlhcy10ZWxlZm9uLWhhamxla3RhbGFuLzl6c2c5MG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNA/69b31bd04d2f0e8d990b13ddB58e25671";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hldGktaGV0ZXMtc3plcmVwbG9pLTIwMjYvczR6cWVzZz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI0/69b31bd04d2f0e8d990b13ddCa746ceda";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9zemphLWJldmFsbGFzLXRlcnZlemV0LWd5YWtvcmktaGliYWsveGowcXY4eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI0/69b31bd04d2f0e8d990b13ddCd2d1edd5";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZWx0dW5lcy1lZ3Jlc3N5LW1hdHlhcy10ZWxlZm9uLWhhamxla3RhbGFuLzl6c2c5MG0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNA/69b31bd04d2f0e8d990b13ddD58e25671";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2VrbGVyLWx1Y2EtcGFyYWxpbXBpYWktYmFqbm9rLWV4YXRsb24vcDlxOXg5eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI0/69b31bd04d2f0e8d990b13ddBab173080";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvYWRvYmV2YWxsYXMtbmF2LXRlcnZlemV0LWRpZ2l0YWxpcy8zenQwcnc5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjQ/69b31bd04d2f0e8d990b13ddB13252365";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL25hZ3ktZHVldHQtZWxvLWVsb2RvbnRvLWdlc3p0ZXNpLXBhbmthLWtvdmFjcy1hcm9uLXRvdmFiYmp1dGFzL3h6a2syZ3M_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yNA/69b31bd04d2f0e8d990b13ddC395a51a0";"https://link.blikk.hu/click/44859040.6537/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9zemphLWJldmFsbGFzLXRlcnZlemV0LWd5YWtvcmktaGliYWsveGowcXY4eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTI0/69b31bd04d2f0e8d990b13ddDd2d1edd5"</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Megszólalt a halálra gázolt rendőr édesapja a baleset részleteiről</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>23.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JvcmFyb3MtZ2Fib3ItamFrbGktbW9uaWthLWJlc3pvbGFzLWhhbGFsLzFkd2Z5NWI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMw/69b31bd04d2f0e8d990b13ddB94d813b1";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9tYWd5YXItY2lnYW55b2svcDczMm43ND91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIz/69b31bd04d2f0e8d990b13ddD5a1f78c9";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9tYWd5YXItY2lnYW55b2svcDczMm43ND91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIz/69b31bd04d2f0e8d990b13ddB5a1f78c9";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3VsZm9sZC9wYW9sby16YW1wb2xsaS1kb25hbGQtbWVsYW5pYS10cnVtcC8xanloenM3P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjM/69b31bd04d2f0e8d990b13ddC51772087";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC92ZXN6cHJlbS1nYXpvbGFzLXJlbmRvci1oYWxhbC1tZWdzem9sYWx0LWFwYS1neWFzei9oNmdydjFwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjM/69b31bd04d2f0e8d990b13ddC33486063";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dlbGVuY3Nlci10aW1lYS1leGF0bG9uLWh1bmdhcnktZXNrdXZvLXV0YXphcy90N2xwOTluP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjM/69b31bd04d2f0e8d990b13ddD96553263";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2dlbGVuY3Nlci10aW1lYS1leGF0bG9uLWh1bmdhcnktZXNrdXZvLXV0YXphcy90N2xwOTluP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjM/69b31bd04d2f0e8d990b13ddB96553263";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2V4YXRsb24taHVuZ2FyeS10djItc3BvcnR2ZXJzZW55LWd5b3p0ZXNlay9qODEzZjY2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjM/69b31bd04d2f0e8d990b13ddCec184a33";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvdG90aC1hbGV4LW1hcmNvLXJvc3NpLXZhbG9nYXRvdHQtc3p1cmtvbG9rL3loa3cxcW0_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMw/69b31bd04d2f0e8d990b13ddCeaedb3a4";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvdGVsZWtvbS12aXZpY2l0dGEtc3pvYm9zemxhaS1rYXB1L3czazk1dGQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMw/69b31bd04d2f0e8d990b13ddCdf3981c6";"https://link.blikk.hu/click/44842099.4869/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2hlcmN6ZWctem9sdGFuLWRpdmF0LXplbmUtZ2l0YXJvemFzL3RoMWduYzc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMw/69b31bd04d2f0e8d990b13ddC2561810f"</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Ezt a 10 hibát ne kövesse el az szja-bevallásában!</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>20.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay9hdXRvL2F1dG9sb3Bhcy0yMDI1LW1hZ3lhcm9yc3phZy8zYmQ2MmJ5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjA/69b31bd04d2f0e8d990b13ddCb2f4c335";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL3VrcmFub2sta2l0aWx0YXMtbWFneWFyb3JzemFnLXNjaGVuZ2VuLzJ2Nmh6MTI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMA/69b31bd04d2f0e8d990b13ddCa45daee4";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvcmVuZG9yb2stZWxnYXpvbGFzYS84OXYzdzUyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjA/69b31bd04d2f0e8d990b13ddC35fbd256";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9zemphLWJldmFsbGFzLXRlcnZlemV0LWd5YWtvcmktaGliYWsveGowcXY4eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddD376fdc35";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC92aXJhZ2JvbHQtZWxsb3BvdHQtdmlyYWdvay12aXNzemFzemVyZXp0ZS1ob3MvejhxbGJxaD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddB4ea36757";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvY3NpcGVzLXRhbWFyYS13aWViZXItb3Jzb2x5YS1raXR1bnRldGVzLWJvdHJhbnkvenF5bG10NT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddB9ece1e5e";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90YXRhYmFueWEtYmFsZXNldC10YXJneWFsYXMvYmRicmd0ND91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddB380e9276";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvdmlkZWtpLWJlbnppbmt1dGFrLXV6ZW1hbnlhZ2hpYW55LWRpemVsLzB2OTc4Mmc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMA/69b31bd04d2f0e8d990b13ddCc9a5f74b";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9zemphLWJldmFsbGFzLXRlcnZlemV0LWd5YWtvcmktaGliYWsveGowcXY4eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddC376fdc35";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvYWRvYmV2YWxsYXMtbmF2LXRlcnZlemV0LWRpZ2l0YWxpcy8zenQwcnc5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMjA/69b31bd04d2f0e8d990b13ddB5d831237";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC92aXJhZ2JvbHQtZWxsb3BvdHQtdmlyYWdvay12aXNzemFzemVyZXp0ZS1ob3MvejhxbGJxaD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddD4ea36757";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3NlZmVrLXNlZmUtcGF0cmlrLWRhdmlkLW5vcmJpLWRvbnRvLWZvZGlqL3cweG56a2Y_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0yMA/69b31bd04d2f0e8d990b13ddC6dd8f460";"https://link.blikk.hu/click/44811792.11402/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvY3NpcGVzLXRhbWFyYS13aWViZXItb3Jzb2x5YS1raXR1bnRldGVzLWJvdHJhbnkvenF5bG10NT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTIw/69b31bd04d2f0e8d990b13ddD9ece1e5e"</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Árulják a berekfürdői horrorházat</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>19.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9zenRhcnN6dG9yaWsvdm9sdC1vbHlhbi1ob2d5LWEtaGFybWFkaWtyb2wtZG9iYWx0YW0tbGUtZ2FiaS1kb2xnYWl0LXRlc3R2ZXJ2aXN6YWx5dWtyb2wtdmFsbG90dGFrLzVudmZwMTE_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOQ/69b31bd04d2f0e8d990b13ddB55c2d951";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvY3NpcGVzLXRhbWFyYS1lbGFkYXMtZXJkZW1yZW5kLWtpdHVudGV0ZXMvMTJsejh6ZT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE5/69b31bd04d2f0e8d990b13ddDe8204277";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvdGgtdmVyYS9idmN6aDd0P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTk/69b31bd04d2f0e8d990b13ddCfdd7cae8";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9nYXN6dHJvL3N1bHQta3J1bXBsaS1yZWNlcHQtbWFyeS1iZXJyeS9zN2R0Z203P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTk/69b31bd04d2f0e8d990b13ddB72ee79ed";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvY3NpcGVzLXRhbWFyYS1lbGFkYXMtZXJkZW1yZW5kLWtpdHVudGV0ZXMvMTJsejh6ZT91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE5/69b31bd04d2f0e8d990b13ddBe8204277";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvdGgtdmVyYS9idmN6aDd0P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTk/69b31bd04d2f0e8d990b13ddDfdd7cae8";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9hdXRvLWhpdGVsLXRhcnRvemFzLXZlZ3JlaGFqdGFzL3d2ZmpmM3o_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOQ/69b31bd04d2f0e8d990b13ddC423bbbb3";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay90ZWNoL2dvb2dsZS1kcml2ZS11ai1mdW5rY2lvay10aXBwZWstdGFuYWNzLXN6YW1pdG9nZXAvOTl2bndyMz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE5/69b31bd04d2f0e8d990b13ddB32358edd";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9wZWNlbC1jc2Fwdml6LXN6ZW5ueWV6ZXR0LWd1c3p0dXN0YWxhbi8xaGR2NXhnP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTk/69b31bd04d2f0e8d990b13ddB2ecbbe15";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvZmVyZmlha25hay9hdXRvL2Jtdy1lbGVrdHJvbW9zLTMtYXMvMmc1YzNiaD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE5/69b31bd04d2f0e8d990b13ddBcb583b3a";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9zYXJwZW50ZWxlLWFscGFrYS1hbGxhdGtpbnphcy1neWlsa29zc2FnLzhsOGNyYmY_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOQ/69b31bd04d2f0e8d990b13ddC3e441951";"https://link.blikk.hu/click/44777796.3955/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZ3llcmVrZ3lpbGtvc3NhZy8zM21teTMwP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTk/69b31bd04d2f0e8d990b13ddC761cfd45"</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Vége Lakatos Márk kapcsolatának?</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>18.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvYXV0by8yMDI2LW9zLXN1enVraS1zLXByZXNzby8zaGUwc2RkP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTg/69b31bd04d2f0e8d990b13ddB2da90a87";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOA/69b31bd04d2f0e8d990b13ddBf4f6133d";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvZGFiYXMtZ3lvbi12YXN1dC12ZXJlcy1rb3JvemVzLXJlbmRvcnNlZy94N20ydnhjP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTg/69b31bd04d2f0e8d990b13ddC546fe277";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2xha2F0b3MtbWFyay1mZXJqZW5lay1zemVyZXRvamUtYm90cmFueS83dmhteTJ5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTg/69b31bd04d2f0e8d990b13ddB5f2c2867";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvYmxpa2stdHYvdGVzenQtcG9saXRpa3VzLWphdGVrLWZlbGlzbWVyLWFrdHVhbGlzLWVtYmVyZWstcG9saXRpa3Vzb2stc3ppbmVzemVrLzMyMXgzMmc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOA/69b31bd04d2f0e8d990b13ddB46f4fd2a";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3J0bC1tYWd5YXJvcnN6YWctc29yb3phdC85eXA4anBnP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTg/69b31bd04d2f0e8d990b13ddBc0f2b92a";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvYmxpa2stdHYvdGVzenQtcG9saXRpa3VzLWphdGVrLWZlbGlzbWVyLWFrdHVhbGlzLWVtYmVyZWstcG9saXRpa3Vzb2stc3ppbmVzemVrLzMyMXgzMmc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOA/69b31bd04d2f0e8d990b13ddD46f4fd2a";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL21pbG8tdmlraS1oYXphc3NhZy1lbHNvLWxhdGFzcmEtbmFneS1kdWV0dC9wNWUwdDM4P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTg/69b31bd04d2f0e8d990b13ddB7579393b";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvc3pvYm9zemxhaS16c29sdC1zem9ib3N6bGFpLWRvbWluaWstbGl2ZXJwb29sLzd3cHBqdGQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOA/69b31bd04d2f0e8d990b13ddCa759e2f1";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC90aXBwZWsvbXVhbnlhZy16YWNza29rLWhlbHlldHQtZmFneWFzenRhcy9sanpkMHRrP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTg/69b31bd04d2f0e8d990b13ddBa7bf1e10";"https://link.blikk.hu/click/44759719.10556/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9iZXJ0YXJneWFsYXMtZml6ZXRlc2VtZWxlcy1pa2VhL2U4MDJiZXo_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xOA/69b31bd04d2f0e8d990b13ddC0478f13f"</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Egyre fogy a magyar olajtartalék, egy szorostól függ a benzinár sorsa</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>17.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvb2xhanRhcnRhbGVrLXV6ZW1hbnlhZy10YXJ0YWxlay9mNjhsdjU5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTc/69b31bd04d2f0e8d990b13ddE6d18b78e";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3BvcnQvbWFneWFyLWZvY2kvbWFneWFyLWJyYXppbC1sYWJkYXJ1Z2FzLzYyanp2cnI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNw/69b31bd04d2f0e8d990b13ddB21314b55";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvYmVuemluYXJzdG9wL2hnbHdlZzc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNw/69b31bd04d2f0e8d990b13ddC6821ef48";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL25hcC1rZWx0ZS1lZ3lrb3JpLW11c29ydmV6ZXRvaS96c2U4cHhzP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTc/69b31bd04d2f0e8d990b13ddDd7216a0a";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9iYW5rb2stYmV0ZXRpLWthbWF0b2svdnR6Y3A4ZD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE3/69b31bd04d2f0e8d990b13ddB378fd169";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC90cmFnaWt1cy1oYWxhbGVzZXQtdWdyYXMvbm5ldmxlYz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE3/69b31bd04d2f0e8d990b13ddC9eff1844";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9neWVyZWttZXJnZXplc2kta2lzZXJsZXQvbTVxOG5sZz91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE3/69b31bd04d2f0e8d990b13ddB33616022";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvb2xhanRhcnRhbGVrLXV6ZW1hbnlhZy10YXJ0YWxlay9mNjhsdjU5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTc/69b31bd04d2f0e8d990b13ddC6d18b78e";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvdmlsYWdwb2xpdGlrYS9uZW1ldC1rb3JtYW55LW1lcnotdHJ1bXAtaXJhbmkta25mbGlrdHVzL3hwOXp5MGI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNw/69b31bd04d2f0e8d990b13ddB8dba9955";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL25hcC1rZWx0ZS1lZ3lrb3JpLW11c29ydmV6ZXRvaS96c2U4cHhzP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTc/69b31bd04d2f0e8d990b13ddBd7216a0a";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9vbmxpbmUtYWRvYmVmaXpldGVzLWxlcGVzZWkvbmNtM3k1Yj91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE3/69b31bd04d2f0e8d990b13ddCb99bd35c";"https://link.blikk.hu/click/44726606.11394/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMvYmVsZm9sZC9rdXR5YS1wZWtzZWctY3VrcmFzemRhLWVyZC1kYW5vcy10YW1hcy84ZTdsMTJzP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTc/69b31bd04d2f0e8d990b13ddBd49ee0fa"</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>„Ez nem önvédelem volt, hanem kivégzés” – Hátulról, hidegvérrel lőtték le a magyar betörőt az osztrák hatóság szerint</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>16.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JlcmVjemtpLXpvbHRhbi12YWxhcy11anJha2V6ZGVzLWJhdGEtZXZhL2h0M3B3bnM_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNg/69b31bd04d2f0e8d990b13ddB00355ea2";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL29zYmF0aC1ub3JiZXJ0LWVzLW9zYmF0aC1tYXJrLXBhbWt1dHlhLXJla29yZC1tdm0tZG9tZS80bmU0ZzYyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTY/69b31bd04d2f0e8d990b13ddD86943347";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2JlcmVjemtpLXpvbHRhbi12YWxhcy11anJha2V6ZGVzLWJhdGEtZXZhL2h0M3B3bnM_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNg/69b31bd04d2f0e8d990b13ddD00355ea2";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3ZlbmN6ZWwtdmVyYS04MC1ldmVzLWxlbm5lLXN6YWttYWktZWxpc21lcmVzL3J3MTZ5emM_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNg/69b31bd04d2f0e8d990b13ddBa9fe2dfd";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9maWxta2xpa2svb3NjYXItMjAyNi1ueWVydGVzZWsvZDYycnd5dD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE2/69b31bd04d2f0e8d990b13ddBfaf8a9e4";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3BhbWt1dHlhLWF6YWhyaWFoLXN6dGFyLXN6YXZhemFzL3c5MXNkbWQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNg/69b31bd04d2f0e8d990b13ddB5e1d62ec";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3ZvbWJlcmctZnJpZ3llcy1zZWZlay1zZWZlLWtpaGl2YXMvYnpxOGU5az91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTE2/69b31bd04d2f0e8d990b13ddBeda08d09";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbWFneWFyLWJldG9yby1hdXN6dHJpYS1neWlsa29zc2FnL20zNmttc3E_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNg/69b31bd04d2f0e8d990b13ddC40ad1956";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL29zYmF0aC1ub3JiZXJ0LWVzLW9zYmF0aC1tYXJrLXBhbWt1dHlhLXJla29yZC1tdm0tZG9tZS80bmU0ZzYyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTY/69b31bd04d2f0e8d990b13ddC86943347";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2xvdGUtYXR0aWxhLWhhbGFsYS1neWFzei1idWNzdS9uMjA3azhyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTY/69b31bd04d2f0e8d990b13ddB6a92066d";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvdmFzYXJsYXMvZXJkaS1pbmdhdGxhbmNzYWxvLWFsZG96YXRhaS81dGNqazl2P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTY/69b31bd04d2f0e8d990b13ddCbe121848";"https://link.blikk.hu/click/44710088.388/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL21hcmNpdXMtMTUtdW5uZXBpLW1lbmV0ZWstdmlkZW8tb3NzemVmb2dsYWxvL3R5MXMyZ3M_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xNg/69b31bd04d2f0e8d990b13ddC96b17875"</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Blikk</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Gombos Edina 11 év után visszatér a TV2 képernyőjére</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>13.03.2026 2026</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbnlvbW9uLXZhZ3l1bmstc3plcmVwamF0ZWtvcy1neWlsa29zLWludGVyanUtc3pvbG8tdXRjYS12b2x0LWlnYXpnYXpvamEta29yb25hdGFudS85MmQzbHMyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTM/69b31bd04d2f0e8d990b13ddBd57fe2e0";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3VkdmFyb3MtZG9yb3R0eWEtcmV2aWN6a3ktZ2Fib3ItbGFueWtlcmVzL2Y0ZDdnOXc_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xMw/69b31bd04d2f0e8d990b13ddB20a835be";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvZ2F6ZGFzYWcvcGVuei9taW5pbWFsYmVyLWVtZWxlcy1la2hvLW5ldHRvLWJlci94MmMzbTZ0P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTM/69b31bd04d2f0e8d990b13ddCc156ddf1";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC90aXBwZWsvaGlkcmF0YWNpby12aXotbmFwaS1mb2x5YWRlay8xMzI3eXBsP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTM/69b31bd04d2f0e8d990b13ddC2a1ee544";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvbXBvcy1rYXR5YS1zenVsZXRlc25hcGphLW9idWRhLXN6aW5oYXp0ZXJlbS1uZXZlL2o2anQ5OTU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xMw/69b31bd04d2f0e8d990b13ddD5712111f";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvYWt0dWFsaXMva3JpbWkvbnlvbW9uLXZhZ3l1bmstc3plcmVwamF0ZWtvcy1neWlsa29zLWludGVyanUtc3pvbG8tdXRjYS12b2x0LWlnYXpnYXpvamEta29yb25hdGFudS85MmQzbHMyP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTM/69b31bd04d2f0e8d990b13ddDd57fe2e0";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvcG9saXRpa2EvbWFneWFyLXBvbGl0aWthL2JhcmF0c2FnLWtvb2xhanZlemV0ZWstbWFneWFyLWRlbGVnYWNpby1raWpldi84ZjFxbmg5P3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTM/69b31bd04d2f0e8d990b13ddC4caad72d";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2F6c2lhLWV4cHJlc3N6LWdvbWJvcy1lZGluYS83M2V0dDRjP3V0bV9zb3VyY2U9bmV3c2xldHRlciZ1dG1fbWVkaXVtPWVtYWlsJnV0bV9jYW1wYWlnbj1zdW1tYXJ5LWRhaWx5JnV0bV9jb250ZW50PTIwMjYtMDMtMTM/69b31bd04d2f0e8d990b13ddC2595c993";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL3RvbXBvcy1rYXR5YS1zenVsZXRlc25hcGphLW9idWRhLXN6aW5oYXp0ZXJlbS1uZXZlL2o2anQ5OTU_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xMw/69b31bd04d2f0e8d990b13ddB5712111f";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvZWxldG1vZC9lZ2VzenNlZy9zY2hvYmVydC1ub3JiaS1ydWJpbnQtcmVrYS1zaGFwZXdheS10ZWp0ZXJtZWstZm9neWFzL3hoemVtbjQ_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xMw/69b31bd04d2f0e8d990b13ddCe179565a";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvYmxpa2stdHYvc3pvbG8tdXRjYS1qYXZpdG9pbnRlemV0LWJvdHJhbnktYXJ2ZXJlcy1pbmdhdGxhbi1wZW56LXZpZGVvL3FnODdmeTI_dXRtX3NvdXJjZT1uZXdzbGV0dGVyJnV0bV9tZWRpdW09ZW1haWwmdXRtX2NhbXBhaWduPXN1bW1hcnktZGFpbHkmdXRtX2NvbnRlbnQ9MjAyNi0wMy0xMw/69b31bd04d2f0e8d990b13ddC2cae0084";"https://link.blikk.hu/click/44677682.2071/aHR0cHM6Ly93d3cuYmxpa2suaHUvc3p0YXJ2aWxhZy9oYXphaS1zenRhcm9rL2F6c2lhLWV4cHJlc3N6LTIwMjYtYm9kaS10ZXNvay1zemVyZXBsb2svMDZtbXh0eD91dG1fc291cmNlPW5ld3NsZXR0ZXImdXRtX21lZGl1bT1lbWFpbCZ1dG1fY2FtcGFpZ249c3VtbWFyeS1kYWlseSZ1dG1fY29udGVudD0yMDI2LTAzLTEz/69b31bd04d2f0e8d990b13ddB52f55d09"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>